<commit_message>
Audit d1: master table regenerated with the 12-unit dossier overlay applied
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -1385,20 +1385,56 @@
           <t>reg-csa-1c-wsh-3</t>
         </is>
       </c>
-      <c r="AB9" s="5" t="n"/>
+      <c r="AB9" s="5" t="inlineStr">
+        <is>
+          <t>unauthored (battalion in-build only)</t>
+        </is>
+      </c>
       <c r="AC9" s="5" t="n"/>
       <c r="AD9" s="5" t="n"/>
       <c r="AE9" s="5" t="n"/>
       <c r="AF9" s="5" t="n"/>
-      <c r="AG9" s="5" t="n"/>
-      <c r="AH9" s="5" t="n"/>
-      <c r="AI9" s="5" t="n"/>
-      <c r="AJ9" s="5" t="n"/>
-      <c r="AK9" s="5" t="n"/>
-      <c r="AL9" s="5" t="n"/>
-      <c r="AM9" s="5" t="n"/>
+      <c r="AG9" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-wsh-3-miller.md</t>
+        </is>
+      </c>
+      <c r="AH9" s="5" t="inlineStr">
+        <is>
+          <t>Capt. M.B. Miller, 3rd Co. Washington Arty; order chain Longstreet -&gt; Walton -&gt; Miller (or-27-2-longstreet verified)</t>
+        </is>
+      </c>
+      <c r="AI9" s="5" t="inlineStr">
+        <is>
+          <t>no company figure located (gap); battalion 240 at build grain</t>
+        </is>
+      </c>
+      <c r="AJ9" s="5" t="inlineStr">
+        <is>
+          <t>[E] inside battalion Peach Orchard frontage, parent centroid (3220,3550) f55; company coord inference +-150m marked</t>
+        </is>
+      </c>
+      <c r="AK9" s="5" t="inlineStr">
+        <is>
+          <t>[D pre-daylight] night arrival with battalion; none in-window</t>
+        </is>
+      </c>
+      <c r="AL9" s="5" t="inlineStr">
+        <is>
+          <t>[A = CA-J3A-1] FIRES THE SIGNAL GUNS 13:07 (jacobs-1864 reading; martin-smith participant grade); then general bombardment fire</t>
+        </is>
+      </c>
+      <c r="AM9" s="5" t="inlineStr">
+        <is>
+          <t>no company K/W/M located (gap); no officer pin (negative at corpus grain)</t>
+        </is>
+      </c>
       <c r="AN9" s="5" t="n"/>
-      <c r="AO9" s="5" t="n"/>
+      <c r="AO9" s="5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -7249,20 +7285,56 @@
           <t>reg-csa-1c-bn-alexander</t>
         </is>
       </c>
-      <c r="AB74" s="5" t="n"/>
+      <c r="AB74" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (static line)</t>
+        </is>
+      </c>
       <c r="AC74" s="5" t="n"/>
       <c r="AD74" s="5" t="n"/>
       <c r="AE74" s="5" t="n"/>
       <c r="AF74" s="5" t="n"/>
-      <c r="AG74" s="5" t="n"/>
-      <c r="AH74" s="5" t="n"/>
-      <c r="AI74" s="5" t="n"/>
-      <c r="AJ74" s="5" t="n"/>
-      <c r="AK74" s="5" t="n"/>
-      <c r="AL74" s="5" t="n"/>
-      <c r="AM74" s="5" t="n"/>
+      <c r="AG74" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-bn-alexander.md; the Alexander-notes-vs-long-cannonade crux recorded not resolved (ED-24 tension 2)</t>
+        </is>
+      </c>
+      <c r="AH74" s="5" t="inlineStr">
+        <is>
+          <t>Col. E.P. Alexander (directing corps arty Jul 3, Longstreet's order) / Maj. Huger at the battalion; 6 batteries; Woolfolk w Jul 2</t>
+        </is>
+      </c>
+      <c r="AI74" s="5" t="inlineStr">
+        <is>
+          <t>576 build adoption; ~24-26 guns (tablet-grade); per-battery figures open</t>
+        </is>
+      </c>
+      <c r="AJ74" s="5" t="inlineStr">
+        <is>
+          <t>[E] ridge line from Peach Orchard NE (tablet verbatim), centroid (3170,4150) f78, frontage ~400-500m; Jul 2 Peach Orchard fight line deferred</t>
+        </is>
+      </c>
+      <c r="AK74" s="5" t="inlineStr">
+        <is>
+          <t>[D] Jul 2 night redeploy into bombardment line; none in-window (fwd displacement NOT attested - negative + conflict slot)</t>
+        </is>
+      </c>
+      <c r="AL74" s="5" t="inlineStr">
+        <is>
+          <t>[A window] core of the cannonade; [C 13:32/13:47 corrected] the two notes to Pickett = CA-J3A-2/3 written from this line; ammunition famine defines the record</t>
+        </is>
+      </c>
+      <c r="AM74" s="5" t="inlineStr">
+        <is>
+          <t>battalion K/W/M open (gap); Jul 2 the bloody day; pin: Woolfolk w Jul 2</t>
+        </is>
+      </c>
       <c r="AN74" s="5" t="n"/>
-      <c r="AO74" s="5" t="n"/>
+      <c r="AO74" s="5" t="inlineStr">
+        <is>
+          <t>T4 (battalion grain)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -7993,20 +8065,56 @@
           <t>reg-csa-1c-bn-wash</t>
         </is>
       </c>
-      <c r="AB80" s="5" t="n"/>
+      <c r="AB80" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (static line)</t>
+        </is>
+      </c>
       <c r="AC80" s="5" t="n"/>
       <c r="AD80" s="5" t="n"/>
       <c r="AE80" s="5" t="n"/>
       <c r="AF80" s="5" t="n"/>
-      <c r="AG80" s="5" t="n"/>
-      <c r="AH80" s="5" t="n"/>
-      <c r="AI80" s="5" t="n"/>
-      <c r="AJ80" s="5" t="n"/>
-      <c r="AK80" s="5" t="n"/>
-      <c r="AL80" s="5" t="n"/>
-      <c r="AM80" s="5" t="n"/>
+      <c r="AG80" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-bn-wash-eshleman.md</t>
+        </is>
+      </c>
+      <c r="AH80" s="5" t="inlineStr">
+        <is>
+          <t>Maj. B.F. Eshleman; 4 cos (Squires/Richardson/Miller/Norcom-w-Jul3); Walton nominal chief with the battalion (divided command vs Alexander recorded)</t>
+        </is>
+      </c>
+      <c r="AI80" s="5" t="inlineStr">
+        <is>
+          <t>240 build adoption (tablet-cited); per-company figures open</t>
+        </is>
+      </c>
+      <c r="AJ80" s="5" t="inlineStr">
+        <is>
+          <t>[D/E] 'Arrived on the field before daylight' Jul 3 (tablet verbatim); [E] Peach Orchard line (3220,3550) f55, frontage ~300m</t>
+        </is>
+      </c>
+      <c r="AK80" s="5" t="inlineStr">
+        <is>
+          <t>[D before ~04:30 daylight] night march onto field; attested-static in window</t>
+        </is>
+      </c>
+      <c r="AL80" s="5" t="inlineStr">
+        <is>
+          <t>[A] CA-J3A-1 signal guns via 3rd Co.; [A window] 10 guns in the general bombardment ('YES + the 13:07 signal guns', tablet-grade)</t>
+        </is>
+      </c>
+      <c r="AM80" s="5" t="inlineStr">
+        <is>
+          <t>battalion K/W/M open (gap); pin: Capt. Norcom w Jul 3; clean single-episode shape (arrived Jul 3)</t>
+        </is>
+      </c>
       <c r="AN80" s="5" t="n"/>
-      <c r="AO80" s="5" t="n"/>
+      <c r="AO80" s="5" t="inlineStr">
+        <is>
+          <t>T4 (battalion grain)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -17953,20 +18061,56 @@
           <t>reg-us-ar-1v</t>
         </is>
       </c>
-      <c r="AB164" s="5" t="n"/>
+      <c r="AB164" s="5" t="inlineStr">
+        <is>
+          <t>unauthored (only Phillips in build)</t>
+        </is>
+      </c>
       <c r="AC164" s="5" t="n"/>
       <c r="AD164" s="5" t="n"/>
       <c r="AE164" s="5" t="n"/>
       <c r="AF164" s="5" t="n"/>
-      <c r="AG164" s="5" t="n"/>
-      <c r="AH164" s="5" t="n"/>
-      <c r="AI164" s="5" t="n"/>
-      <c r="AJ164" s="5" t="n"/>
-      <c r="AK164" s="5" t="n"/>
-      <c r="AL164" s="5" t="n"/>
-      <c r="AM164" s="5" t="n"/>
+      <c r="AG164" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ar-1v-mcgilvery.md; his July 3 opening clock (OR pp.882-883) still unverified; ED-35 candidate: cast the line as a command unit</t>
+        </is>
+      </c>
+      <c r="AH164" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Col. McGilvery; July 3 line = composite command of 3 Reserve brigades + III Corps battery under Hunt's direct control; Bigelow w July 2 -&gt; Milton</t>
+        </is>
+      </c>
+      <c r="AI164" s="5" t="inlineStr">
+        <is>
+          <t>no engaged-men figure located (gap); '39 guns' secondary-grade; tablet-verified 9-battery roster is the stronger form</t>
+        </is>
+      </c>
+      <c r="AJ164" s="5" t="inlineStr">
+        <is>
+          <t>[C p.881] July 2 Wheatfield Rd line from ~15:30; [D] Trostle stand + Plum Run line; [E] July 3 massed lower-Cemetery-Ridge line, ref point Phillips (4212,4080) f265; sheet-8 Daniels/Rank labels CONFLICT with OOB (ECF)</t>
+        </is>
+      </c>
+      <c r="AK164" s="5" t="inlineStr">
+        <is>
+          <t>[C ~15:30 Jul 2] march to Sickles; [D] fighting retreat by prolonge; [C tablet ~15:00 Jul 3] Cooper's B/1st PA joins line from E Cemetery Hill [B: ~15-20 min leg]</t>
+        </is>
+      </c>
+      <c r="AL164" s="5" t="inlineStr">
+        <is>
+          <t>[A window] ORDERED SILENCE under Hunt's policy (CA-J3A-4's largest component); 'fired about one hour and a half... 10,000 rounds' (or-27-1-mcgilvery p.884); [C ~15:00] first line 'completely broken up and scattered by our fire'; oblique raking fire through all three lines; then Wilcox/Lang smashed with 16th VT</t>
+        </is>
+      </c>
+      <c r="AM164" s="5" t="inlineStr">
+        <is>
+          <t>brigade K/W/M not located (gap; July 2 dominates via Bigelow's stand); pin: Bigelow w July 2</t>
+        </is>
+      </c>
       <c r="AN164" s="5" t="n"/>
-      <c r="AO164" s="5" t="n"/>
+      <c r="AO164" s="5" t="inlineStr">
+        <is>
+          <t>T4 (brigade grain)</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -18481,20 +18625,56 @@
           <t>reg-us-ii-arty</t>
         </is>
       </c>
-      <c r="AB170" s="5" t="n"/>
+      <c r="AB170" s="5" t="inlineStr">
+        <is>
+          <t>command record (batteries in-build individually)</t>
+        </is>
+      </c>
       <c r="AC170" s="5" t="n"/>
       <c r="AD170" s="5" t="n"/>
       <c r="AE170" s="5" t="n"/>
       <c r="AF170" s="5" t="n"/>
-      <c r="AG170" s="5" t="n"/>
-      <c r="AH170" s="5" t="n"/>
-      <c r="AI170" s="5" t="n"/>
-      <c r="AJ170" s="5" t="n"/>
-      <c r="AK170" s="5" t="n"/>
-      <c r="AL170" s="5" t="n"/>
-      <c r="AM170" s="5" t="n"/>
+      <c r="AG170" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-arty-hazard.md; ED-34 candidate (activity classes)</t>
+        </is>
+      </c>
+      <c r="AH170" s="5" t="inlineStr">
+        <is>
+          <t>Capt. J.G. Hazard; worst commander attrition of any Union arty bde: Rorty k, Cushing k, Woodruff mw, Sheldon w, Milne mw (or-27-1-hazard)</t>
+        </is>
+      </c>
+      <c r="AI170" s="5" t="inlineStr">
+        <is>
+          <t>600 aggregate (stone-sentinels) vs battery-page sum 602 - consistent, both carried; 26 guns</t>
+        </is>
+      </c>
+      <c r="AJ170" s="5" t="inlineStr">
+        <is>
+          <t>[E] 5-battery line Ziegler's Grove -&gt; Rorty's left, ~530m frontage = the convergence target square (battery coords in their rows)</t>
+        </is>
+      </c>
+      <c r="AK170" s="5" t="inlineStr">
+        <is>
+          <t>static except Brown's ordered withdrawal + post-repulse replacements</t>
+        </is>
+      </c>
+      <c r="AL170" s="5" t="inlineStr">
+        <is>
+          <t>[A window] FOUGHT THE CANNONADE THROUGHOUT under Hancock's counter-order; long-range ammo exhausted (or-27-1-hazard) -&gt; canister-only repulse fight</t>
+        </is>
+      </c>
+      <c r="AM170" s="5" t="inlineStr">
+        <is>
+          <t>150 (25k/120w/5m), 35% - highest-pct Union arty bde loss; flat-then-spike shape vs the silent-then-fire lines; 5 officer pins at battery grain</t>
+        </is>
+      </c>
       <c r="AN170" s="5" t="n"/>
-      <c r="AO170" s="5" t="n"/>
+      <c r="AO170" s="5" t="inlineStr">
+        <is>
+          <t>T4 (brigade grain)</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -18833,20 +19013,56 @@
           <t>reg-us-xi-arty</t>
         </is>
       </c>
-      <c r="AB174" s="5" t="n"/>
+      <c r="AB174" s="5" t="inlineStr">
+        <is>
+          <t>unauthored</t>
+        </is>
+      </c>
       <c r="AC174" s="5" t="n"/>
       <c r="AD174" s="5" t="n"/>
       <c r="AE174" s="5" t="n"/>
       <c r="AF174" s="5" t="n"/>
-      <c r="AG174" s="5" t="n"/>
-      <c r="AH174" s="5" t="n"/>
-      <c r="AI174" s="5" t="n"/>
-      <c r="AJ174" s="5" t="n"/>
-      <c r="AK174" s="5" t="n"/>
-      <c r="AL174" s="5" t="n"/>
-      <c r="AM174" s="5" t="n"/>
+      <c r="AG174" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-xi-arty-osborn.md</t>
+        </is>
+      </c>
+      <c r="AH174" s="5" t="inlineStr">
+        <is>
+          <t>Maj. T.W. Osborn; Jul 3 group exceeds organic brigade (Reserve + I Corps attachments under his direction)</t>
+        </is>
+      </c>
+      <c r="AI174" s="5" t="inlineStr">
+        <is>
+          <t>no men figure located (gap); ~39 guns secondary-grade; tablet-verified 9-battery roster is the stronger form</t>
+        </is>
+      </c>
+      <c r="AJ174" s="5" t="inlineStr">
+        <is>
+          <t>[E multi-day] Cemetery Hill plateau Jul 1 retreat -&gt; Jul 4; coords deferred (square's N margin)</t>
+        </is>
+      </c>
+      <c r="AK174" s="5" t="inlineStr">
+        <is>
+          <t>group attested-static Jul 3</t>
+        </is>
+      </c>
+      <c r="AL174" s="5" t="inlineStr">
+        <is>
+          <t>[A window] counter-battery under the crossfire; [C ~14:30] THE CEASE-FIRE RUSE (proposed Osborn, adopted Hunt/Howard) = CA-J3A-4/5's sharpest component; [D] ~1,600 rounds into Pettigrew's left (secondary-grade)</t>
+        </is>
+      </c>
+      <c r="AM174" s="5" t="inlineStr">
+        <is>
+          <t>brigade K/W/M open (gap); Jul 1-2 dominate the shape; no Jul 3 officer pin located (negative)</t>
+        </is>
+      </c>
       <c r="AN174" s="5" t="n"/>
-      <c r="AO174" s="5" t="n"/>
+      <c r="AO174" s="5" t="inlineStr">
+        <is>
+          <t>T4 (group grain)</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -21385,20 +21601,56 @@
           <t>reg-us-arty-hq</t>
         </is>
       </c>
-      <c r="AB203" s="5" t="n"/>
+      <c r="AB203" s="5" t="inlineStr">
+        <is>
+          <t>command record</t>
+        </is>
+      </c>
       <c r="AC203" s="5" t="n"/>
       <c r="AD203" s="5" t="n"/>
       <c r="AE203" s="5" t="n"/>
       <c r="AF203" s="5" t="n"/>
-      <c r="AG203" s="5" t="n"/>
-      <c r="AH203" s="5" t="n"/>
-      <c r="AI203" s="5" t="n"/>
-      <c r="AJ203" s="5" t="n"/>
-      <c r="AK203" s="5" t="n"/>
-      <c r="AL203" s="5" t="n"/>
-      <c r="AM203" s="5" t="n"/>
+      <c r="AG203" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-arty-hq-hunt.md; NEW register row this pass</t>
+        </is>
+      </c>
+      <c r="AH203" s="5" t="inlineStr">
+        <is>
+          <t>Brig. Gen. H.J. Hunt, Chief of Artillery AoP; authority contested by Hancock on the II Corps front - the dispute IS CA-J3A-4's sectoral shape</t>
+        </is>
+      </c>
+      <c r="AI203" s="5" t="inlineStr">
+        <is>
+          <t>n/a (command entry); Reserve 2,375 men / 114 guns nominal under command</t>
+        </is>
+      </c>
+      <c r="AJ203" s="5" t="inlineStr">
+        <is>
+          <t>[C] ~11-13:00 line inspection ride; [A vs CA-J3A-1] on Little Round Top at the opening; [A window] at Cowan's guns at the climax (horse shot, brown-1985-filson)</t>
+        </is>
+      </c>
+      <c r="AK203" s="5" t="inlineStr">
+        <is>
+          <t>command-grain ride sequence (times the order delivery)</t>
+        </is>
+      </c>
+      <c r="AL203" s="5" t="inlineStr">
+        <is>
+          <t>[C ~11:00] withhold-fire instruction; [C ~14:30] the slacken/cease order (CA-J3A-4); [D] Hancock counter-order conflict; [D] repulse-window battery reinforcements</t>
+        </is>
+      </c>
+      <c r="AM203" s="5" t="inlineStr">
+        <is>
+          <t>n/a; horse killed at Cowan's guns</t>
+        </is>
+      </c>
       <c r="AN203" s="5" t="n"/>
-      <c r="AO203" s="5" t="n"/>
+      <c r="AO203" s="5" t="inlineStr">
+        <is>
+          <t>T2 (command record)</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -21633,20 +21885,56 @@
           <t>reg-us-ii-b2</t>
         </is>
       </c>
-      <c r="AB205" s="5" t="n"/>
+      <c r="AB205" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (ED-7 stands)</t>
+        </is>
+      </c>
       <c r="AC205" s="5" t="n"/>
       <c r="AD205" s="5" t="n"/>
       <c r="AE205" s="5" t="n"/>
       <c r="AF205" s="5" t="n"/>
-      <c r="AG205" s="5" t="n"/>
-      <c r="AH205" s="5" t="n"/>
-      <c r="AI205" s="5" t="n"/>
-      <c r="AJ205" s="5" t="n"/>
-      <c r="AK205" s="5" t="n"/>
-      <c r="AL205" s="5" t="n"/>
-      <c r="AM205" s="5" t="n"/>
+      <c r="AG205" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-arnold.md</t>
+        </is>
+      </c>
+      <c r="AH205" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Arnold survived unwounded ('gallantly fighting his own battery and saving it', or-27-1-hazard); 6x 3-in Ordnance rifles</t>
+        </is>
+      </c>
+      <c r="AI205" s="5" t="inlineStr">
+        <is>
+          <t>139 men (stone-sentinels; civilwarintheeast derivative corroboration only)</t>
+        </is>
+      </c>
+      <c r="AJ205" s="5" t="inlineStr">
+        <is>
+          <t>[E] wall N of inner angle (4425,4955) f260 +-30m, ~80m N of Angle corner (Bachelder); attested-static with ED-7 withdrawal dispute riding the claim</t>
+        </is>
+      </c>
+      <c r="AK205" s="5" t="inlineStr">
+        <is>
+          <t>none authored (ED-7: neither withdrawal-timing reading strong enough to move traced geometry)</t>
+        </is>
+      </c>
+      <c r="AL205" s="5" t="inlineStr">
+        <is>
+          <t>[A window] served through the cannonade; [D] canister into Fry/Marshall closing on the wall; left-section gun's last double-shotted round into 26th NC (claim-arnold-canister)</t>
+        </is>
+      </c>
+      <c r="AM205" s="5" t="inlineStr">
+        <is>
+          <t>4k/24w of 139 (stone-sentinels); July 3 cannonade-window dominated; pin (negative): Arnold unwounded per Hazard's report</t>
+        </is>
+      </c>
       <c r="AN205" s="5" t="n"/>
-      <c r="AO205" s="5" t="n"/>
+      <c r="AO205" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -22253,20 +22541,56 @@
           <t>reg-us-ii-b3</t>
         </is>
       </c>
-      <c r="AB210" s="5" t="n"/>
+      <c r="AB210" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC210" s="5" t="n"/>
       <c r="AD210" s="5" t="n"/>
       <c r="AE210" s="5" t="n"/>
       <c r="AF210" s="5" t="n"/>
-      <c r="AG210" s="5" t="n"/>
-      <c r="AH210" s="5" t="n"/>
-      <c r="AI210" s="5" t="n"/>
-      <c r="AJ210" s="5" t="n"/>
-      <c r="AK210" s="5" t="n"/>
-      <c r="AL210" s="5" t="n"/>
-      <c r="AM210" s="5" t="n"/>
+      <c r="AG210" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-brown.md; ED-33 candidate on what 'the 18 guns have gone' observed</t>
+        </is>
+      </c>
+      <c r="AH210" s="5" t="inlineStr">
+        <is>
+          <t>Lt. T.F. Brown w July 2 -&gt; Lt. Perrin July 3; Lt. Milne detached to Cushing (mw); 6 Napoleons, 4 serviceable July 3 (brown-1985-filson)</t>
+        </is>
+      </c>
+      <c r="AI210" s="5" t="inlineStr">
+        <is>
+          <t>103 men (stone-sentinels, single-source, flagged)</t>
+        </is>
+      </c>
+      <c r="AJ210" s="5" t="inlineStr">
+        <is>
+          <t>[E] 4-gun line S of Copse (4445,4785) f262 +-30m (Bachelder); [C/D ~14:40] withdrawn over crest to park (4610,4800)</t>
+        </is>
+      </c>
+      <c r="AK210" s="5" t="inlineStr">
+        <is>
+          <t>[D mid-cannonade] ordered withdrawal ~165m by piece [B: &lt;=10 min leg]; no other July 3 movement</t>
+        </is>
+      </c>
+      <c r="AL210" s="5" t="inlineStr">
+        <is>
+          <t>[A window] counter-battery 13:07-~14:40 until long-range ammo out; then SILENT (withdrawn) - one of two real events behind Alexander's 'guns have gone' reading (CA-J3A-4)</t>
+        </is>
+      </c>
+      <c r="AM210" s="5" t="inlineStr">
+        <is>
+          <t>28 whole-battle (stone-sentinels), K/W split not carried - thin; mostly July 2; pins: Brown w Jul 2, Milne mw Jul 3 (on Cushing's rolls)</t>
+        </is>
+      </c>
       <c r="AN210" s="5" t="n"/>
-      <c r="AO210" s="5" t="n"/>
+      <c r="AO210" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -24981,20 +25305,56 @@
           <t>reg-us-ii-b1</t>
         </is>
       </c>
-      <c r="AB232" s="5" t="n"/>
+      <c r="AB232" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC232" s="5" t="n"/>
       <c r="AD232" s="5" t="n"/>
       <c r="AE232" s="5" t="n"/>
       <c r="AF232" s="5" t="n"/>
-      <c r="AG232" s="5" t="n"/>
-      <c r="AH232" s="5" t="n"/>
-      <c r="AI232" s="5" t="n"/>
-      <c r="AJ232" s="5" t="n"/>
-      <c r="AK232" s="5" t="n"/>
-      <c r="AL232" s="5" t="n"/>
-      <c r="AM232" s="5" t="n"/>
+      <c r="AG232" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-rorty.md; no rounds-expended record (negative)</t>
+        </is>
+      </c>
+      <c r="AH232" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Rorty k July 3 (overrun, hand-to-hand) -&gt; Lt. Sheldon w same action -&gt; Lt. Rogers; 4x 10-pdr Parrotts (stone-sentinels)</t>
+        </is>
+      </c>
+      <c r="AI232" s="5" t="inlineStr">
+        <is>
+          <t>114 men (stone-sentinels, single-source)</t>
+        </is>
+      </c>
+      <c r="AJ232" s="5" t="inlineStr">
+        <is>
+          <t>[E] (4435,4570) f262 ~250m S of Copse, fronting prone 19th MA (Bachelder; waitt-1906 pp.234-237); attested-static</t>
+        </is>
+      </c>
+      <c r="AK232" s="5" t="inlineStr">
+        <is>
+          <t>none July 3 (died in place)</t>
+        </is>
+      </c>
+      <c r="AL232" s="5" t="inlineStr">
+        <is>
+          <t>[A window vs CA-J3A-1/5] fought the cannonade to wreckage: 4-&gt;3-&gt;2-&gt;1 gun sequence + caisson burst (waitt-1906 verbatim) - the line's most granular gun-attrition record; [D] canister into Kemper, position briefly overrun</t>
+        </is>
+      </c>
+      <c r="AM232" s="5" t="inlineStr">
+        <is>
+          <t>10k/16w of 114 (stone-sentinels); inverse of the usual shape: steady loss under cannonade + spike at the melee; pins: Rorty k, Sheldon w [D ~15:20-30]</t>
+        </is>
+      </c>
       <c r="AN232" s="5" t="n"/>
-      <c r="AO232" s="5" t="n"/>
+      <c r="AO232" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
@@ -26469,20 +26829,56 @@
           <t>reg-us-ii-b4</t>
         </is>
       </c>
-      <c r="AB244" s="5" t="n"/>
+      <c r="AB244" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC244" s="5" t="n"/>
       <c r="AD244" s="5" t="n"/>
       <c r="AE244" s="5" t="n"/>
       <c r="AF244" s="5" t="n"/>
-      <c r="AG244" s="5" t="n"/>
-      <c r="AH244" s="5" t="n"/>
-      <c r="AI244" s="5" t="n"/>
-      <c r="AJ244" s="5" t="n"/>
-      <c r="AK244" s="5" t="n"/>
-      <c r="AL244" s="5" t="n"/>
-      <c r="AM244" s="5" t="n"/>
+      <c r="AG244" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-woodruff.md</t>
+        </is>
+      </c>
+      <c r="AH244" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Woodruff mw July 3 (d. July 4) -&gt; Lt. McCrea (or-27-1-hazard); 6 Napoleons</t>
+        </is>
+      </c>
+      <c r="AI244" s="5" t="inlineStr">
+        <is>
+          <t>120 men (stone-sentinels, single-source)</t>
+        </is>
+      </c>
+      <c r="AJ244" s="5" t="inlineStr">
+        <is>
+          <t>[E] Ziegler's Grove (4570,5095) f252 +-40m - NOT the Angle proper (library note; OSM grove centroid (4584,5101)); attested-static</t>
+        </is>
+      </c>
+      <c r="AK244" s="5" t="inlineStr">
+        <is>
+          <t>none July 3</t>
+        </is>
+      </c>
+      <c r="AL244" s="5" t="inlineStr">
+        <is>
+          <t>[A window] under the cannonade, Napoleons outranged; [D 15:16-30] canister into Pettigrew's left with Osborn's converging fire - half of why ED-5 authors no northern breach</t>
+        </is>
+      </c>
+      <c r="AM244" s="5" t="inlineStr">
+        <is>
+          <t>CONFLICT carried: 1k+29w (30) vs 1k+24w (25), same nominal source two extractions (oob-strengths); repulse-window dominated; pin: Woodruff mw [D in repulse fight]</t>
+        </is>
+      </c>
       <c r="AN244" s="5" t="n"/>
-      <c r="AO244" s="5" t="n"/>
+      <c r="AO244" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -28901,20 +29297,56 @@
           <t>reg-us-i-3-3</t>
         </is>
       </c>
-      <c r="AB266" s="5" t="n"/>
+      <c r="AB266" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC266" s="5" t="n"/>
       <c r="AD266" s="5" t="n"/>
       <c r="AE266" s="5" t="n"/>
       <c r="AF266" s="5" t="n"/>
-      <c r="AG266" s="5" t="n"/>
-      <c r="AH266" s="5" t="n"/>
-      <c r="AI266" s="5" t="n"/>
-      <c r="AJ266" s="5" t="n"/>
-      <c r="AK266" s="5" t="n"/>
-      <c r="AL266" s="5" t="n"/>
-      <c r="AM266" s="5" t="n"/>
+      <c r="AG266" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-i-3-3-stannard.md; wheel clock verified-negative (no witness clock exists)</t>
+        </is>
+      </c>
+      <c r="AH266" s="5" t="inlineStr">
+        <is>
+          <t>Stannard (w July 3 thigh, during 2nd flank move) -&gt; Randall; 13/14/16 VT engaged, 12/15 VT train guard (or-27-oob; stone-sentinels)</t>
+        </is>
+      </c>
+      <c r="AI266" s="5" t="inlineStr">
+        <is>
+          <t>1,950 brigade (stone-sentinels) vs 1,788 sum of engaged rgts (480+647+661) - ~160-man gap, both carried (oob-strengths #3)</t>
+        </is>
+      </c>
+      <c r="AJ266" s="5" t="inlineStr">
+        <is>
+          <t>[E] advanced line fwd of main position, ctr (4300,4470) f260 +-50m (Bachelder sheet 3); [A vs CA-J3A-8] 13VT wheeled anchor (4326,4764) f15 (200-yd monument statement, coord inferred +-40m)</t>
+        </is>
+      </c>
+      <c r="AK266" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J3A-8 ~15:20] change front fwd on 1st co., 13th then 16th, ~180m [B: 3-4 min at 1.4 m/s]; [D after CA-J3A-9] 16th reversal S vs Wilcox/Lang ~300m</t>
+        </is>
+      </c>
+      <c r="AL266" s="5" t="inlineStr">
+        <is>
+          <t>[D 15:16-20] front fire punishing Kemper's oblique; [A vs CA-J3A-8] flank fire at ~60 yd (Sturtevant pp.304-305), 243 prisoners (13VT monument); [D] 2nd flank fire, 2nd FL colors taken (veazey-or)</t>
+        </is>
+      </c>
+      <c r="AM266" s="5" t="inlineStr">
+        <is>
+          <t>45/275/30=350 of 1,950, 18% (stone-sentinels); episode split unattested - build decay is reconstruction; pin: Stannard w [D during 2nd flank move]</t>
+        </is>
+      </c>
       <c r="AN266" s="5" t="n"/>
-      <c r="AO266" s="5" t="n"/>
+      <c r="AO266" s="5" t="inlineStr">
+        <is>
+          <t>T4 (T5-grade inside Angle window via V2 claims)</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Audit d1 final: overlay verified-layer, master table regen, pass-1 report, owner-readable copies
12 units at audited T-levels (Miller T3; Hunt T2 command record; ten at
T4). Pass report: five chain-strengthening facts, EC honesty table,
ED-32..38 candidates, sources ledger, pass-2 reference-frame set.
Copies in docs/benchmarks/captures/audit-d1/. Suites: reconstruction
103, pipeline 59, tool 108 - green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -1387,7 +1387,7 @@
       </c>
       <c r="AB9" s="5" t="inlineStr">
         <is>
-          <t>unauthored (battalion in-build only)</t>
+          <t>unauthored (documented in-window mover - battalion in-build only)</t>
         </is>
       </c>
       <c r="AC9" s="5" t="n"/>
@@ -1396,37 +1396,37 @@
       <c r="AF9" s="5" t="n"/>
       <c r="AG9" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/csa-1c-wsh-3-miller.md</t>
+          <t>Dossier: reconstruction/dossiers/csa-1c-wsh-3-miller.md; second-gun/Owen detail OPEN (owen-1885 access failed)</t>
         </is>
       </c>
       <c r="AH9" s="5" t="inlineStr">
         <is>
-          <t>Capt. M.B. Miller, 3rd Co. Washington Arty; order chain Longstreet -&gt; Walton -&gt; Miller (or-27-2-longstreet verified)</t>
+          <t>Capt. M.B. Miller; 3 Napoleons (Lts Hero, McElroy) + Squires's 1st Co. Napoleon attached 'all under command of Captain Miller' (or-27-2-eshleman); order chain Longstreet -&gt; Walton -&gt; Eshleman/Miller closed verbatim at every link</t>
         </is>
       </c>
       <c r="AI9" s="5" t="inlineStr">
         <is>
-          <t>no company figure located (gap); battalion 240 at build grain</t>
+          <t>92 men / 3 Napoleons (addressing-gettysburg-oob, B&amp;M-type, hop flagged) + 1st Co. gun (77-man company)</t>
         </is>
       </c>
       <c r="AJ9" s="5" t="inlineStr">
         <is>
-          <t>[E] inside battalion Peach Orchard frontage, parent centroid (3220,3550) f55; company coord inference +-150m marked</t>
+          <t>[D pre-daylight] 'about 100 yards to the left of the peach orchard, and on the immediate left of Captain Taylor's battery' (or-27-2-eshleman) - company-grain, +-80m; [D post-cannonade] advanced position 400-500 yd to the front</t>
         </is>
       </c>
       <c r="AK9" s="5" t="inlineStr">
         <is>
-          <t>[D pre-daylight] night arrival with battalion; none in-window</t>
+          <t>[D] night arrival; [D after CA-J3A-5/6] ADVANCED 400-500 yd supporting the charge, 'opened with deadly effect' [B: ~410m ~6-8 min] - retires the attested-static reading; horse losses left 'but one gun' usable (marker)</t>
         </is>
       </c>
       <c r="AL9" s="5" t="inlineStr">
         <is>
-          <t>[A = CA-J3A-1] FIRES THE SIGNAL GUNS 13:07 (jacobs-1864 reading; martin-smith participant grade); then general bombardment fire</t>
+          <t>[A = CA-J3A-1] 'Two guns in quick succession were fired from Captain Miller's battery' (or-27-2-eshleman); 13:07 = Jacobs's reading; then bombardment + advanced-position canister work; rounds expended: attested-absent</t>
         </is>
       </c>
       <c r="AM9" s="5" t="inlineStr">
         <is>
-          <t>no company K/W/M located (gap); no officer pin (negative at corpus grain)</t>
+          <t>'Losses heavy but not reported in detail' (marker) - attested-unreported; battalion aggregate 3 off w + 3k/23w/16m is the ceiling</t>
         </is>
       </c>
       <c r="AN9" s="5" t="n"/>
@@ -7306,7 +7306,7 @@
       </c>
       <c r="AI74" s="5" t="inlineStr">
         <is>
-          <t>576 build adoption; ~24-26 guns (tablet-grade); per-battery figures open</t>
+          <t>576 men / 24 guns (B&amp;M-type, hop flagged; matches build); tablet armament verbatim; Ashland Parrott conflict (20-pdr tablet vs 10-pdr reproduction) carried</t>
         </is>
       </c>
       <c r="AJ74" s="5" t="inlineStr">
@@ -7316,17 +7316,17 @@
       </c>
       <c r="AK74" s="5" t="inlineStr">
         <is>
-          <t>[D] Jul 2 night redeploy into bombardment line; none in-window (fwd displacement NOT attested - negative + conflict slot)</t>
+          <t>[D] Jul 2 night redeploy to dawn line (Taylor tablet 03:00); IN-WINDOW CONFLICT: SHSP 'ordering those that had over 20 rounds left to limber up and follow Pickett' vs OR 'batteries all maintained their respective positions' - carried; build follows the OR</t>
         </is>
       </c>
       <c r="AL74" s="5" t="inlineStr">
         <is>
-          <t>[A window] core of the cannonade; [C 13:32/13:47 corrected] the two notes to Pickett = CA-J3A-2/3 written from this line; ammunition famine defines the record</t>
+          <t>[A window] core of cannonade, '75 guns' in his wing (SHSP); [C 13:32/13:47 corr.] the two notes = CA-J3A-2/3 (SHSP wording verified; 13:30-vs-13:25 internal variant); ammunition famine verbatim ('not over 20 rounds to the gun were left'); rounds expended attested-absent in OR</t>
         </is>
       </c>
       <c r="AM74" s="5" t="inlineStr">
         <is>
-          <t>battalion K/W/M open (gap); Jul 2 the bloody day; pin: Woolfolk w Jul 2</t>
+          <t>OR return verbatim: 19k/114w/6m = 139 + 116 horses, 1 howitzer destroyed (Jul 2-3 joint - no primary day split); Taylor's marker 2k/10w only per-battery figure; pins: Woolfolk w Jul 2, Gilbert w (SNIPPET)</t>
         </is>
       </c>
       <c r="AN74" s="5" t="n"/>
@@ -8086,27 +8086,27 @@
       </c>
       <c r="AI80" s="5" t="inlineStr">
         <is>
-          <t>240 build adoption (tablet-cited); per-company figures open</t>
+          <t>CONFLICT: build 240 vs 338 (B&amp;M-type, hop flagged; '340' SNIPPET variant); 8 Napoleons + 2 12-pdr howitzers (tablet + OR concur) -&gt; ED-38 candidate</t>
         </is>
       </c>
       <c r="AJ80" s="5" t="inlineStr">
         <is>
-          <t>[D/E] 'Arrived on the field before daylight' Jul 3 (tablet verbatim); [E] Peach Orchard line (3220,3550) f55, frontage ~300m</t>
+          <t>[D before daylight] per-company layout verbatim (or-27-2-eshleman): 3rd Co ~100yd left of Peach Orchard on Taylor's left, 4th on Miller's left, 2nd on Norcom's left, 2 howitzers reserve; Pendleton: 'nearly sixty guns for that wing'; centroid (3220,3550) f55; [E] park near old school-house at dark; [C 09:00 Jul 4] Cashtown (tablet-only)</t>
         </is>
       </c>
       <c r="AK80" s="5" t="inlineStr">
         <is>
-          <t>[D before ~04:30 daylight] night march onto field; attested-static in window</t>
+          <t>[D] night march (Sorrel's July 1 5:30 PM order verbatim, walton-shsp5-1877; Owen-as-quoted: started ~10:30-11 PM, wagon-train delay); in-window: Miller+Battles advance 400-500yd; Norcom's Napoleons moved several hundred yd left then disabled; howitzers brought forward</t>
         </is>
       </c>
       <c r="AL80" s="5" t="inlineStr">
         <is>
-          <t>[A] CA-J3A-1 signal guns via 3rd Co.; [A window] 10 guns in the general bombardment ('YES + the 13:07 signal guns', tablet-grade)</t>
+          <t>[A = CA-J3A-1] the signal guns verbatim; bombardment; captured Union 3-in rifle served by Richardson's co. until axle-struck (marker + OR); 'About thirty minutes after the signal guns... our infantry moved forward' AMBIGUOUS - conflict-flagged, rule 4; rounds: attested-absent</t>
         </is>
       </c>
       <c r="AM80" s="5" t="inlineStr">
         <is>
-          <t>battalion K/W/M open (gap); pin: Capt. Norcom w Jul 3; clean single-episode shape (arrived Jul 3)</t>
+          <t>OR return verbatim: 3 officers w; 3k/23w/16m men + 37 horses, 3 guns disabled, 1 limber blown up (tablet folds to 3/26/16=45); all July 3 (clean single-day); pin: Norcom w 'early in the day'</t>
         </is>
       </c>
       <c r="AN80" s="5" t="n"/>
@@ -18082,12 +18082,12 @@
       </c>
       <c r="AI164" s="5" t="inlineStr">
         <is>
-          <t>no engaged-men figure located (gap); '39 guns' secondary-grade; tablet-verified 9-battery roster is the stronger form</t>
+          <t>PRIMARY now: 15 officers + 368 men taken into action (organic 4 batteries, OR p. 884 footnote); line gun count 'total, thirty-nine guns' (his OR) vs Hunt B&amp;L 41 - carried</t>
         </is>
       </c>
       <c r="AJ164" s="5" t="inlineStr">
         <is>
-          <t>[C p.881] July 2 Wheatfield Rd line from ~15:30; [D] Trostle stand + Plum Run line; [E] July 3 massed lower-Cemetery-Ridge line, ref point Phillips (4212,4080) f265; sheet-8 Daniels/Rank labels CONFLICT with OOB (ECF)</t>
+          <t>[C ~15:30 Jul 2] Wheatfield Rd line; [C 17:45] retire 250 yd by stages; Trostle stand; 400-yd-rear line; [E Jul 3] low-ground line w/ earthwork, roster VERBATIM left-&gt;right incl. 'a New Jersey battery' + Rank's section (OR-vs-OOB conflict -&gt; ED-37); ref point Phillips (4212,4080)</t>
         </is>
       </c>
       <c r="AK164" s="5" t="inlineStr">
@@ -18097,18 +18097,18 @@
       </c>
       <c r="AL164" s="5" t="inlineStr">
         <is>
-          <t>[A window] ORDERED SILENCE under Hunt's policy (CA-J3A-4's largest component); 'fired about one hour and a half... 10,000 rounds' (or-27-1-mcgilvery p.884); [C ~15:00] first line 'completely broken up and scattered by our fire'; oblique raking fire through all three lines; then Wilcox/Lang smashed with 16th VT</t>
+          <t>[C 12:30 stated] opening '140 guns', overshoots 20-100 ft; [A window] pre-arranged hold-fire verbatim; the 'some general' breach put down; [C] 1.5h then deliberate battery-by-battery reply; [C ~15:00] first line 'completely broken up and scattered'; oblique raking fire through all three lines; Wilcox/Lang smashed</t>
         </is>
       </c>
       <c r="AM164" s="5" t="inlineStr">
         <is>
-          <t>brigade K/W/M not located (gap; July 2 dominates via Bigelow's stand); pin: Bigelow w July 2</t>
+          <t>tablet verbatim: 1 off + 16 men k, 10 off + 61 w, 5 m = 93 (~24% of 383); July 2 dominates (Bigelow w at the Trostle stand; horse pins); July 3 light per his own overshoot statement</t>
         </is>
       </c>
       <c r="AN164" s="5" t="n"/>
       <c r="AO164" s="5" t="inlineStr">
         <is>
-          <t>T4 (brigade grain)</t>
+          <t>T4 (brigade/line grain)</t>
         </is>
       </c>
     </row>
@@ -18661,12 +18661,12 @@
       </c>
       <c r="AL170" s="5" t="inlineStr">
         <is>
-          <t>[A window] FOUGHT THE CANNONADE THROUGHOUT under Hancock's counter-order; long-range ammo exhausted (or-27-1-hazard) -&gt; canister-only repulse fight</t>
+          <t>[C ~08:00] morning exchanges (3 of Cushing's limbers exploded; Woodruff 8 forenoon engagements); [A window] 'did not at first reply, till the fire of the enemy becoming too terrible' then fired ALL long-range ammo in 'an hour and a quarter'; [D] 'half the valley had been passed over... before the guns dared expend a round'; canister 'with terrible effect'; consolidation 5-&gt;3 batteries after (all or-27-1-hazard, read live pp. 477-481)</t>
         </is>
       </c>
       <c r="AM170" s="5" t="inlineStr">
         <is>
-          <t>150 (25k/120w/5m), 35% - highest-pct Union arty bde loss; flat-then-spike shape vs the silent-then-fire lines; 5 officer pins at battery grain</t>
+          <t>'one-third' of the brigade; 28k/119w/3m (report note) vs tablet 3+24k/5+114w/3m = 149; July 2 splits primary for Brown's (1k/7w/2m+24 horses) and Rorty's (1k/8w); 5 officer pins verbatim</t>
         </is>
       </c>
       <c r="AN170" s="5" t="n"/>
@@ -19024,7 +19024,7 @@
       <c r="AF174" s="5" t="n"/>
       <c r="AG174" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-xi-arty-osborn.md</t>
+          <t>Dossier: reconstruction/dossiers/us-xi-arty-osborn.md; HEADLINE: contemporary motive ('no satisfactory results') vs postwar ruse - ED-33's sharpest evidence; ruse verbatim unreachable (verified absence)</t>
         </is>
       </c>
       <c r="AH174" s="5" t="inlineStr">
@@ -19034,7 +19034,7 @@
       </c>
       <c r="AI174" s="5" t="inlineStr">
         <is>
-          <t>no men figure located (gap); ~39 guns secondary-grade; tablet-verified 9-battery roster is the stronger form</t>
+          <t>his OR: 26 guns organic Jul 1 -&gt; 52 on the hill Jul 2 morning (roster verbatim); ~36 his command Jul 3 (seminar); men figure still open; '~1,600 rounds' DOWNGRADED - his report: 'I am unable to give any definite estimate'</t>
         </is>
       </c>
       <c r="AJ174" s="5" t="inlineStr">
@@ -19049,12 +19049,12 @@
       </c>
       <c r="AL174" s="5" t="inlineStr">
         <is>
-          <t>[A window] counter-battery under the crossfire; [C ~14:30] THE CEASE-FIRE RUSE (proposed Osborn, adopted Hunt/Howard) = CA-J3A-4/5's sharpest component; [D] ~1,600 rounds into Pettigrew's left (secondary-grade)</t>
+          <t>[A window] deliberate counter-battery under the crossfire; [D] HIS OWN cease verbatim: 'as no satisfactory results were obtained, I ordered all our guns to cease firing... a few moments later the infantry of the enemy broke over the crest' - tightest Union cease-to-step-off coupling; [D] repulse fire 'havoc... truly surprising', artillery ignored by his order</t>
         </is>
       </c>
       <c r="AM174" s="5" t="inlineStr">
         <is>
-          <t>brigade K/W/M open (gap); Jul 1-2 dominate the shape; no Jul 3 officer pin located (negative)</t>
+          <t>tablet verbatim: 1 off + 6 men k, 3 off + 50 w, 9 m = 69; 98 horses (OR materiel table concurs); 1 gun captured/1 disabled/2 dismounted; pin: Wilkeson mw Jul 1 at the first fire -&gt; Bancroft</t>
         </is>
       </c>
       <c r="AN174" s="5" t="n"/>
@@ -21637,18 +21637,18 @@
       </c>
       <c r="AL203" s="5" t="inlineStr">
         <is>
-          <t>[C ~11:00] withhold-fire instruction; [C ~14:30] the slacken/cease order (CA-J3A-4); [D] Hancock counter-order conflict; [D] repulse-window battery reinforcements</t>
+          <t>[C 10:00] husband-ammunition instruction verbatim; [C 14:30] 'About 2.30 p.m. ... I directed that the fire should be gradually stopped... and the enemy soon slackened his fire also' (or-27-1-hunt) = CA-J3A-4 clock-fixed by its author; [C ~15:00] 'About 3 p.m., and soon after the enemy's fire had ceased, he formed a column of attack'; [B] 32,781 rounds of 270/gun carried - the economy arithmetic primary</t>
         </is>
       </c>
       <c r="AM203" s="5" t="inlineStr">
         <is>
-          <t>n/a; horse killed at Cowan's guns</t>
+          <t>army artillery return: 7 off + 98 men k, 33 off + 532 w, 67 m, 881 horses (or-27-1-hunt); July 3 officer list confirms Rorty/Cushing k, Woodruff/Milne mw</t>
         </is>
       </c>
       <c r="AN203" s="5" t="n"/>
       <c r="AO203" s="5" t="inlineStr">
         <is>
-          <t>T2 (command record)</t>
+          <t>T2 (command record; order events clock-fixed)</t>
         </is>
       </c>
     </row>
@@ -21921,7 +21921,7 @@
       </c>
       <c r="AL205" s="5" t="inlineStr">
         <is>
-          <t>[A window] served through the cannonade; [D] canister into Fry/Marshall closing on the wall; left-section gun's last double-shotted round into 26th NC (claim-arnold-canister)</t>
+          <t>[A window] served through the cannonade; 'expended every round, and the lines of the enemy still advanced' (or-27-1-hazard); [D] 'final shots were double-shotted canister' into Fry/Marshall; then withdrew his own AND Cushing's battery (Hazard); Hunt: withdrawn 'toward the close'</t>
         </is>
       </c>
       <c r="AM205" s="5" t="inlineStr">
@@ -22582,7 +22582,7 @@
       </c>
       <c r="AM210" s="5" t="inlineStr">
         <is>
-          <t>28 whole-battle (stone-sentinels), K/W split not carried - thin; mostly July 2; pins: Brown w Jul 2, Milne mw Jul 3 (on Cushing's rolls)</t>
+          <t>7k/19w/2m = 28 whole battle (tablet split closes the flag); July 2 PRIMARY: 1k/7w/2m + 24 horses killed 6 disabled, 2 guns to rear (or-27-1-hazard); Brown w neck by musket-shot; Milne mw on Cushing's rolls</t>
         </is>
       </c>
       <c r="AN210" s="5" t="n"/>
@@ -25346,7 +25346,7 @@
       </c>
       <c r="AM232" s="5" t="inlineStr">
         <is>
-          <t>10k/16w of 114 (stone-sentinels); inverse of the usual shape: steady loss under cannonade + spike at the melee; pins: Rorty k, Sheldon w [D ~15:20-30]</t>
+          <t>10k/16w of 114 (monument); July 2 PRIMARY: 1k/8w + 13 horses (or-27-1-hazard); 'entirely exhausted; its ammunition expended; its horses and men killed and disabled'; pins Rorty k (1 day in command), Sheldon w - confirmed in Hunt's officer list</t>
         </is>
       </c>
       <c r="AN232" s="5" t="n"/>
@@ -26865,12 +26865,12 @@
       </c>
       <c r="AL244" s="5" t="inlineStr">
         <is>
-          <t>[A window] under the cannonade, Napoleons outranged; [D 15:16-30] canister into Pettigrew's left with Osborn's converging fire - half of why ED-5 authors no northern breach</t>
+          <t>[C ~08:00-noon] EIGHT separate forenoon engagements (only II Corps battery active); [A window] under the cannonade; [D] canister into Pettigrew's left; last battery in action - 'Woodruff still remained in the grove, and poured death and destruction' (or-27-1-hazard)</t>
         </is>
       </c>
       <c r="AM244" s="5" t="inlineStr">
         <is>
-          <t>CONFLICT carried: 1k+29w (30) vs 1k+24w (25), same nominal source two extractions (oob-strengths); repulse-window dominated; pin: Woodruff mw [D in repulse fight]</t>
+          <t>RESOLVED toward 30: tablet 'killed 1 man, wounded 1 officer and 28 men' (re-verified); pin: Woodruff mw 'at the very moment of victory', d. Jul 4, buried on the field at his own request (or-27-1-hazard)</t>
         </is>
       </c>
       <c r="AN244" s="5" t="n"/>

</xml_diff>

<commit_message>
Audit d2: index + 23-unit overlay entries; master table regenerated (35 rows carry audited T-levels)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -7445,20 +7445,56 @@
           <t>reg-csa-2c-bn-latimer</t>
         </is>
       </c>
-      <c r="AB75" s="5" t="n"/>
+      <c r="AB75" s="5" t="inlineStr">
+        <is>
+          <t>unauthored</t>
+        </is>
+      </c>
       <c r="AC75" s="5" t="n"/>
       <c r="AD75" s="5" t="n"/>
       <c r="AE75" s="5" t="n"/>
       <c r="AF75" s="5" t="n"/>
-      <c r="AG75" s="5" t="n"/>
-      <c r="AH75" s="5" t="n"/>
-      <c r="AI75" s="5" t="n"/>
-      <c r="AJ75" s="5" t="n"/>
-      <c r="AK75" s="5" t="n"/>
-      <c r="AL75" s="5" t="n"/>
-      <c r="AM75" s="5" t="n"/>
+      <c r="AG75" s="5" t="inlineStr">
+        <is>
+          <t>Group dossier: reconstruction/dossiers/csa-2c-arty-ewell-wing.md - Brown's corps report corrects 'near-silence' to structured partial participation (ED-45 candidate)</t>
+        </is>
+      </c>
+      <c r="AH75" s="5" t="inlineStr">
+        <is>
+          <t>Latimer mw Jul 2 (Benner's Hill) -&gt; Capt. Raine</t>
+        </is>
+      </c>
+      <c r="AI75" s="5" t="inlineStr">
+        <is>
+          <t>356 (hop)</t>
+        </is>
+      </c>
+      <c r="AJ75" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 Benner's Hill (the Wainwright-group duel's other side); Jul 3 position unstated (open)</t>
+        </is>
+      </c>
+      <c r="AK75" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 withdrawal of three batteries under fire</t>
+        </is>
+      </c>
+      <c r="AL75" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 duel; Jul 3 ABSENT-FROM-RECORD in Brown's report (probably-limited, NOT attested-silent)</t>
+        </is>
+      </c>
+      <c r="AM75" s="5" t="inlineStr">
+        <is>
+          <t>Latimer mw = the pin; figures unfetched</t>
+        </is>
+      </c>
       <c r="AN75" s="5" t="n"/>
-      <c r="AO75" s="5" t="n"/>
+      <c r="AO75" s="5" t="inlineStr">
+        <is>
+          <t>T2 (group grain)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -7569,20 +7605,56 @@
           <t>reg-csa-1c-bn-cabell</t>
         </is>
       </c>
-      <c r="AB76" s="5" t="n"/>
+      <c r="AB76" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (consolidated line + post-assault forward move)</t>
+        </is>
+      </c>
       <c r="AC76" s="5" t="n"/>
       <c r="AD76" s="5" t="n"/>
       <c r="AE76" s="5" t="n"/>
       <c r="AF76" s="5" t="n"/>
-      <c r="AG76" s="5" t="n"/>
-      <c r="AH76" s="5" t="n"/>
-      <c r="AI76" s="5" t="n"/>
-      <c r="AJ76" s="5" t="n"/>
-      <c r="AK76" s="5" t="n"/>
-      <c r="AL76" s="5" t="n"/>
-      <c r="AM76" s="5" t="n"/>
+      <c r="AG76" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-bn-cabell.md</t>
+        </is>
+      </c>
+      <c r="AH76" s="5" t="inlineStr">
+        <is>
+          <t>Col. Cabell; Manly/Fraser/McCarthy/Carlton; 16 guns (tablet); Fraser w Jul 2 (dangerous), Carlton w Jul 3, Couper/Jennings w</t>
+        </is>
+      </c>
+      <c r="AI76" s="5" t="inlineStr">
+        <is>
+          <t>384 (build) vs 380 (SS compilation) - both hops carried (ED-38)</t>
+        </is>
+      </c>
+      <c r="AJ76" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 wood-edge line, right near the Emmitsburg road, 600-700 yd from the Peach Orchard guns; [C/D] Jul 3 six guns near a brick house on the road + Carlton/McCarthy en echelon BEFORE Pickett; [C ~16:00] post-assault line on the road ~700 yd from Cemetery Hill, held till night; j3-03 McCARTY label ~(3500,4670)</t>
+        </is>
+      </c>
+      <c r="AK76" s="5" t="inlineStr">
+        <is>
+          <t>[D] Jul 3 pre-dawn consolidation move north; [C ~16:00] forward onto the road; [D] withdrawal after dark</t>
+        </is>
+      </c>
+      <c r="AL76" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 duel; [C +7] 'about 1 p.m....over two hours' cannonade (chain-agreeing CSA clock); McCarthy morning probe fired 20 rounds; ROUNDS: ~3,300 Jul 2-3 (tablet) [B: ~206/gun]</t>
+        </is>
+      </c>
+      <c r="AM76" s="5" t="inlineStr">
+        <is>
+          <t>tablet 12k/30w/4m + 80 horses vs SS 15k/57w - carried (report table unfetched); Jul 2 pins Fraser; Jul 3 pins Carlton/Jennings</t>
+        </is>
+      </c>
       <c r="AN76" s="5" t="n"/>
-      <c r="AO76" s="5" t="n"/>
+      <c r="AO76" s="5" t="inlineStr">
+        <is>
+          <t>T4 (battalion grain)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -7693,20 +7765,56 @@
           <t>reg-csa-2c-bn-carter</t>
         </is>
       </c>
-      <c r="AB77" s="5" t="n"/>
+      <c r="AB77" s="5" t="inlineStr">
+        <is>
+          <t>attested-static</t>
+        </is>
+      </c>
       <c r="AC77" s="5" t="n"/>
       <c r="AD77" s="5" t="n"/>
       <c r="AE77" s="5" t="n"/>
       <c r="AF77" s="5" t="n"/>
-      <c r="AG77" s="5" t="n"/>
-      <c r="AH77" s="5" t="n"/>
-      <c r="AI77" s="5" t="n"/>
-      <c r="AJ77" s="5" t="n"/>
-      <c r="AK77" s="5" t="n"/>
-      <c r="AL77" s="5" t="n"/>
-      <c r="AM77" s="5" t="n"/>
+      <c r="AG77" s="5" t="inlineStr">
+        <is>
+          <t>Group dossier: reconstruction/dossiers/csa-2c-arty-ewell-wing.md - Brown's corps report corrects 'near-silence' to structured partial participation (ED-45 candidate)</t>
+        </is>
+      </c>
+      <c r="AH77" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Col. Carter (Rodes); Reese/W.Carter/Page/Fry</t>
+        </is>
+      </c>
+      <c r="AI77" s="5" t="inlineStr">
+        <is>
+          <t>384 (hop)</t>
+        </is>
+      </c>
+      <c r="AJ77" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 foot of the high ridge (Page vs O'Neal front); [C] Jul 3 ten rifled guns 'on the high ridge on the right and left of the railroad cut'</t>
+        </is>
+      </c>
+      <c r="AK77" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 legs; [C] Jul 2 ATTESTED IDLE ('held in readiness...not engaged')</t>
+        </is>
+      </c>
+      <c r="AL77" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 fights; [C] Jul 3 diversion fire on Cemetery Hill covering Dance; observation 'Their fire slackened, and finally ceased' = CSA-side CA-J3A-4-&gt;5 sequence witness [D]</t>
+        </is>
+      </c>
+      <c r="AM77" s="5" t="inlineStr">
+        <is>
+          <t>Jul 1 PRIMARY per-battery: Page 2k/2mw/26w + 17 horses; rest unfetched</t>
+        </is>
+      </c>
       <c r="AN77" s="5" t="n"/>
-      <c r="AO77" s="5" t="n"/>
+      <c r="AO77" s="5" t="inlineStr">
+        <is>
+          <t>T2 (group grain)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -7817,20 +7925,56 @@
           <t>reg-csa-2c-bn-dance</t>
         </is>
       </c>
-      <c r="AB78" s="5" t="n"/>
+      <c r="AB78" s="5" t="inlineStr">
+        <is>
+          <t>attested-static</t>
+        </is>
+      </c>
       <c r="AC78" s="5" t="n"/>
       <c r="AD78" s="5" t="n"/>
       <c r="AE78" s="5" t="n"/>
       <c r="AF78" s="5" t="n"/>
-      <c r="AG78" s="5" t="n"/>
-      <c r="AH78" s="5" t="n"/>
-      <c r="AI78" s="5" t="n"/>
-      <c r="AJ78" s="5" t="n"/>
-      <c r="AK78" s="5" t="n"/>
-      <c r="AL78" s="5" t="n"/>
-      <c r="AM78" s="5" t="n"/>
+      <c r="AG78" s="5" t="inlineStr">
+        <is>
+          <t>Group dossier: reconstruction/dossiers/csa-2c-arty-ewell-wing.md - Brown's corps report corrects 'near-silence' to structured partial participation (ED-45 candidate)</t>
+        </is>
+      </c>
+      <c r="AH78" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Dance; 2nd Corps reserve (Brown)</t>
+        </is>
+      </c>
+      <c r="AI78" s="5" t="inlineStr">
+        <is>
+          <t>480 (hop)</t>
+        </is>
+      </c>
+      <c r="AJ78" s="5" t="inlineStr">
+        <is>
+          <t>[C] Seminary/Oak ridge north sector, covered by Carter's ten rifles at the railroad cut</t>
+        </is>
+      </c>
+      <c r="AK78" s="5" t="inlineStr">
+        <is>
+          <t>none Jul 3 (static)</t>
+        </is>
+      </c>
+      <c r="AL78" s="5" t="inlineStr">
+        <is>
+          <t>[C] JUL 3 ENGAGED: 'The First Virginia Artillery...engaged the enemy's batteries, in order to divert their fire' (or-27-2-jtbrown) - the wing's firing battalion; Jul 2 Watson's/Smith's batteries aided Latimer's duel</t>
+        </is>
+      </c>
+      <c r="AM78" s="5" t="inlineStr">
+        <is>
+          <t>unfetched (open)</t>
+        </is>
+      </c>
       <c r="AN78" s="5" t="n"/>
-      <c r="AO78" s="5" t="n"/>
+      <c r="AO78" s="5" t="inlineStr">
+        <is>
+          <t>T2 (group grain)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -7941,20 +8085,56 @@
           <t>reg-csa-1c-bn-dearing</t>
         </is>
       </c>
-      <c r="AB79" s="5" t="n"/>
+      <c r="AB79" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (static line; daybreak advance attested)</t>
+        </is>
+      </c>
       <c r="AC79" s="5" t="n"/>
       <c r="AD79" s="5" t="n"/>
       <c r="AE79" s="5" t="n"/>
       <c r="AF79" s="5" t="n"/>
-      <c r="AG79" s="5" t="n"/>
-      <c r="AH79" s="5" t="n"/>
-      <c r="AI79" s="5" t="n"/>
-      <c r="AJ79" s="5" t="n"/>
-      <c r="AK79" s="5" t="n"/>
-      <c r="AL79" s="5" t="n"/>
-      <c r="AM79" s="5" t="n"/>
+      <c r="AG79" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-bn-dearing.md</t>
+        </is>
+      </c>
+      <c r="AH79" s="5" t="inlineStr">
+        <is>
+          <t>Maj. Dearing; Stribling/Caskie/Macon/Blount; 18 guns (tablet verbatim); Maj. Read w Jul 3 morning; HIS OWN OR REPORT FOUND (pass 1 assumed none)</t>
+        </is>
+      </c>
+      <c r="AI79" s="5" t="inlineStr">
+        <is>
+          <t>432 (B&amp;M-type hop per ED-38)</t>
+        </is>
+      </c>
+      <c r="AJ79" s="5" t="inlineStr">
+        <is>
+          <t>[C] arrived dusk Jul 2 (Pendleton chain); [C/D] daybreak Jul 3 to 'the crest of the hill immediately in front of the enemy's position'; RELATIONS PRIMARY: Cabell left+rear, Washington Arty right+rear; j3-03 labels CASKIE(3610,4480) BLOUNT(3670,4550) MACON(3620,4310) on the road-crest line</t>
+        </is>
+      </c>
+      <c r="AK79" s="5" t="inlineStr">
+        <is>
+          <t>[D] night march chain; [C/D] daybreak advance; withdrawal CONFLICT: tablet 'about 4 P.M.' vs his own 18:00 repulse fire - carried</t>
+        </is>
+      </c>
+      <c r="AL79" s="5" t="inlineStr">
+        <is>
+          <t>[D] daybreak skirmish (Stribling ~12 rounds); [A vs CA-J3A-1] deliberate by-battery fire at the signal; ammunition 'completely exhausted, excepting a few round in my rifled guns'; silent-under-fire 'upward of an hour'; rounds total attested-absent</t>
+        </is>
+      </c>
+      <c r="AM79" s="5" t="inlineStr">
+        <is>
+          <t>per-battery PRIMARY (3 of 4): Stribling 3w+10h, Macon 3k/3w+8h, Blount 5kw+12h; Caskie = extraction gap (flagged); all Jul 3</t>
+        </is>
+      </c>
       <c r="AN79" s="5" t="n"/>
-      <c r="AO79" s="5" t="n"/>
+      <c r="AO79" s="5" t="inlineStr">
+        <is>
+          <t>T4 (battalion grain)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -8086,7 +8266,7 @@
       </c>
       <c r="AI80" s="5" t="inlineStr">
         <is>
-          <t>CONFLICT: build 240 vs 338 (B&amp;M-type, hop flagged; '340' SNIPPET variant); 8 Napoleons + 2 12-pdr howitzers (tablet + OR concur) -&gt; ED-38 candidate</t>
+          <t>ADOPTED ED-38: 338 (B&amp;M-type, hop cited; build's 240 retired; '340' SNIPPET variant recorded); 8 Napoleons + 2 12-pdr howitzers (tablet + OR concur)</t>
         </is>
       </c>
       <c r="AJ80" s="5" t="inlineStr">
@@ -8225,20 +8405,56 @@
           <t>reg-csa-3c-bn-garnett</t>
         </is>
       </c>
-      <c r="AB81" s="5" t="n"/>
+      <c r="AB81" s="5" t="inlineStr">
+        <is>
+          <t>attested-static + ATTESTED SILENT Jul 3</t>
+        </is>
+      </c>
       <c r="AC81" s="5" t="n"/>
       <c r="AD81" s="5" t="n"/>
       <c r="AE81" s="5" t="n"/>
       <c r="AF81" s="5" t="n"/>
-      <c r="AG81" s="5" t="n"/>
-      <c r="AH81" s="5" t="n"/>
-      <c r="AI81" s="5" t="n"/>
-      <c r="AJ81" s="5" t="n"/>
-      <c r="AK81" s="5" t="n"/>
-      <c r="AL81" s="5" t="n"/>
-      <c r="AM81" s="5" t="n"/>
+      <c r="AG81" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-bn-garnett.md; ED-44 candidate (attested-silence rendering rule); subtracts 15 tubes from every cannonade gun-count claim</t>
+        </is>
+      </c>
+      <c r="AH81" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Col. J.J. Garnett / Maj. Richardson (rifle group); Maurin/Moore/Lewis/Grandy; 9 rifles + 6 smoothbores</t>
+        </is>
+      </c>
+      <c r="AI81" s="5" t="inlineStr">
+        <is>
+          <t>360 (hop, ED-38)</t>
+        </is>
+      </c>
+      <c r="AJ81" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 pike support; [C] Jul 2 rifles opposite Cemetery Hill; [C/D] Jul 3 rifles right of Pegram on Anderson's front; smoothbores in reserve (park class, 200m)</t>
+        </is>
+      </c>
+      <c r="AK81" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1/2/3 postings; [C] Jul 4 reoccupation; Richardson + 5 rifles to Imboden's train</t>
+        </is>
+      </c>
+      <c r="AL81" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 fire 15:00 -&gt; ~30 min before sunset (the one fire episode); JUL 3 NEGATIVE VERBATIM: 'did not fire a single shot, having received orders to that effect'; smoothbores 'bore no part in these actions'; tablet concurs</t>
+        </is>
+      </c>
+      <c r="AM81" s="5" t="inlineStr">
+        <is>
+          <t>UNFETCHED (p. 654 gap - open slot, not attested-absent)</t>
+        </is>
+      </c>
       <c r="AN81" s="5" t="n"/>
-      <c r="AO81" s="5" t="n"/>
+      <c r="AO81" s="5" t="inlineStr">
+        <is>
+          <t>T2 (negative-evidence)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -8349,20 +8565,56 @@
           <t>reg-csa-2c-bn-jones</t>
         </is>
       </c>
-      <c r="AB82" s="5" t="n"/>
+      <c r="AB82" s="5" t="inlineStr">
+        <is>
+          <t>unauthored</t>
+        </is>
+      </c>
       <c r="AC82" s="5" t="n"/>
       <c r="AD82" s="5" t="n"/>
       <c r="AE82" s="5" t="n"/>
       <c r="AF82" s="5" t="n"/>
-      <c r="AG82" s="5" t="n"/>
-      <c r="AH82" s="5" t="n"/>
-      <c r="AI82" s="5" t="n"/>
-      <c r="AJ82" s="5" t="n"/>
-      <c r="AK82" s="5" t="n"/>
-      <c r="AL82" s="5" t="n"/>
-      <c r="AM82" s="5" t="n"/>
+      <c r="AG82" s="5" t="inlineStr">
+        <is>
+          <t>Group dossier: reconstruction/dossiers/csa-2c-arty-ewell-wing.md - Brown's corps report corrects 'near-silence' to structured partial participation (ED-45 candidate)</t>
+        </is>
+      </c>
+      <c r="AH82" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Col. H.P. Jones (Early)</t>
+        </is>
+      </c>
+      <c r="AI82" s="5" t="inlineStr">
+        <is>
+          <t>290 (hop)</t>
+        </is>
+      </c>
+      <c r="AJ82" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 3 ATTESTED-ELSEWHERE: 'operated with the cavalry'; Tanner's battery with the wagon train (Williamsport)</t>
+        </is>
+      </c>
+      <c r="AK82" s="5" t="inlineStr">
+        <is>
+          <t>off-field legs (not researched this pass)</t>
+        </is>
+      </c>
+      <c r="AL82" s="5" t="inlineStr">
+        <is>
+          <t>[C] off the main field Jul 3 - subtracts ~16 tubes from cannonade census</t>
+        </is>
+      </c>
+      <c r="AM82" s="5" t="inlineStr">
+        <is>
+          <t>unfetched (open)</t>
+        </is>
+      </c>
       <c r="AN82" s="5" t="n"/>
-      <c r="AO82" s="5" t="n"/>
+      <c r="AO82" s="5" t="inlineStr">
+        <is>
+          <t>T2 (group grain)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -8597,20 +8849,56 @@
           <t>reg-csa-3c-bn-mcintosh</t>
         </is>
       </c>
-      <c r="AB84" s="5" t="n"/>
+      <c r="AB84" s="5" t="inlineStr">
+        <is>
+          <t>attested-static (Jul 2-3 line)</t>
+        </is>
+      </c>
       <c r="AC84" s="5" t="n"/>
       <c r="AD84" s="5" t="n"/>
       <c r="AE84" s="5" t="n"/>
       <c r="AF84" s="5" t="n"/>
-      <c r="AG84" s="5" t="n"/>
-      <c r="AH84" s="5" t="n"/>
-      <c r="AI84" s="5" t="n"/>
-      <c r="AJ84" s="5" t="n"/>
-      <c r="AK84" s="5" t="n"/>
-      <c r="AL84" s="5" t="n"/>
-      <c r="AM84" s="5" t="n"/>
+      <c r="AG84" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-bn-mcintosh.md</t>
+        </is>
+      </c>
+      <c r="AH84" s="5" t="inlineStr">
+        <is>
+          <t>Maj. McIntosh; Rice/Hurt/Wallace/Johnson; 16 guns incl. 2 Whitworths (tablet)</t>
+        </is>
+      </c>
+      <c r="AI84" s="5" t="inlineStr">
+        <is>
+          <t>384 (hop, ED-38)</t>
+        </is>
+      </c>
+      <c r="AJ84" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 Cashtown pike flank (railroad-cut enfilade); [C] Jul 2-3 'behind a stone wall, on the range of hills to the left of the town' (wall segment unresolved - radius 150m band; pass-3 crop item)</t>
+        </is>
+      </c>
+      <c r="AK84" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 in with Pender; [D] one-mile advance Jul 1-&gt;2; [C] Jul 4 afternoon withdrawal to Marsh Creek</t>
+        </is>
+      </c>
+      <c r="AL84" s="5" t="inlineStr">
+        <is>
+          <t>[C] railroad-cut enfilade Jul 1; [A window] Jul 3 sustained fire; ROUNDS ITEMIZED: 213 Napoleon + 1,049 rifle + 133 Whitworth = 1,395 (verbatim) [B: Napoleon 36/gun = range-limited signature]</t>
+        </is>
+      </c>
+      <c r="AM84" s="5" t="inlineStr">
+        <is>
+          <t>24 k&amp;w + 16 captured + 38 horses (report) vs tablet 7k/25w(16 captured) - k+w totals disagree, carried; no per-day split</t>
+        </is>
+      </c>
       <c r="AN84" s="5" t="n"/>
-      <c r="AO84" s="5" t="n"/>
+      <c r="AO84" s="5" t="inlineStr">
+        <is>
+          <t>T4 (battalion grain)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -8721,20 +9009,56 @@
           <t>reg-csa-2c-bn-nelson</t>
         </is>
       </c>
-      <c r="AB85" s="5" t="n"/>
+      <c r="AB85" s="5" t="inlineStr">
+        <is>
+          <t>attested-static</t>
+        </is>
+      </c>
       <c r="AC85" s="5" t="n"/>
       <c r="AD85" s="5" t="n"/>
       <c r="AE85" s="5" t="n"/>
       <c r="AF85" s="5" t="n"/>
-      <c r="AG85" s="5" t="n"/>
-      <c r="AH85" s="5" t="n"/>
-      <c r="AI85" s="5" t="n"/>
-      <c r="AJ85" s="5" t="n"/>
-      <c r="AK85" s="5" t="n"/>
-      <c r="AL85" s="5" t="n"/>
-      <c r="AM85" s="5" t="n"/>
+      <c r="AG85" s="5" t="inlineStr">
+        <is>
+          <t>Group dossier: reconstruction/dossiers/csa-2c-arty-ewell-wing.md - Brown's corps report corrects 'near-silence' to structured partial participation (ED-45 candidate)</t>
+        </is>
+      </c>
+      <c r="AH85" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Col. Nelson</t>
+        </is>
+      </c>
+      <c r="AI85" s="5" t="inlineStr">
+        <is>
+          <t>264 (hop)</t>
+        </is>
+      </c>
+      <c r="AJ85" s="5" t="inlineStr">
+        <is>
+          <t>[D] Oak Hill sector, position unstated in fetched pages (radius 300m, flagged)</t>
+        </is>
+      </c>
+      <c r="AK85" s="5" t="inlineStr">
+        <is>
+          <t>none stated</t>
+        </is>
+      </c>
+      <c r="AL85" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 3 'a portion' engaged (diversion mission, or-27-2-jtbrown); remainder = absence-of-record, NOT attested-silent</t>
+        </is>
+      </c>
+      <c r="AM85" s="5" t="inlineStr">
+        <is>
+          <t>unfetched (open)</t>
+        </is>
+      </c>
       <c r="AN85" s="5" t="n"/>
-      <c r="AO85" s="5" t="n"/>
+      <c r="AO85" s="5" t="inlineStr">
+        <is>
+          <t>T2 (group grain)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -8845,20 +9169,56 @@
           <t>reg-csa-3c-bn-pegram</t>
         </is>
       </c>
-      <c r="AB86" s="5" t="n"/>
+      <c r="AB86" s="5" t="inlineStr">
+        <is>
+          <t>attested-static (Jul 2-3 line)</t>
+        </is>
+      </c>
       <c r="AC86" s="5" t="n"/>
       <c r="AD86" s="5" t="n"/>
       <c r="AE86" s="5" t="n"/>
       <c r="AF86" s="5" t="n"/>
-      <c r="AG86" s="5" t="n"/>
-      <c r="AH86" s="5" t="n"/>
-      <c r="AI86" s="5" t="n"/>
-      <c r="AJ86" s="5" t="n"/>
-      <c r="AK86" s="5" t="n"/>
-      <c r="AL86" s="5" t="n"/>
-      <c r="AM86" s="5" t="n"/>
+      <c r="AG86" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-bn-pegram.md; ED-43 candidate (tablet casualty scope rule)</t>
+        </is>
+      </c>
+      <c r="AH86" s="5" t="inlineStr">
+        <is>
+          <t>Maj. Pegram / report by Capt. Brunson; Crenshaw/Marye/Brander/Zimmerman/McGraw; 20 guns (tablet); ordnance officer mw Jul 1</t>
+        </is>
+      </c>
+      <c r="AI86" s="5" t="inlineStr">
+        <is>
+          <t>480 (hop, ED-38)</t>
+        </is>
+      </c>
+      <c r="AJ86" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 eminence ~1 mi west (Marye's section fired the arc's opening 8-10 rounds); [C] Jul 2-3 right of Fairfield pike, ~1,400 yd from the Union guns; j3-03 labels BRANDER(3900,5900) ZIMMERMAN(3820,5720) MARYE(3720,5620)</t>
+        </is>
+      </c>
+      <c r="AK86" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 approach; [D] one-mile-forward repost Jul 1-&gt;2; static after; retreat losses recorded</t>
+        </is>
+      </c>
+      <c r="AL86" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 line forced Union guns back 'three distinct times'; [C] Jul 2 opportunistic enfilade; [A window] Jul 3 cannonade; ROUNDS: 3,800 three days (report verbatim; tablet concurs)</t>
+        </is>
+      </c>
+      <c r="AM86" s="5" t="inlineStr">
+        <is>
+          <t>PER-DAY PRIMARY (only one in set): Jul 1 2k/8w/6h; Jul 2 2k/7w/25h; Jul 3 10k/37w/38h; tablet's 47 = Jul 3 row misread as total (conflict carried)</t>
+        </is>
+      </c>
       <c r="AN86" s="5" t="n"/>
-      <c r="AO86" s="5" t="n"/>
+      <c r="AO86" s="5" t="inlineStr">
+        <is>
+          <t>T4 (battalion grain)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -18072,7 +18432,7 @@
       <c r="AF164" s="5" t="n"/>
       <c r="AG164" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-ar-1v-mcgilvery.md; his July 3 opening clock (OR pp.882-883) still unverified; ED-35 candidate: cast the line as a command unit</t>
+          <t>Dossier: reconstruction/dossiers/us-ar-1v-mcgilvery.md; ED-35 ADOPTED (cast the line as a command unit); ED-37 ADOPTED as recorded conflict (resolution open)</t>
         </is>
       </c>
       <c r="AH164" s="5" t="inlineStr">
@@ -18087,7 +18447,7 @@
       </c>
       <c r="AJ164" s="5" t="inlineStr">
         <is>
-          <t>[C ~15:30 Jul 2] Wheatfield Rd line; [C 17:45] retire 250 yd by stages; Trostle stand; 400-yd-rear line; [E Jul 3] low-ground line w/ earthwork, roster VERBATIM left-&gt;right incl. 'a New Jersey battery' + Rank's section (OR-vs-OOB conflict -&gt; ED-37); ref point Phillips (4212,4080)</t>
+          <t>[C ~15:30 Jul 2] Wheatfield Rd line; [C 17:45] retire 250 yd by stages; Trostle stand; 400-yd-rear line; [E Jul 3] low-ground line w/ earthwork, roster VERBATIM left-&gt;right incl. 'a New Jersey battery' + Rank's section (OR-vs-OOB conflict, ED-37 adopted-as-recorded); ref point Phillips (4212,4080)</t>
         </is>
       </c>
       <c r="AK164" s="5" t="inlineStr">
@@ -18537,20 +18897,56 @@
           <t>reg-us-i-arty</t>
         </is>
       </c>
-      <c r="AB169" s="5" t="n"/>
+      <c r="AB169" s="5" t="inlineStr">
+        <is>
+          <t>unauthored (components partially in-build)</t>
+        </is>
+      </c>
       <c r="AC169" s="5" t="n"/>
       <c r="AD169" s="5" t="n"/>
       <c r="AE169" s="5" t="n"/>
       <c r="AF169" s="5" t="n"/>
-      <c r="AG169" s="5" t="n"/>
-      <c r="AH169" s="5" t="n"/>
-      <c r="AI169" s="5" t="n"/>
-      <c r="AJ169" s="5" t="n"/>
-      <c r="AK169" s="5" t="n"/>
-      <c r="AL169" s="5" t="n"/>
-      <c r="AM169" s="5" t="n"/>
+      <c r="AG169" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-i-arty-wainwright.md; p. 356 fetch gap recorded</t>
+        </is>
+      </c>
+      <c r="AH169" s="5" t="inlineStr">
+        <is>
+          <t>Col. Wainwright; Hall/Stevens/Reynolds-Wilber/Cooper/Stewart batteries; Davison w Jul 1 -&gt; Sgt. Mitchell commended</t>
+        </is>
+      </c>
+      <c r="AI169" s="5" t="inlineStr">
+        <is>
+          <t>no brigade figure (negative); component strengths on battery rows</t>
+        </is>
+      </c>
+      <c r="AJ169" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 Seminary Ridge; [C] E Cemetery Hill layout VERBATIM (B/4US across the road, I/1NY, Cooper, Reynolds = 13 three-inch guns; 5th ME 50 yd forward on the knoll) - the East-Hill left-to-right frame</t>
+        </is>
+      </c>
+      <c r="AK169" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 fighting withdrawal (peremptory order); [C] Jul 2 Cooper-out/Ricketts-in rotation; [A 15:00] Cooper detached to left centre Jul 3</t>
+        </is>
+      </c>
+      <c r="AL169" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 fight (83 men + 80 horses day-1 loss); [C] Jul 2 wheat-field battery silenced in ~90 min (28 dead horses = Latimer's ground); dusk assault 'almost entirely repelled by the artillery'; Jul 3 occasional + general; rounds via components (Cooper 1,050; Breck 1,290 itemized; Ricketts 1,200; Hill WV 1,120)</t>
+        </is>
+      </c>
+      <c r="AM169" s="5" t="inlineStr">
+        <is>
+          <t>Jul 1 primary 83+80 horses; Jul 2-3 on component returns (no roll-up fetched)</t>
+        </is>
+      </c>
       <c r="AN169" s="5" t="n"/>
-      <c r="AO169" s="5" t="n"/>
+      <c r="AO169" s="5" t="inlineStr">
+        <is>
+          <t>T4 (group grain)</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -18636,7 +19032,7 @@
       <c r="AF170" s="5" t="n"/>
       <c r="AG170" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-ii-arty-hazard.md; ED-34 candidate (activity classes)</t>
+          <t>Dossier: reconstruction/dossiers/us-ii-arty-hazard.md; ED-34 ADOPTED (fought-to-exhaustion class exemplar)</t>
         </is>
       </c>
       <c r="AH170" s="5" t="inlineStr">
@@ -19024,7 +19420,7 @@
       <c r="AF174" s="5" t="n"/>
       <c r="AG174" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-xi-arty-osborn.md; HEADLINE: contemporary motive ('no satisfactory results') vs postwar ruse - ED-33's sharpest evidence; ruse verbatim unreachable (verified absence)</t>
+          <t>Dossier: reconstruction/dossiers/us-xi-arty-osborn.md; HEADLINE: contemporary motive ('no satisfactory results') vs postwar ruse - ED-33 adopted on this evidence; ruse verbatim unreachable (verified absence)</t>
         </is>
       </c>
       <c r="AH174" s="5" t="inlineStr">
@@ -22045,20 +22441,56 @@
           <t>reg-us-ar-hq</t>
         </is>
       </c>
-      <c r="AB206" s="5" t="n"/>
+      <c r="AB206" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (park track)</t>
+        </is>
+      </c>
       <c r="AC206" s="5" t="n"/>
       <c r="AD206" s="5" t="n"/>
       <c r="AE206" s="5" t="n"/>
       <c r="AF206" s="5" t="n"/>
-      <c r="AG206" s="5" t="n"/>
-      <c r="AH206" s="5" t="n"/>
-      <c r="AI206" s="5" t="n"/>
-      <c r="AJ206" s="5" t="n"/>
-      <c r="AK206" s="5" t="n"/>
-      <c r="AL206" s="5" t="n"/>
-      <c r="AM206" s="5" t="n"/>
+      <c r="AG206" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ar-hq-tyler-park.md; ED-42 candidate (issues-vs-expenditures two-ledger rule)</t>
+        </is>
+      </c>
+      <c r="AH206" s="5" t="inlineStr">
+        <is>
+          <t>Tyler -&gt; Robertson after Jul 3 incapacitation (register; report silent - carried); 5 brigades + ammunition train; Gillett ordnance officer</t>
+        </is>
+      </c>
+      <c r="AI206" s="5" t="inlineStr">
+        <is>
+          <t>2,375 / 114 guns nominal (hop) minus B+M 1st CT Heavy (to Westminster, verbatim)</t>
+        </is>
+      </c>
+      <c r="AJ206" s="5" t="inlineStr">
+        <is>
+          <t>[C] June 29-Jul 1 march (Frederick-&gt;Taneytown; 22:30 Jul 1 report to Gibbon); [C] park ~1.5 mi from town; [C] 70 wagons sent rear morning Jul 3</t>
+        </is>
+      </c>
+      <c r="AK206" s="5" t="inlineStr">
+        <is>
+          <t>[C] march legs; [C] Jul 2 six batteries/34 guns to Sickles (moves by detachment); [A window] crisis battery legs originate here</t>
+        </is>
+      </c>
+      <c r="AL206" s="5" t="inlineStr">
+        <is>
+          <t>AMMUNITION LEDGER PRIMARY: 19,189 rounds ISSUED + 4,694 left (Gillett annex) - the supply-side physics of Hunt's economy order; wagon-doctrine caution verbatim</t>
+        </is>
+      </c>
+      <c r="AM206" s="5" t="inlineStr">
+        <is>
+          <t>distributed to component returns (Turnbull's 1+8k/14w/45 horses worst); consolidated tables pp. 874-877 unfetched (open)</t>
+        </is>
+      </c>
       <c r="AN206" s="5" t="n"/>
-      <c r="AO206" s="5" t="n"/>
+      <c r="AO206" s="5" t="inlineStr">
+        <is>
+          <t>T3 (park/command grain)</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -22552,7 +22984,7 @@
       <c r="AF210" s="5" t="n"/>
       <c r="AG210" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-btty-brown.md; ED-33 candidate on what 'the 18 guns have gone' observed</t>
+          <t>Dossier: reconstruction/dossiers/us-btty-brown.md; ED-33 ADOPTED: his ~14:40 withdrawal = the contributing event behind Alexander's '18 guns' reading (Osborn's cease primary)</t>
         </is>
       </c>
       <c r="AH210" s="5" t="inlineStr">
@@ -22701,20 +23133,56 @@
           <t>reg-us-i-b4</t>
         </is>
       </c>
-      <c r="AB211" s="5" t="n"/>
+      <c r="AB211" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC211" s="5" t="n"/>
       <c r="AD211" s="5" t="n"/>
       <c r="AE211" s="5" t="n"/>
       <c r="AF211" s="5" t="n"/>
-      <c r="AG211" s="5" t="n"/>
-      <c r="AH211" s="5" t="n"/>
-      <c r="AI211" s="5" t="n"/>
-      <c r="AJ211" s="5" t="n"/>
-      <c r="AK211" s="5" t="n"/>
-      <c r="AL211" s="5" t="n"/>
-      <c r="AM211" s="5" t="n"/>
+      <c r="AG211" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-cooper.md; best tier-B rounds basis in the set</t>
+        </is>
+      </c>
+      <c r="AH211" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Cooper; B/1st PA; I Corps bde (Wainwright); 4x 3-in rifles</t>
+        </is>
+      </c>
+      <c r="AI211" s="5" t="inlineStr">
+        <is>
+          <t>114 (monument verbatim; build concurs)</t>
+        </is>
+      </c>
+      <c r="AJ211" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 noon left of 3rd Div then Seminary (Reynolds Ave mon (3172,7044)); [C] E Cemetery Hill Jul 1 dusk - Jul 3 (Wainwright layout verbatim; main mon (5050,5776)); [A tablet 15:00] Hancock Ave tablet (4473,4096) = ridge crest at I/II Corps boundary - RESOLVES pass-1 'joins McGilvery' slot (sheet-vs-tablet conflict carried)</t>
+        </is>
+      </c>
+      <c r="AK211" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 legs; [C ~19:00 Jul 2] out to refit (Ricketts in); [A vs CA-J3A-5; B: 8-12 min] the 15:00 during-cannonade transfer</t>
+        </is>
+      </c>
+      <c r="AL211" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 25-shot opening + Seminary fight; [C] Jul 2 2.5-h silencing duel; [C] Jul 3 case-&gt;canister rout; ROUNDS PER DAY: ~400/500/150 = 1,050 (report + monument concur) [B: Jul 3 ~20-25 min fire]</t>
+        </is>
+      </c>
+      <c r="AM211" s="5" t="inlineStr">
+        <is>
+          <t>12 total (3k/9w); PER-DAY PINS: Jul 2 2k/6w, Jul 3 1w (report) - monument's July-3 heading wrong by the battery's own report</t>
+        </is>
+      </c>
       <c r="AN211" s="5" t="n"/>
-      <c r="AO211" s="5" t="n"/>
+      <c r="AO211" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -22825,20 +23293,56 @@
           <t>reg-us-vi-b2</t>
         </is>
       </c>
-      <c r="AB212" s="5" t="n"/>
+      <c r="AB212" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (T5 window in Angle cast)</t>
+        </is>
+      </c>
       <c r="AC212" s="5" t="n"/>
       <c r="AD212" s="5" t="n"/>
       <c r="AE212" s="5" t="n"/>
       <c r="AF212" s="5" t="n"/>
-      <c r="AG212" s="5" t="n"/>
-      <c r="AH212" s="5" t="n"/>
-      <c r="AI212" s="5" t="n"/>
-      <c r="AJ212" s="5" t="n"/>
-      <c r="AK212" s="5" t="n"/>
-      <c r="AL212" s="5" t="n"/>
-      <c r="AM212" s="5" t="n"/>
+      <c r="AG212" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-cowan.md; ED-40 candidate (crisis slot naming)</t>
+        </is>
+      </c>
+      <c r="AH212" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Cowan unwounded; 6x 3-in rifles; VI Corps battery detached to II Corps front; Hunt at the guns at climax</t>
+        </is>
+      </c>
+      <c r="AI212" s="5" t="inlineStr">
+        <is>
+          <t>113 (stone-sentinels, single-source; build concurs)</t>
+        </is>
+      </c>
+      <c r="AJ212" s="5" t="inlineStr">
+        <is>
+          <t>[C] VI Corps march arrival 22:00 Jul 2; [C ~10:00] to Newton, park &lt;100 yd rear; [A vs CA-J3A-7..9] the Brown slot: mon-cowan (4428,4788), 17m from build hold; j3-03 'COWAN' between CUSHING and BROWN</t>
+        </is>
+      </c>
+      <c r="AK212" s="5" t="inlineStr">
+        <is>
+          <t>[C] march legs; [A] slot-fill move at a gallop ~150m [B: ~1 min]</t>
+        </is>
+      </c>
+      <c r="AL212" s="5" t="inlineStr">
+        <is>
+          <t>[C +67] opening 'about noon' (early pole, rule 4); [A] canister 200 yd -&gt; &lt;20 yd ('DOUBLE CANISTER AT TEN YARDS' monument); [D] exploded 4 limbers of one CSA battery; rounds attested-absent</t>
+        </is>
+      </c>
+      <c r="AM212" s="5" t="inlineStr">
+        <is>
+          <t>5k/6w + 14 horses (report; monument + SS page variants carried); single-episode Jul 3 profile</t>
+        </is>
+      </c>
       <c r="AN212" s="5" t="n"/>
-      <c r="AO212" s="5" t="n"/>
+      <c r="AO212" s="5" t="inlineStr">
+        <is>
+          <t>T4 (full arc; T5 window in-build)</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -23569,20 +24073,56 @@
           <t>reg-us-ar-4v-5</t>
         </is>
       </c>
-      <c r="AB218" s="5" t="n"/>
+      <c r="AB218" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC218" s="5" t="n"/>
       <c r="AD218" s="5" t="n"/>
       <c r="AE218" s="5" t="n"/>
       <c r="AF218" s="5" t="n"/>
-      <c r="AG218" s="5" t="n"/>
-      <c r="AH218" s="5" t="n"/>
-      <c r="AI218" s="5" t="n"/>
-      <c r="AJ218" s="5" t="n"/>
-      <c r="AK218" s="5" t="n"/>
-      <c r="AL218" s="5" t="n"/>
-      <c r="AM218" s="5" t="n"/>
+      <c r="AG218" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-fitzhugh.md; ED-41 candidate (crisis-reinforcement class)</t>
+        </is>
+      </c>
+      <c r="AH218" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Fitzhugh (also cmdg 4th Vol Bde); K/1st NY + 11th NY attached; 6x 3-in rifles</t>
+        </is>
+      </c>
+      <c r="AI218" s="5" t="inlineStr">
+        <is>
+          <t>149 (stone-sentinels; build concurs)</t>
+        </is>
+      </c>
+      <c r="AJ218" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2-3 Baltimore pike near Slocum; [crisis] 'near the stone fence in front of General Webb's division', enemy at 75 yd; monument on Cemetery Hill = pre-crisis semantics</t>
+        </is>
+      </c>
+      <c r="AK218" s="5" t="inlineStr">
+        <is>
+          <t>13:00-vs-15:00 move-clock CONFLICT (his 1 p.m. vs Parsons's 3 p.m. + SS at-the-gallop); 89-round expenditure is the physical tiebreaker toward 15:00</t>
+        </is>
+      </c>
+      <c r="AL218" s="5" t="inlineStr">
+        <is>
+          <t>[A window] first attack collapsed in 30-45 min of his fire; second (Wilcox/Lang) broken by enfilade; ROUNDS ITEMIZED: 57 percussion + 15 shrapnel + 17 time = 89 [B: ~8-10 min full-battery fire]</t>
+        </is>
+      </c>
+      <c r="AM218" s="5" t="inlineStr">
+        <is>
+          <t>K+11NY: 7w + 5 horses; brigade 36 (2k/34w tablet); single-episode</t>
+        </is>
+      </c>
       <c r="AN218" s="5" t="n"/>
-      <c r="AO218" s="5" t="n"/>
+      <c r="AO218" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -24685,20 +25225,56 @@
           <t>reg-us-ar-4v-3</t>
         </is>
       </c>
-      <c r="AB227" s="5" t="n"/>
+      <c r="AB227" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC227" s="5" t="n"/>
       <c r="AD227" s="5" t="n"/>
       <c r="AE227" s="5" t="n"/>
       <c r="AF227" s="5" t="n"/>
-      <c r="AG227" s="5" t="n"/>
-      <c r="AH227" s="5" t="n"/>
-      <c r="AI227" s="5" t="n"/>
-      <c r="AJ227" s="5" t="n"/>
-      <c r="AK227" s="5" t="n"/>
-      <c r="AL227" s="5" t="n"/>
-      <c r="AM227" s="5" t="n"/>
+      <c r="AG227" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-parsons.md; ED-37 file: Parsons ELIMINATED as McGilvery's 'New Jersey battery' (was at the pike all morning); Clark's B/1st NJ the surviving candidate</t>
+        </is>
+      </c>
+      <c r="AH227" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Parsons; A/1st NJ; 4th Vol Bde; 6 guns (armament single-source, flagged)</t>
+        </is>
+      </c>
+      <c r="AI227" s="5" t="inlineStr">
+        <is>
+          <t>116 (build compilation, hop flagged)</t>
+        </is>
+      </c>
+      <c r="AJ227" s="5" t="inlineStr">
+        <is>
+          <t>[C] Baltimore pike Jul 2-3; [C +10] 'about one-fourth of a mile south of Gettysburg Cemetery and near the Second Division' - vs Fitzhugh's in-front-of-Webb (tension carried); pair order: Parsons left, Fitzhugh right</t>
+        </is>
+      </c>
+      <c r="AK227" s="5" t="inlineStr">
+        <is>
+          <t>[C ~15:00] Hunt's order, pike-&gt;ridge at speed [B: 5-8 min]</t>
+        </is>
+      </c>
+      <c r="AL227" s="5" t="inlineStr">
+        <is>
+          <t>[A] case into the advancing infantry (~40 rds per Fitzhugh); [D] then ~120 shot + ~80 shell counter-battery until Hunt's cease = ~240 rounds total [B: 20-30 min]</t>
+        </is>
+      </c>
+      <c r="AM227" s="5" t="inlineStr">
+        <is>
+          <t>2k/7w + 5 horses; single-episode</t>
+        </is>
+      </c>
       <c r="AN227" s="5" t="n"/>
-      <c r="AO227" s="5" t="n"/>
+      <c r="AO227" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -25181,20 +25757,56 @@
           <t>reg-us-v-b4</t>
         </is>
       </c>
-      <c r="AB231" s="5" t="n"/>
+      <c r="AB231" s="5" t="inlineStr">
+        <is>
+          <t>attested-static (Jul 3)</t>
+        </is>
+      </c>
       <c r="AC231" s="5" t="n"/>
       <c r="AD231" s="5" t="n"/>
       <c r="AE231" s="5" t="n"/>
       <c r="AF231" s="5" t="n"/>
-      <c r="AG231" s="5" t="n"/>
-      <c r="AH231" s="5" t="n"/>
-      <c r="AI231" s="5" t="n"/>
-      <c r="AJ231" s="5" t="n"/>
-      <c r="AK231" s="5" t="n"/>
-      <c r="AL231" s="5" t="n"/>
-      <c r="AM231" s="5" t="n"/>
+      <c r="AG231" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-rittenhouse.md; rittenhouse-mollus-1887 = the T-ceiling item</t>
+        </is>
+      </c>
+      <c r="AH231" s="5" t="inlineStr">
+        <is>
+          <t>Hazlett k Jul 2 on the summit -&gt; Rittenhouse; D/5th US; 6x 10-pdr Parrotts; V Corps bde (Martin)</t>
+        </is>
+      </c>
+      <c r="AI231" s="5" t="inlineStr">
+        <is>
+          <t>73 = 2 off + 71 men (tablet)</t>
+        </is>
+      </c>
+      <c r="AJ231" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet 17:45 Jul 2] LRT summit, hand-hauled; ~(4430,2600) +-50m (j3-03 HAZLETT'S bar; NO register marker - gap flagged); attested-static Jul 3</t>
+        </is>
+      </c>
+      <c r="AK231" s="5" t="inlineStr">
+        <is>
+          <t>[C 16:30-17:45 Jul 2] march + summit haul [B: haul is the constraint]; none after</t>
+        </is>
+      </c>
+      <c r="AL231" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 evening fire into the Devil's Den flank; [E + cross-cited] Jul 3 enfilade on the assault (Hunt's 'McGilvery and Rittenhouse...drift' statement); OWN ACCOUNT ACCESS-FAILED (gdg.org TLS) - EC5 deliberately thin; rounds unfetched</t>
+        </is>
+      </c>
+      <c r="AM231" s="5" t="inlineStr">
+        <is>
+          <t>14 (1 off + 8 men k, 5 w, tablet; ~19% of 73); Jul 2 dominates [D]; brigade frame 44 total (Martin)</t>
+        </is>
+      </c>
       <c r="AN231" s="5" t="n"/>
-      <c r="AO231" s="5" t="n"/>
+      <c r="AO231" s="5" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -26333,20 +26945,56 @@
           <t>reg-us-ar-1r-4</t>
         </is>
       </c>
-      <c r="AB240" s="5" t="n"/>
+      <c r="AB240" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC240" s="5" t="n"/>
       <c r="AD240" s="5" t="n"/>
       <c r="AE240" s="5" t="n"/>
       <c r="AF240" s="5" t="n"/>
-      <c r="AG240" s="5" t="n"/>
-      <c r="AH240" s="5" t="n"/>
-      <c r="AI240" s="5" t="n"/>
-      <c r="AJ240" s="5" t="n"/>
-      <c r="AK240" s="5" t="n"/>
-      <c r="AL240" s="5" t="n"/>
-      <c r="AM240" s="5" t="n"/>
+      <c r="AG240" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-weir.md; Tyler's 'no report received' vs the printed report - OR artifact recorded</t>
+        </is>
+      </c>
+      <c r="AH240" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Weir (w Jul 3 per register; report silent - carried); 6 Napoleons; 1st Regular Bde (Ransom w), Artillery Reserve</t>
+        </is>
+      </c>
+      <c r="AI240" s="5" t="inlineStr">
+        <is>
+          <t>123 = 2 off + 121 men (tablet verbatim)</t>
+        </is>
+      </c>
+      <c r="AJ240" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 park then 16:00 forward position ~500 yd (Hancock order); 3 guns lost/recaptured by 13th VT (tablet verbatim); [D] Jul 3 fell back, then 'conducted to General Webb's position...under a heavy musketry fire' (crisis window)</t>
+        </is>
+      </c>
+      <c r="AK240" s="5" t="inlineStr">
+        <is>
+          <t>[C 16:00 Jul 2] park-&gt;front [B: 15-20 min]; [D] Jul 2 overrun scramble; [D] Jul 3 crisis move to Webb</t>
+        </is>
+      </c>
+      <c r="AL240" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 shot/case, canister out; [D] Jul 3 canister at short range; ROUNDS PRIMARY: 50 shot + 160 case + 70 canister = 280 (or-27-1-weir) [B: ~23-31 min cumulative battery fire]</t>
+        </is>
+      </c>
+      <c r="AM240" s="5" t="inlineStr">
+        <is>
+          <t>16 = 2k + 2 off/12 men w (tablet); Jul 2 dominates [D]; Baldwin w pin</t>
+        </is>
+      </c>
       <c r="AN240" s="5" t="n"/>
-      <c r="AO240" s="5" t="n"/>
+      <c r="AO240" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -26457,20 +27105,56 @@
           <t>reg-us-xi-b2</t>
         </is>
       </c>
-      <c r="AB241" s="5" t="n"/>
+      <c r="AB241" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC241" s="5" t="n"/>
       <c r="AD241" s="5" t="n"/>
       <c r="AE241" s="5" t="n"/>
       <c r="AF241" s="5" t="n"/>
-      <c r="AG241" s="5" t="n"/>
-      <c r="AH241" s="5" t="n"/>
-      <c r="AI241" s="5" t="n"/>
-      <c r="AJ241" s="5" t="n"/>
-      <c r="AK241" s="5" t="n"/>
-      <c r="AL241" s="5" t="n"/>
-      <c r="AM241" s="5" t="n"/>
+      <c r="AG241" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-wheeler.md; three-halt rhythm = pass-3 approach-leg pacing input</t>
+        </is>
+      </c>
+      <c r="AH241" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Wheeler; 13th NY Indep; XI Corps bde (Osborn); 4x 3-in rifles</t>
+        </is>
+      </c>
+      <c r="AI241" s="5" t="inlineStr">
+        <is>
+          <t>118 (stone-sentinels; build concurs)</t>
+        </is>
+      </c>
+      <c r="AJ241" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 Dilger's right then wheat field; [E] Jul 2-3 Cemetery Hill (Osborn group); [C stated 16:00, profile -35] crisis position by Hancock, enemy column 400 yd off</t>
+        </is>
+      </c>
+      <c r="AK241" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 double-quick legs + retreat; [C] crisis move hill-&gt;II Corps front [B: 3-5 min; build path 668m matches]</t>
+        </is>
+      </c>
+      <c r="AL241" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 counter-battery; [E] hill group fire; [A] crisis canister enfilade - column 'brought to a halt three times'; ROUNDS: 850 whole battle [B: ~212/gun, needs per-day split - none stated]</t>
+        </is>
+      </c>
+      <c r="AM241" s="5" t="inlineStr">
+        <is>
+          <t>10w/3m + 12 horses (report; monument 8w variant); Jul 1 vs Jul 3 split bracketed only</t>
+        </is>
+      </c>
       <c r="AN241" s="5" t="n"/>
-      <c r="AO241" s="5" t="n"/>
+      <c r="AO241" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -29173,20 +29857,56 @@
           <t>reg-us-ii-2-3</t>
         </is>
       </c>
-      <c r="AB265" s="5" t="n"/>
+      <c r="AB265" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (crisis rush authored in Angle cast)</t>
+        </is>
+      </c>
       <c r="AC265" s="5" t="n"/>
       <c r="AD265" s="5" t="n"/>
       <c r="AE265" s="5" t="n"/>
       <c r="AF265" s="5" t="n"/>
-      <c r="AG265" s="5" t="n"/>
-      <c r="AH265" s="5" t="n"/>
-      <c r="AI265" s="5" t="n"/>
-      <c r="AJ265" s="5" t="n"/>
-      <c r="AK265" s="5" t="n"/>
-      <c r="AL265" s="5" t="n"/>
-      <c r="AM265" s="5" t="n"/>
+      <c r="AG265" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-2-3-hall.md; p.438 extraction gap + 'Should be Arnold's' footnote -&gt; ED-40 candidate</t>
+        </is>
+      </c>
+      <c r="AH265" s="5" t="inlineStr">
+        <is>
+          <t>Col. Hall unwounded; Revere (20MA) mw Jul 2, Steele (7MI) k, Thoman (59NY) k Jul 3 (or-27-1-hall pp.435-440, stub UPGRADED)</t>
+        </is>
+      </c>
+      <c r="AI265" s="5" t="inlineStr">
+        <is>
+          <t>920 (build compilation, hop flagged; division 3,773 primary via Harrow)</t>
+        </is>
+      </c>
+      <c r="AJ265" s="5" t="inlineStr">
+        <is>
+          <t>[E] two-line layout: wall row 59NY(4375,4756) 7MI(4379,4728) 20MA(4381,4688) + support row 42NY(4447,4750) 19MA(4445,4692); rails-shelter verbatim; Bachelder j3-03 concurs</t>
+        </is>
+      </c>
+      <c r="AK265" s="5" t="inlineStr">
+        <is>
+          <t>[D Jul 2] 42NY+19MA to Humphreys; [A vs CA-J3A-9] by-the-flank rush to Webb ~150-250m [B: 3-5 min]; 10-min melee duration stated</t>
+        </is>
+      </c>
+      <c r="AL265" s="5" t="inlineStr">
+        <is>
+          <t>[C +5] 'At 1 o'clock' opening; 'At 3 o'clock exactly the fire slackened, and his first line advanced'; fire ladder 200 yd -&gt; 50 paces; 20 flags in 100 yd square</t>
+        </is>
+      </c>
+      <c r="AM265" s="5" t="inlineStr">
+        <is>
+          <t>tablet 377 (6+75k/29+253w/14m); Jul 2 share attested; pins Revere mw Jul 2, Steele/Thoman k Jul 3 crisis</t>
+        </is>
+      </c>
       <c r="AN265" s="5" t="n"/>
-      <c r="AO265" s="5" t="n"/>
+      <c r="AO265" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
@@ -29308,7 +30028,7 @@
       <c r="AF266" s="5" t="n"/>
       <c r="AG266" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-i-3-3-stannard.md; wheel clock verified-negative (no witness clock exists)</t>
+          <t>Dossier: reconstruction/dossiers/us-i-3-3-stannard.md; ED-32 adopted 2026-07-11; wheel clock verified-negative (no witness clock exists)</t>
         </is>
       </c>
       <c r="AH266" s="5" t="inlineStr">
@@ -29318,7 +30038,7 @@
       </c>
       <c r="AI266" s="5" t="inlineStr">
         <is>
-          <t>1,950 brigade (stone-sentinels) vs 1,788 sum of engaged rgts (480+647+661) - ~160-man gap, both carried (oob-strengths #3)</t>
+          <t>ADOPTED ED-32: 1,788 engaged = sum of engaged rgts (480+647+661); the 1,950 brigade figure failed re-verification and is kept only as a recorded failed reading (oob-strengths #3)</t>
         </is>
       </c>
       <c r="AJ266" s="5" t="inlineStr">
@@ -32677,20 +33397,56 @@
           <t>reg-us-ii-2-1</t>
         </is>
       </c>
-      <c r="AB293" s="5" t="n"/>
+      <c r="AB293" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (crisis incline-right)</t>
+        </is>
+      </c>
       <c r="AC293" s="5" t="n"/>
       <c r="AD293" s="5" t="n"/>
       <c r="AE293" s="5" t="n"/>
       <c r="AF293" s="5" t="n"/>
-      <c r="AG293" s="5" t="n"/>
-      <c r="AH293" s="5" t="n"/>
-      <c r="AI293" s="5" t="n"/>
-      <c r="AJ293" s="5" t="n"/>
-      <c r="AK293" s="5" t="n"/>
-      <c r="AL293" s="5" t="n"/>
-      <c r="AM293" s="5" t="n"/>
+      <c r="AG293" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-2-1-harrow.md; division-sum gap 3,580 vs 3,773 recorded</t>
+        </is>
+      </c>
+      <c r="AH293" s="5" t="inlineStr">
+        <is>
+          <t>Harrow to division (Gibbon w) -&gt; Heath (19ME) took brigade; Ward (15MA)/Huston (82NY) mw Jul 2; Colvill/Adams/Downie (1MN) w</t>
+        </is>
+      </c>
+      <c r="AI293" s="5" t="inlineStr">
+        <is>
+          <t>1,410 (build, hop); division primary 3,773 in / 1,657 lost (or-27-1-harrow)</t>
+        </is>
+      </c>
+      <c r="AJ293" s="5" t="inlineStr">
+        <is>
+          <t>[E] single-line axis x~4384, z 4560-4645: 19ME(4384,4644) 15MA(4384,4610) 1MN(4385,4567) 82NY(4385,4564); Rorty's guns inside the span (4412,4597)</t>
+        </is>
+      </c>
+      <c r="AK293" s="5" t="inlineStr">
+        <is>
+          <t>[C Jul 2] 15MA+82NY to Emmitsburg Rd + retire; [D] 1MN charge; [A vs CA-J3A-9] incline-right to the Copse [B: 2-5 min]</t>
+        </is>
+      </c>
+      <c r="AL293" s="5" t="inlineStr">
+        <is>
+          <t>[C +7] 'At 1 p.m....until nearly 3 p.m.' cannonade; enemy 'from the woods, 1,000 yards in front'; melee 'nearly an hour'; convergence-target statement (Hall's right/Webb's left)</t>
+        </is>
+      </c>
+      <c r="AM293" s="5" t="inlineStr">
+        <is>
+          <t>722 two-day (148k/574w, report) vs 768 (tablet) - carried; Jul 2 pins Ward/Huston mw; Jul 3 Blinn mw</t>
+        </is>
+      </c>
       <c r="AN293" s="5" t="n"/>
-      <c r="AO293" s="5" t="n"/>
+      <c r="AO293" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
@@ -34537,20 +35293,56 @@
           <t>reg-us-ii-3-3</t>
         </is>
       </c>
-      <c r="AB308" s="5" t="n"/>
+      <c r="AB308" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (one in-window leg)</t>
+        </is>
+      </c>
       <c r="AC308" s="5" t="n"/>
       <c r="AD308" s="5" t="n"/>
       <c r="AE308" s="5" t="n"/>
       <c r="AF308" s="5" t="n"/>
-      <c r="AG308" s="5" t="n"/>
-      <c r="AH308" s="5" t="n"/>
-      <c r="AI308" s="5" t="n"/>
-      <c r="AJ308" s="5" t="n"/>
-      <c r="AK308" s="5" t="n"/>
-      <c r="AL308" s="5" t="n"/>
-      <c r="AM308" s="5" t="n"/>
+      <c r="AG308" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-3-3-willard.md; 4-lines vs Smyth's 3-lines carried</t>
+        </is>
+      </c>
+      <c r="AH308" s="5" t="inlineStr">
+        <is>
+          <t>Willard k Jul 2 -&gt; Sherrill mw Jul 3 ('about 4 p.m.' stated) -&gt; Bull; 39/111/125/126 NY</t>
+        </is>
+      </c>
+      <c r="AI308" s="5" t="inlineStr">
+        <is>
+          <t>1,510 (build compilation, hop flagged)</t>
+        </is>
+      </c>
+      <c r="AJ308" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 massed near Bryan barn; Jul 2 evening Plum Run charge ground; [E Jul 3] slope east of wall, monuments interleave Smyth's row (39NY 4467,4988; 125NY 4468,5053; 111NY 4458,5127; 126NY 4543,5267)</t>
+        </is>
+      </c>
+      <c r="AK308" s="5" t="inlineStr">
+        <is>
+          <t>[C ~15:00 Jul 2] quarter-mile left; [D] Plum Run charge; [A vs CA-J3A-5 tablet 15:00] moved up to Smyth's line [B: 2-4 min]</t>
+        </is>
+      </c>
+      <c r="AL308" s="5" t="inlineStr">
+        <is>
+          <t>[C] 39NY skirmish (28 lost, exact); [C +7] 'About 1 p.m....about two hours' cannonade; [A] 4-line advance repulsed 'after an engagement of about an hour'</t>
+        </is>
+      </c>
+      <c r="AM308" s="5" t="inlineStr">
+        <is>
+          <t>report: attested-unreported ('unable to report'); tablet 714; episode pins: 39NY 28 (Jul 2 skirmish), Willard k, Sherrill mw</t>
+        </is>
+      </c>
       <c r="AN308" s="5" t="n"/>
-      <c r="AO308" s="5" t="n"/>
+      <c r="AO308" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
@@ -34785,20 +35577,56 @@
           <t>reg-us-ii-3-2</t>
         </is>
       </c>
-      <c r="AB310" s="5" t="n"/>
+      <c r="AB310" s="5" t="inlineStr">
+        <is>
+          <t>attested-static (July 2-4 wall line)</t>
+        </is>
+      </c>
       <c r="AC310" s="5" t="n"/>
       <c r="AD310" s="5" t="n"/>
       <c r="AE310" s="5" t="n"/>
       <c r="AF310" s="5" t="n"/>
-      <c r="AG310" s="5" t="n"/>
-      <c r="AH310" s="5" t="n"/>
-      <c r="AI310" s="5" t="n"/>
-      <c r="AJ310" s="5" t="n"/>
-      <c r="AK310" s="5" t="n"/>
-      <c r="AL310" s="5" t="n"/>
-      <c r="AM310" s="5" t="n"/>
+      <c r="AG310" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-3-2-smyth.md</t>
+        </is>
+      </c>
+      <c r="AH310" s="5" t="inlineStr">
+        <is>
+          <t>Col. Smyth w July 3 during cannonade -&gt; Lt. Col. Pierce; 14CT/1DE/12NJ/10NYbn/108NY (or-27-1-smyth)</t>
+        </is>
+      </c>
+      <c r="AI310" s="5" t="inlineStr">
+        <is>
+          <t>1,190 (build compilation, hop flagged; no primary)</t>
+        </is>
+      </c>
+      <c r="AJ310" s="5" t="inlineStr">
+        <is>
+          <t>[C] wall S of Bryan barn from 04:00 Jul 2; monument row 14CT(4449,4951) 1DE(4451,5038) 12NJ(4453,5096) 108NY(4527,5218); Bachelder j3-03 concurs (20-30m)</t>
+        </is>
+      </c>
+      <c r="AK310" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1 march (06:30 order); [C] 04:00 Jul 2 posting; static after</t>
+        </is>
+      </c>
+      <c r="AL310" s="5" t="inlineStr">
+        <is>
+          <t>[C] 1DE skirmish + 108NY supports Woodruff 08:00 Jul 2; Bliss barn burned Jul 3 (14CT); [C -53] 'At 2 p.m.' cannonade (cluster member); [A] 3-line repulse, 12NJ fire at 20 yd, 1,200-1,500 prisoners, 9 flags</t>
+        </is>
+      </c>
+      <c r="AM310" s="5" t="inlineStr">
+        <is>
+          <t>352 (his OR recap) vs 366 (tablet) - both carried; 108NY 'about half' lost; pins Smyth w (cannonade), Lt. Smith k (flag in hand)</t>
+        </is>
+      </c>
       <c r="AN310" s="5" t="n"/>
-      <c r="AO310" s="5" t="n"/>
+      <c r="AO310" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Audit d3: Wilcox/Lang dossiers + index + 11-unit overlay; master table regenerated (46 rows carry audited T-levels)
Wilcox: the CA-J3A-10 executor record (1,200 primary; the 20-30-min
delayed launch envelope; per-day 577/204 closing exactly against the
return). Lang: near-700/455 exact match, the -53 late-stated clock
joins the Longstreet/Smyth cluster, the 2d Florida capture pocket as
the 16th Vermont's receiving side.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -13669,20 +13669,56 @@
           <t>reg-csa-1c-pic-3</t>
         </is>
       </c>
-      <c r="AB125" s="5" t="n"/>
+      <c r="AB125" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (T5 window)</t>
+        </is>
+      </c>
       <c r="AC125" s="5" t="n"/>
       <c r="AD125" s="5" t="n"/>
       <c r="AE125" s="5" t="n"/>
       <c r="AF125" s="5" t="n"/>
-      <c r="AG125" s="5" t="n"/>
-      <c r="AH125" s="5" t="n"/>
-      <c r="AI125" s="5" t="n"/>
-      <c r="AJ125" s="5" t="n"/>
-      <c r="AK125" s="5" t="n"/>
-      <c r="AL125" s="5" t="n"/>
-      <c r="AM125" s="5" t="n"/>
+      <c r="AG125" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-pic-3-armistead.md; NO brigade OR report (verified negative)</t>
+        </is>
+      </c>
+      <c r="AH125" s="5" t="inlineStr">
+        <is>
+          <t>Armistead mw&amp;c under captured guns (T5 t~8720; mon-armistead 16m agreement) -&gt; Col. Aylett (w); Hodges k, Edmonds k at wall</t>
+        </is>
+      </c>
+      <c r="AI125" s="5" t="inlineStr">
+        <is>
+          <t>1,650 (ED-9, no primary); crossing party ~150 (T5)</t>
+        </is>
+      </c>
+      <c r="AJ125" s="5" t="inlineStr">
+        <is>
+          <t>[E +-120m] j3-02 morning label ~(3150,4780) behind Spangler's Woods (2nd line west of crest); fall point (4412,4865)+-25 (T5)</t>
+        </is>
+      </c>
+      <c r="AK125" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J3A-6] second-line step-off; closed onto first line BEFORE wall (peyton 75-paces relation); ED-8 recross 8700-9000</t>
+        </is>
+      </c>
+      <c r="AL125" s="5" t="inlineStr">
+        <is>
+          <t>[A window] bombardment share UNQUANTIFIED (open); activity concentrates at wall - crossing, Cushing's guns, ~10-min penetration (T5)</t>
+        </is>
+      </c>
+      <c r="AM125" s="5" t="inlineStr">
+        <is>
+          <t>1,191 = 88/460/643 (anv-return = aylett-1863 EXACT match; regt k+w 71/108/170/104/121); 643 missing at/east of wall; headnote missing-scope at full force</t>
+        </is>
+      </c>
       <c r="AN125" s="5" t="n"/>
-      <c r="AO125" s="5" t="n"/>
+      <c r="AO125" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc (T5 in Angle window)</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -13793,20 +13829,56 @@
           <t>reg-csa-3c-het-2</t>
         </is>
       </c>
-      <c r="AB126" s="5" t="n"/>
+      <c r="AB126" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (wings flagged reconstruction)</t>
+        </is>
+      </c>
       <c r="AC126" s="5" t="n"/>
       <c r="AD126" s="5" t="n"/>
       <c r="AE126" s="5" t="n"/>
       <c r="AF126" s="5" t="n"/>
-      <c r="AG126" s="5" t="n"/>
-      <c r="AH126" s="5" t="n"/>
-      <c r="AI126" s="5" t="n"/>
-      <c r="AJ126" s="5" t="n"/>
-      <c r="AK126" s="5" t="n"/>
-      <c r="AL126" s="5" t="n"/>
-      <c r="AM126" s="5" t="n"/>
+      <c r="AG126" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-het-2-brockenbrough.md; NO OR report (verified negative)</t>
+        </is>
+      </c>
+      <c r="AH126" s="5" t="inlineStr">
+        <is>
+          <t>Col. Brockenbrough (unwounded; replaced after battle); NO officer pins located (open); two-wing split (Mayo) has NO primary in corpus - build-inherited, flagged</t>
+        </is>
+      </c>
+      <c r="AI126" s="5" t="inlineStr">
+        <is>
+          <t>CORRUPTED record bounded: stone-sentinels page = Davis duplicate (DO-NOT-USE stands); range 800-1,100, Mayo-hop ~880 = build basis (ED-48 candidate)</t>
+        </is>
+      </c>
+      <c r="AJ126" s="5" t="inlineStr">
+        <is>
+          <t>[D] division LEFT (davis-jr order); j3-02 label ~(3320,5980)+-120 (northernmost of column); advance axis toward Bliss/Bryan north front (+-150m)</t>
+        </is>
+      </c>
+      <c r="AK126" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J3A-5/6] step-off w/ division; THE EARLY BREAK - documented from outside (Jones 'whole line on the left had given way'; Engelhard/Lane enfilade column)</t>
+        </is>
+      </c>
+      <c r="AL126" s="5" t="inlineStr">
+        <is>
+          <t>[A window] bombardment w/ division (no figure, open); received 8th Ohio flank + Osborn arc; no brigade-authored fire statement (negative)</t>
+        </is>
+      </c>
+      <c r="AM126" s="5" t="inlineStr">
+        <is>
+          <t>PRIMARY FLOOR (new): 148 = 25/123/no-missing (anv-return regt-grain 42/48/34/24); build's 100 decay is BELOW the documented k+w floor (ED-48 consequence); no episode split exists (open)</t>
+        </is>
+      </c>
       <c r="AN126" s="5" t="n"/>
-      <c r="AO126" s="5" t="n"/>
+      <c r="AO126" s="5" t="inlineStr">
+        <is>
+          <t>T3 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -13917,20 +13989,56 @@
           <t>reg-csa-3c-het-4</t>
         </is>
       </c>
-      <c r="AB127" s="5" t="n"/>
+      <c r="AB127" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC127" s="5" t="n"/>
       <c r="AD127" s="5" t="n"/>
       <c r="AE127" s="5" t="n"/>
       <c r="AF127" s="5" t="n"/>
-      <c r="AG127" s="5" t="n"/>
-      <c r="AH127" s="5" t="n"/>
-      <c r="AI127" s="5" t="n"/>
-      <c r="AJ127" s="5" t="n"/>
-      <c r="AK127" s="5" t="n"/>
-      <c r="AL127" s="5" t="n"/>
-      <c r="AM127" s="5" t="n"/>
+      <c r="AG127" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-het-4-davis.md; division report clock +5 (CSA twin of Hall)</t>
+        </is>
+      </c>
+      <c r="AH127" s="5" t="inlineStr">
+        <is>
+          <t>Davis (unwounded, wrote brigade + division reports); Jul 1: 7 of 9 field officers hit; Jul 3: ALL field officers k/w</t>
+        </is>
+      </c>
+      <c r="AI127" s="5" t="inlineStr">
+        <is>
+          <t>2,000 'present first day' (stone-sentinels, scope caveat); 11th Miss DETACHED Jul 1 (division train guard, primary) - fresh regiment atop Jul 1 survivors on Jul 3</t>
+        </is>
+      </c>
+      <c r="AJ127" s="5" t="inlineStr">
+        <is>
+          <t>[C +5] 9am shift behind Pegram's bn; j3-02 label ~(3330,5760)+-100; mon-11ms start (3471,5621) corroborates (modern-era caution); farthest advance mon-11ms-1 Bryan barn (4448,5115)</t>
+        </is>
+      </c>
+      <c r="AK127" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J3A-5/6] cease-fire trigger, dressed right, oblique left; fences deranging/rectified; fall-back to morning line ~16:00 [C +5]</t>
+        </is>
+      </c>
+      <c r="AL127" s="5" t="inlineStr">
+        <is>
+          <t>[A window] 2-hr bombardment 'no time to prepare means for protection'; no fire until 3/4-mi fence then grape/canister/shell; musket-range 'suffered severely'</t>
+        </is>
+      </c>
+      <c r="AM127" s="5" t="inlineStr">
+        <is>
+          <t>897 = 180/717/NO-missing (anv-return: 232/202/265/198); BOMBARDMENT PRIMARY 2k/21w (best in batch, pairs w/ Garnett's ~20); 11th Miss 202 k+w = Jul 3 only (day-split anchor)</t>
+        </is>
+      </c>
       <c r="AN127" s="5" t="n"/>
-      <c r="AO127" s="5" t="n"/>
+      <c r="AO127" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -14041,20 +14149,56 @@
           <t>reg-csa-3c-het-3</t>
         </is>
       </c>
-      <c r="AB128" s="5" t="n"/>
+      <c r="AB128" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC128" s="5" t="n"/>
       <c r="AD128" s="5" t="n"/>
       <c r="AE128" s="5" t="n"/>
       <c r="AF128" s="5" t="n"/>
-      <c r="AG128" s="5" t="n"/>
-      <c r="AH128" s="5" t="n"/>
-      <c r="AI128" s="5" t="n"/>
-      <c r="AJ128" s="5" t="n"/>
-      <c r="AK128" s="5" t="n"/>
-      <c r="AL128" s="5" t="n"/>
-      <c r="AM128" s="5" t="n"/>
+      <c r="AG128" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-het-3-fry.md; claim-fry-guide now executor-documented</t>
+        </is>
+      </c>
+      <c r="AH128" s="5" t="inlineStr">
+        <is>
+          <t>Archer c Jul 1 -&gt; Fry (w&amp;c Jul 3 at works) -&gt; Shepard; 7 field officers in, 2 out; order 1TN-13AL-14TN-7TN-5ALbn</t>
+        </is>
+      </c>
+      <c r="AI128" s="5" t="inlineStr">
+        <is>
+          <t>PRIMARY 1,048 (shepard, =build); Jul 3 basis = 1,048 - Jul 1 losses (open); NOT engaged Jul 2 (attested negative)</t>
+        </is>
+      </c>
+      <c r="AJ128" s="5" t="inlineStr">
+        <is>
+          <t>[D] division right in front of works from night Jul 2; j3-02 label ~(3400,5100)+-100; lane w/ two stout fences at 180-200 yd from works</t>
+        </is>
+      </c>
+      <c r="AK128" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J3A-5/6] step-off at cease-fire trigger; the CONVERGENCE executed ('Guide right', touched Pickett's left at half-way); lane crossing; fell back to start</t>
+        </is>
+      </c>
+      <c r="AL128" s="5" t="inlineStr">
+        <is>
+          <t>[D] enemy held fire until 'fine range'; at works 'as long as any other troops'; color record: 4 of 5 flags captured AT/WITHIN works (13 color-bearers down) - ED-5 substance</t>
+        </is>
+      </c>
+      <c r="AM128" s="5" t="inlineStr">
+        <is>
+          <t>677 = 16/144/517 (anv-return; =shepard's own 677 of 1,048 EXACT); 76% capture share (Jul 1 creek pocket ~75 + Jul 3 works); ED-49 exemplar</t>
+        </is>
+      </c>
       <c r="AN128" s="5" t="n"/>
-      <c r="AO128" s="5" t="n"/>
+      <c r="AO128" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -14167,7 +14311,7 @@
       </c>
       <c r="AB129" s="5" t="inlineStr">
         <is>
-          <t>authored-ok</t>
+          <t>authored-ok (T5 window)</t>
         </is>
       </c>
       <c r="AC129" s="5" t="inlineStr">
@@ -14192,17 +14336,45 @@
       </c>
       <c r="AG129" s="5" t="inlineStr">
         <is>
-          <t>Format example row - overwrite freely.</t>
-        </is>
-      </c>
-      <c r="AH129" s="5" t="n"/>
-      <c r="AI129" s="5" t="n"/>
-      <c r="AJ129" s="5" t="n"/>
-      <c r="AK129" s="5" t="n"/>
-      <c r="AL129" s="5" t="n"/>
-      <c r="AM129" s="5" t="n"/>
+          <t>Dossier: reconstruction/dossiers/csa-1c-pic-1-garnett.md; Peyton page-verified this pass</t>
+        </is>
+      </c>
+      <c r="AH129" s="5" t="inlineStr">
+        <is>
+          <t>Garnett k ~25 paces from wall (peyton) -&gt; Maj. Peyton; pins: Ellis (19VA) k in bombardment, every rgt cdr k/w</t>
+        </is>
+      </c>
+      <c r="AI129" s="5" t="inlineStr">
+        <is>
+          <t>PRIMARY 1,287 men + ~140 officers (peyton, previous-evening report; ED-46 candidate) vs 1,480 ED-9 build basis - conflict carried</t>
+        </is>
+      </c>
+      <c r="AJ129" s="5" t="inlineStr">
+        <is>
+          <t>[C ~09:00] reached field; [C/E ~12:00] behind Alexander's gun crest; build start (3200,4930)+-60 (j3-03 bars); 800-1,000 yd to the line (peyton)</t>
+        </is>
+      </c>
+      <c r="AK129" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J3A-6] Pickett-in-person order, quick time; three-fence climb w/ skirmishers at last fence; recoil at 20 paces then three-line rush; dissolution-class retreat (~300 came off)</t>
+        </is>
+      </c>
+      <c r="AL129" s="5" t="inlineStr">
+        <is>
+          <t>[A window] under cannonade overs 'one hour' (duration conflict carried); LRT enfilade received (10 men/shell, peyton); loading-and-firing advance; hand-to-hand at works</t>
+        </is>
+      </c>
+      <c r="AM129" s="5" t="inlineStr">
+        <is>
+          <t>941 = 78/324/539 (anv-return regt-grain: 54/87/44/77/62 + staff; ED-49 scope); bombardment ~20 k&amp;w PRIMARY; &gt;half fallen by wall fight; missing mostly k/w (report+headnote)</t>
+        </is>
+      </c>
       <c r="AN129" s="5" t="n"/>
-      <c r="AO129" s="5" t="n"/>
+      <c r="AO129" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc (T5 in Angle window)</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -14313,20 +14485,56 @@
           <t>reg-csa-1c-pic-2</t>
         </is>
       </c>
-      <c r="AB130" s="5" t="n"/>
+      <c r="AB130" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (T5 window)</t>
+        </is>
+      </c>
       <c r="AC130" s="5" t="n"/>
       <c r="AD130" s="5" t="n"/>
       <c r="AE130" s="5" t="n"/>
       <c r="AF130" s="5" t="n"/>
-      <c r="AG130" s="5" t="n"/>
-      <c r="AH130" s="5" t="n"/>
-      <c r="AI130" s="5" t="n"/>
-      <c r="AJ130" s="5" t="n"/>
-      <c r="AK130" s="5" t="n"/>
-      <c r="AL130" s="5" t="n"/>
-      <c r="AM130" s="5" t="n"/>
+      <c r="AG130" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-pic-2-kemper.md; NO brigade OR report (verified negative)</t>
+        </is>
+      </c>
+      <c r="AH130" s="5" t="inlineStr">
+        <is>
+          <t>Kemper w&amp;c (rescued; T5 t~8640, Peyton brackets earlier) -&gt; Col. Mayo; Williams/Patton mw, Otey w; staff 1k/3w (return)</t>
+        </is>
+      </c>
+      <c r="AI130" s="5" t="inlineStr">
+        <is>
+          <t>1,575 (ED-9/stone-sentinels, no primary; negative - no morning report survives)</t>
+        </is>
+      </c>
+      <c r="AJ130" s="5" t="inlineStr">
+        <is>
+          <t>[E] right of Garnett behind gun line; oblique/lapping convergence (peyton); wounding point (4370,4790)+-50 (T5)</t>
+        </is>
+      </c>
+      <c r="AK130" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J3A-6] step-off w/ division; convergence leg 50-60 yd behind-right of Garnett; flank crisis vs Stannard wheel (CA-J3A-8)</t>
+        </is>
+      </c>
+      <c r="AL130" s="5" t="inlineStr">
+        <is>
+          <t>[A window] bombardment: 'suffered severely' (Wilcox cross-brigade comparison - worse than Garnett's ~20); LRT enfilade on right; Rorty canister + Stannard front/flank fire received</t>
+        </is>
+      </c>
+      <c r="AM130" s="5" t="inlineStr">
+        <is>
+          <t>731 = 58/356/317 (anv-return regt-grain: 64/67/94/109/128; 58k vs stone-sentinels 56k conflict carried); 317 missing concentrate at flank collapse (Stannard's 243 prisoners = Union pin)</t>
+        </is>
+      </c>
       <c r="AN130" s="5" t="n"/>
-      <c r="AO130" s="5" t="n"/>
+      <c r="AO130" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc (T5 in Angle window)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -14437,20 +14645,56 @@
           <t>reg-csa-3c-het-1</t>
         </is>
       </c>
-      <c r="AB131" s="5" t="n"/>
+      <c r="AB131" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC131" s="5" t="n"/>
       <c r="AD131" s="5" t="n"/>
       <c r="AE131" s="5" t="n"/>
       <c r="AF131" s="5" t="n"/>
-      <c r="AG131" s="5" t="n"/>
-      <c r="AH131" s="5" t="n"/>
-      <c r="AI131" s="5" t="n"/>
-      <c r="AJ131" s="5" t="n"/>
-      <c r="AK131" s="5" t="n"/>
-      <c r="AL131" s="5" t="n"/>
-      <c r="AM131" s="5" t="n"/>
+      <c r="AG131" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-het-1-marshall.md</t>
+        </is>
+      </c>
+      <c r="AH131" s="5" t="inlineStr">
+        <is>
+          <t>Pettigrew (to division) -&gt; Marshall k Jul 3 (CONFLICT: Davis rpt 'w&amp;c' vs Young 'supposed killed' vs register k - k adopted) -&gt; Maj. Jones; Jul 1: Burgwyn k, Lane w; 1 field officer left after Jul 3</t>
+        </is>
+      </c>
+      <c r="AI131" s="5" t="inlineStr">
+        <is>
+          <t>2,000 'present on the first day' (stone-sentinels, Jul-1 scope caveat); 26NC regt primary: 800+ -&gt; 216 unhurt (Jul 1) -&gt; ~80 (Jul 4) (young-26nc); Jul 3 basis ~900 [B subtraction, open for primary]</t>
+        </is>
+      </c>
+      <c r="AJ131" s="5" t="inlineStr">
+        <is>
+          <t>[D] Jul 2 eve: 1 mi right, rear of batteries; [C +5] 9am quarter-mile shift behind Pegram; j3-02 label ~(3550,5360)+-100; farthest advance mon-26nc-1 (4431.7,4923.9) at the wall</t>
+        </is>
+      </c>
+      <c r="AK131" s="5" t="inlineStr">
+        <is>
+          <t>[C +65 via jones] 'About 2 o'clock' step-off w/ launch confusion (close-right vs give-way-left, corrected); ~3/4 mi advance; deadly volley from left at wall; retreat to morning line by ~16:00</t>
+        </is>
+      </c>
+      <c r="AL131" s="5" t="inlineStr">
+        <is>
+          <t>[A window] two-hour bombardment (division); canister from half-way, musketry hail at 250-300 yd (range ladder cross vs Woodruff/Arnold/Smyth)</t>
+        </is>
+      </c>
+      <c r="AM131" s="5" t="inlineStr">
+        <is>
+          <t>1,105 = 190/915/NO-missing-column (anv-return; 26NC 588 = 86k/502w); ED-49 cleanest exemplar (Jul 3 capture mass absent); 26NC day split ~584 Jul 1 / ~136 Jul 3 [B]; 11 color-bearers down Jul 1, colors lost Jul 3</t>
+        </is>
+      </c>
       <c r="AN131" s="5" t="n"/>
-      <c r="AO131" s="5" t="n"/>
+      <c r="AO131" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -15925,20 +16169,56 @@
           <t>reg-csa-3c-pen-2</t>
         </is>
       </c>
-      <c r="AB143" s="5" t="n"/>
+      <c r="AB143" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC143" s="5" t="n"/>
       <c r="AD143" s="5" t="n"/>
       <c r="AE143" s="5" t="n"/>
       <c r="AF143" s="5" t="n"/>
-      <c r="AG143" s="5" t="n"/>
-      <c r="AH143" s="5" t="n"/>
-      <c r="AI143" s="5" t="n"/>
-      <c r="AJ143" s="5" t="n"/>
-      <c r="AK143" s="5" t="n"/>
-      <c r="AL143" s="5" t="n"/>
-      <c r="AM143" s="5" t="n"/>
+      <c r="AG143" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-pen-2-lane.md</t>
+        </is>
+      </c>
+      <c r="AH143" s="5" t="inlineStr">
+        <is>
+          <t>Lane (cdr; division command Jul 2 eve + after Trimble fell) -&gt; Col. Avery in intervals; Avery/Barry brought left rgts out under orders</t>
+        </is>
+      </c>
+      <c r="AI143" s="5" t="inlineStr">
+        <is>
+          <t>PRIMARY 1,355 effective incl. ambulance/rear guard (lane-jh, =build); Jul 1-2 loss 'but slight' - serviceable Jul 3 basis</t>
+        </is>
+      </c>
+      <c r="AJ143" s="5" t="inlineStr">
+        <is>
+          <t>[D] Jul 2 by Garnett's bn (frame); Jul 3 rear of Heth's right, Lowrance on right, behind Poague/Pegram line; j3-02 pre-move label ~(3050,5750)+-120; 'no second line in rear of [Heth's] left' (structural primary)</t>
+        </is>
+      </c>
+      <c r="AK143" s="5" t="inlineStr">
+        <is>
+          <t>[D] morning lateral ~1.2km [B 15-20 min]; advance ~1 mi, left checked by Trimble; passed through collapsing front WITHOUT halting; withdrew when enfiladed from left; reformed in rear of artillery</t>
+        </is>
+      </c>
+      <c r="AL143" s="5" t="inlineStr">
+        <is>
+          <t>[A window] two-hour bombardment exposure (no figure); fire reserved to 'good range' then silenced guns on front (reads vs Woodruff/Arnold wreckage - corroborated); raking artillery from right</t>
+        </is>
+      </c>
+      <c r="AM143" s="5" t="inlineStr">
+        <is>
+          <t>ED-47 candidate: Lane's 660 of 1,355 (total) vs return 389 (k+w only; return's own footnote carries the 660); regt k+w 89/45/104/63/88; mass falls Jul 3 (crest fire window + flank collapse)</t>
+        </is>
+      </c>
       <c r="AN143" s="5" t="n"/>
-      <c r="AO143" s="5" t="n"/>
+      <c r="AO143" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -16049,20 +16329,56 @@
           <t>reg-csa-3c-and-4</t>
         </is>
       </c>
-      <c r="AB144" s="5" t="n"/>
+      <c r="AB144" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC144" s="5" t="n"/>
       <c r="AD144" s="5" t="n"/>
       <c r="AE144" s="5" t="n"/>
       <c r="AF144" s="5" t="n"/>
-      <c r="AG144" s="5" t="n"/>
-      <c r="AH144" s="5" t="n"/>
-      <c r="AI144" s="5" t="n"/>
-      <c r="AJ144" s="5" t="n"/>
-      <c r="AK144" s="5" t="n"/>
-      <c r="AL144" s="5" t="n"/>
-      <c r="AM144" s="5" t="n"/>
+      <c r="AG144" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-and-4-lang.md</t>
+        </is>
+      </c>
+      <c r="AH144" s="5" t="inlineStr">
+        <is>
+          <t>Col. Lang (Perry absent typhoid); pins: McCaslan (AAAG) k in Jul 3 retreat; Moore (2FL) w&amp;c, Gardner (5FL) w; 8FL colors lost Jul 2</t>
+        </is>
+      </c>
+      <c r="AI144" s="5" t="inlineStr">
+        <is>
+          <t>PRIMARY 'near 700 strong' (lang, =build) - smallest brigade in the assault's orbit</t>
+        </is>
+      </c>
+      <c r="AJ144" s="5" t="inlineStr">
+        <is>
+          <t>[C/D ~07:00] up with Wilcox's left to foot of gun hill, skirmishers one crest fwd; j3-01 label ~(3230,4820)+-120; reform on old line, night withdrawal to woods</t>
+        </is>
+      </c>
+      <c r="AK144" s="5" t="inlineStr">
+        <is>
+          <t>[D] standing conform-to-Wilcox order ('I would receive no further orders'); advanced after Pickett's troops retired; left flanked in the woods, retreat order inaudible in the din; 2FL colors + pocket captured (16th VT object, veazey cross)</t>
+        </is>
+      </c>
+      <c r="AL144" s="5" t="inlineStr">
+        <is>
+          <t>[C -53] bombardment 'nearly 2 p.m. ... till nearly 4 p.m.' (late-stated pole, joins Longstreet/Smyth cluster); no formed fire window Jul 3 (movement and reception only)</t>
+        </is>
+      </c>
+      <c r="AM144" s="5" t="inlineStr">
+        <is>
+          <t>455 = 33/217/205 (return = lang's own 455 of ~700 EXACT; regt k+w 81/75/94) - 65% loss rate, highest documented in batch; day split [B]: Jul 2 ~300 (his figure) -&gt; Jul 3 ~155 concentrated in the capture pocket + retreat</t>
+        </is>
+      </c>
       <c r="AN144" s="5" t="n"/>
-      <c r="AO144" s="5" t="n"/>
+      <c r="AO144" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -16297,20 +16613,56 @@
           <t>reg-csa-3c-pen-4</t>
         </is>
       </c>
-      <c r="AB146" s="5" t="n"/>
+      <c r="AB146" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC146" s="5" t="n"/>
       <c r="AD146" s="5" t="n"/>
       <c r="AE146" s="5" t="n"/>
       <c r="AF146" s="5" t="n"/>
-      <c r="AG146" s="5" t="n"/>
-      <c r="AH146" s="5" t="n"/>
-      <c r="AI146" s="5" t="n"/>
-      <c r="AJ146" s="5" t="n"/>
-      <c r="AK146" s="5" t="n"/>
-      <c r="AL146" s="5" t="n"/>
-      <c r="AM146" s="5" t="n"/>
+      <c r="AG146" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-pen-4-lowrance.md</t>
+        </is>
+      </c>
+      <c r="AH146" s="5" t="inlineStr">
+        <is>
+          <t>Scales w Jul 1 -&gt; Lowrance (w Jul 1, again Jul 3 per register - report silent, flag); Jul 1: every field officer save one disabled</t>
+        </is>
+      </c>
+      <c r="AI146" s="5" t="inlineStr">
+        <is>
+          <t>PRIMARY ~500 from Jul 1 evening ('depressed, dilapidated, almost unorganized') = Jul 3 basis; build 1,250 = pre-Jul-1 (decay must cross the 500 waypoint)</t>
+        </is>
+      </c>
+      <c r="AJ146" s="5" t="inlineStr">
+        <is>
+          <t>[D] Jul 2: extreme right on line w/ artillery (its only guard); Jul 3: second line in rear of POAGUE's bn (primary frame anchor); right of Lane; works touched on right at climax</t>
+        </is>
+      </c>
+      <c r="AK146" s="5" t="inlineStr">
+        <is>
+          <t>[D] morning lateral right; advance 1 mi over 'wide, hot, already crimson plain'; at 2/3 way front-line troops 'came tearing through our ranks'; retreat without orders, rallied on start line</t>
+        </is>
+      </c>
+      <c r="AL146" s="5" t="inlineStr">
+        <is>
+          <t>[A window + B] '&gt;= one hour under a most galling fire' (his duration) / 'two hours' (Engelhard) - both carried; climax: '800 guns' combined two-brigade strength pin at the works</t>
+        </is>
+      </c>
+      <c r="AM146" s="5" t="inlineStr">
+        <is>
+          <t>535 = 102/323/110 (anv-return regt k+w 126/66/89/64/79) vs SCALES'S OWN Jul-1 table 545 (48/381/116) - July-1-scoped table LARGER than 3-day return (ED-49 starkest exemplar); build decay 599 flagged for reconciliation</t>
+        </is>
+      </c>
       <c r="AN146" s="5" t="n"/>
-      <c r="AO146" s="5" t="n"/>
+      <c r="AO146" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -17909,20 +18261,56 @@
           <t>reg-csa-3c-and-1</t>
         </is>
       </c>
-      <c r="AB159" s="5" t="n"/>
+      <c r="AB159" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC159" s="5" t="n"/>
       <c r="AD159" s="5" t="n"/>
       <c r="AE159" s="5" t="n"/>
       <c r="AF159" s="5" t="n"/>
-      <c r="AG159" s="5" t="n"/>
-      <c r="AH159" s="5" t="n"/>
-      <c r="AI159" s="5" t="n"/>
-      <c r="AJ159" s="5" t="n"/>
-      <c r="AK159" s="5" t="n"/>
-      <c r="AL159" s="5" t="n"/>
-      <c r="AM159" s="5" t="n"/>
+      <c r="AG159" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-and-1-wilcox.md; CA-J3A-10 executor</t>
+        </is>
+      </c>
+      <c r="AH159" s="5" t="inlineStr">
+        <is>
+          <t>Wilcox (unwounded); 4 of 5 rgt cdrs w JUL 2 (Forney, Pinckard, Sanders, Fletcher); no rgt-cdr losses Jul 3</t>
+        </is>
+      </c>
+      <c r="AI159" s="5" t="inlineStr">
+        <is>
+          <t>PRIMARY Jul 3: 'about 1,200' (wilcox) - closes exactly vs build 1,777 start - 577 Jul 2 loss; order R-L 9-10-11-8-14 Ala</t>
+        </is>
+      </c>
+      <c r="AJ159" s="5" t="inlineStr">
+        <is>
+          <t>[D] before sunrise: line parallel to Emmitsburg pike ~200 yd W, Alexander's guns in front; j3-01 label ~(3100,4400)+-120 (04:00-08:00 window = exact bracket); farthest advance = ravine below McGilvery crest (build displacement understates - flag)</t>
+        </is>
+      </c>
+      <c r="AK159" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J3A-6 +20-30 min] the DELAYED LAUNCH (three staff officers in succession; Alexander concurs; Lang sequences after repulse - one envelope); halt at ravine awaiting artillery that had no ammunition; withdrew on own judgment</t>
+        </is>
+      </c>
+      <c r="AL159" s="5" t="inlineStr">
+        <is>
+          <t>[A window] bombardment: '&lt;a dozen k&amp;w' + Kemper-severity contrast + Anderson's 'suffered most seriously' of his division (compatible); advance under three-sided artillery, no musketry phase; 'Not a man of the division ... could I see'</t>
+        </is>
+      </c>
+      <c r="AM159" s="5" t="inlineStr">
+        <is>
+          <t>PER-DAY PRIMARY: Jul 2 577 / Jul 3 204 / total 777 = return 51/469/257 EXACT; 257 missing 'nearly all killed or wounded, few unwounded prisoners'; Jul 3 cause mix artillery-dominated (distinct from every front-line brigade)</t>
+        </is>
+      </c>
       <c r="AN159" s="5" t="n"/>
-      <c r="AO159" s="5" t="n"/>
+      <c r="AO159" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Audit d4: CSA completion (Poague T4, ED-36 frame closed; 2c artillery command record) + 5 dossier upgrades + index + 6-unit overlay; master table regenerated (52 rows carry audited T-levels)
Poague: report No. 562 transcribed in full (attested July 1-2 non-
participation; two-position geometry sheet-corroborated; the six-
howitzer never-fired negative; tablet 657-round expenditure; return 32
= tablet 32, ED-43 satisfied). Second Corps artillery command record
consolidates the pass-2 wing dossier (return's 'Brown's Battalion'
alias recorded; register gap re-flagged). Upgrades: Trimble SHSP 26
closed (road-fence wounding conflict vs Engelhard's near-the-works;
reach-envelope conflict vs Lane), Rittenhouse gains the Norton same-
hill witness, Kemper/Armistead morning-report sweep closed verified-
negative with B&M-type readings carried, Lowrance's Poague note closed.

Suites: reconstruction 117+1s, pipeline 59, tool 108.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -9329,20 +9329,56 @@
           <t>reg-csa-3c-bn-poague</t>
         </is>
       </c>
-      <c r="AB87" s="5" t="n"/>
+      <c r="AB87" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC87" s="5" t="n"/>
       <c r="AD87" s="5" t="n"/>
       <c r="AE87" s="5" t="n"/>
       <c r="AF87" s="5" t="n"/>
-      <c r="AG87" s="5" t="n"/>
-      <c r="AH87" s="5" t="n"/>
-      <c r="AI87" s="5" t="n"/>
-      <c r="AJ87" s="5" t="n"/>
-      <c r="AK87" s="5" t="n"/>
-      <c r="AL87" s="5" t="n"/>
-      <c r="AM87" s="5" t="n"/>
+      <c r="AG87" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-bn-poague.md; ED-36 Third Corps frame COMPLETE (Lowrance's anchor closed); memoir (Gunner with Stonewall) print-only acquisition item</t>
+        </is>
+      </c>
+      <c r="AH87" s="5" t="inlineStr">
+        <is>
+          <t>Maj. W.T. Poague; Wyatt (Albemarle Va), Graham (Charlotte NC), Ward (Madison Miss), Brooke (Va); 16 guns: 7 Nap + 6 how + 1 Parrott + 2 3-in (tablet); Jul 3 split command Wyatt/Ward; Ward-mw tradition NOT in corpus (open pin)</t>
+        </is>
+      </c>
+      <c r="AI87" s="5" t="inlineStr">
+        <is>
+          <t>build 384 (B&amp;M-type hop, ED-38 class); no personnel primary</t>
+        </is>
+      </c>
+      <c r="AJ87" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 1-2 OFF THE LINE (Cashtown detach, attested non-participation); [C] Jul 2 late evening two-position line: 5 guns left of Anderson's division near Pegram + 5 Napoleons 400 yd right, ~1,400 yd from the Union batteries; j3-03 WYATT (3427,5220), GRAHAM (3489,5325), POAGUE'S BATT. bar (3467,4894) +-120m</t>
+        </is>
+      </c>
+      <c r="AK87" s="5" t="inlineStr">
+        <is>
+          <t>[C/D] Jul 2 night effortful emplacement ('at last succeeded'); [D] post-repulse howitzers ordered up (no fire); [C] Jul 4 dusk withdrawal to Hagerstown</t>
+        </is>
+      </c>
+      <c r="AL87" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 3 ~07:00 unordered affair (Hill's order; Poague ceased it; 8 Wyatt horses; enemy caisson exploded) - do NOT smooth into the cannonade; [A window] participated in the 13:07 general engagement; HOWITZER NEGATIVE: 6 tubes present-never-firing all battle (ED-44); tablet expenditure 657 rounds / 17 horses (ED-42 battery-side) [B: ~60-90 min deliberate fire for 10 guns]</t>
+        </is>
+      </c>
+      <c r="AM87" s="5" t="inlineStr">
+        <is>
+          <t>return 2/24/6 = 32, batteries '*Not reported in detail' (ED-49 gap); tablet prints the same 32 - ED-43 corroboration SATISFIED; episode split: morning affair + cannonade window, Jul 1-2 zero</t>
+        </is>
+      </c>
       <c r="AN87" s="5" t="n"/>
-      <c r="AO87" s="5" t="n"/>
+      <c r="AO87" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -30565,20 +30601,56 @@
           <t>reg-us-ii-2-2</t>
         </is>
       </c>
-      <c r="AB267" s="5" t="n"/>
+      <c r="AB267" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC267" s="5" t="n"/>
       <c r="AD267" s="5" t="n"/>
       <c r="AE267" s="5" t="n"/>
       <c r="AF267" s="5" t="n"/>
-      <c r="AG267" s="5" t="n"/>
-      <c r="AH267" s="5" t="n"/>
-      <c r="AI267" s="5" t="n"/>
-      <c r="AJ267" s="5" t="n"/>
-      <c r="AK267" s="5" t="n"/>
-      <c r="AL267" s="5" t="n"/>
-      <c r="AM267" s="5" t="n"/>
+      <c r="AG267" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-2-2-webb.md; CA-J3A-9: Armistead 'passed over the fence with probably over 100' - report twin of the ~150 party claim</t>
+        </is>
+      </c>
+      <c r="AH267" s="5" t="inlineStr">
+        <is>
+          <t>Webb w Jul 3 (MoH); O'Kane (69th) k Jul 3, Baxter (72nd) w Jul 2; 106th PA detached to Howard Jul 2 'a little before dark' - brigade fights Jul 3 three-regiment (or-27-1-webb)</t>
+        </is>
+      </c>
+      <c r="AI267" s="5" t="inlineStr">
+        <is>
+          <t>ED-9 1,250 held; NO primary; Jul 3 subtraction of the 106th is primary (or-27-1-webb); division context 3,800 engaged (or-27-1-gibbon)</t>
+        </is>
+      </c>
+      <c r="AJ267" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 06:30 Granite Ridge, 69th at fence in advance; [E/T5] wall/clump geometry held via V2 claims; j3-02 WEBB bar (4391,4827) +-100m</t>
+        </is>
+      </c>
+      <c r="AK267" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 ~18:30 counterattack vs Wright (beyond one Brown gun, ~250 prisoners); [E] Jul 3 morning 71st to the wall, 72nd reserve under crest; [T5] the crisis window held</t>
+        </is>
+      </c>
+      <c r="AL267" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J3A-1/4] 'About 1 p.m. more than twenty batteries'; 'By 2.45 silenced the Rhode Island battery' (ED-33 timed by the brigade CO); 3 Cushing guns to the fence (vs V2's 2 - conflict on claim); captures ~1,000 prisoners/6 flags/1,400 arms</t>
+        </is>
+      </c>
+      <c r="AM267" s="5" t="inlineStr">
+        <is>
+          <t>CONFLICT: report 525 (43 off + 482 men) vs return 491 (69th 137, 71st 98, 72nd 192, 106th 64); build decay 490 = return; pins Webb w, O'Kane k, Baxter w Jul 2</t>
+        </is>
+      </c>
       <c r="AN267" s="5" t="n"/>
-      <c r="AO267" s="5" t="n"/>
+      <c r="AO267" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc (T5 window held)</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
@@ -30685,20 +30757,56 @@
         </is>
       </c>
       <c r="AA268" s="2" t="inlineStr"/>
-      <c r="AB268" s="5" t="n"/>
+      <c r="AB268" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC268" s="5" t="n"/>
       <c r="AD268" s="5" t="n"/>
       <c r="AE268" s="5" t="n"/>
       <c r="AF268" s="5" t="n"/>
-      <c r="AG268" s="5" t="n"/>
-      <c r="AH268" s="5" t="n"/>
-      <c r="AI268" s="5" t="n"/>
-      <c r="AJ268" s="5" t="n"/>
-      <c r="AK268" s="5" t="n"/>
-      <c r="AL268" s="5" t="n"/>
-      <c r="AM268" s="5" t="n"/>
+      <c r="AG268" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-3-1-carroll.md (first-class element); clockProfile or-27-1-sawyer -55 [-70,-40] weak (late-stated cluster)</t>
+        </is>
+      </c>
+      <c r="AH268" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Col. Franklin Sawyer; detached from Carroll on the advanced picket line from Jul 2 evening, 24+ hours (or-27-1-sawyer; or-27-1-carroll)</t>
+        </is>
+      </c>
+      <c r="AI268" s="5" t="inlineStr">
+        <is>
+          <t>no primary; build 209 (compilation, flagged)</t>
+        </is>
+      </c>
+      <c r="AJ268" s="5" t="inlineStr">
+        <is>
+          <t>[C/E] advanced picket line W of the corridor + reserve knoll: j3-02 draws TWO '8 ohio' bars (4255,5308)/(4390,5273) +-120m; j3-03 bars not redrawn (cartographic omission - presence attested through the action)</t>
+        </is>
+      </c>
+      <c r="AK268" s="5" t="inlineStr">
+        <is>
+          <t>[D] Jul 2 evening forward to the picket line; [D] THE FLANK ACTION: 'changed front forward on the left company ... front to the left flank of the advancing rebel column' (Brockenbrough's documented counterpart)</t>
+        </is>
+      </c>
+      <c r="AL268" s="5" t="inlineStr">
+        <is>
+          <t>[C -55] 'Soon after 2 p.m. ... sixty-four pieces ... in a semicircle which inclosed my position'; [D] flank fire BEFORE Smyth's front volley (sequence bracket); ~200 prisoners, 3 flags (34th NC, 38th Va - pocket mixing)</t>
+        </is>
+      </c>
+      <c r="AM268" s="5" t="inlineStr">
+        <is>
+          <t>return 102 = report 102 EXACT; SPLIT IS PRIMARY: ~45 of 102 fell on the picket line BY NOON Jul 3 - flat-attrition-then-moderate-spike shape (ED-50 candidate), NOT a climax spike</t>
+        </is>
+      </c>
       <c r="AN268" s="5" t="n"/>
-      <c r="AO268" s="5" t="n"/>
+      <c r="AO268" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
@@ -31181,20 +31289,56 @@
           <t>reg-us-i-3-1</t>
         </is>
       </c>
-      <c r="AB272" s="5" t="n"/>
+      <c r="AB272" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC272" s="5" t="n"/>
       <c r="AD272" s="5" t="n"/>
       <c r="AE272" s="5" t="n"/>
       <c r="AF272" s="5" t="n"/>
-      <c r="AG272" s="5" t="n"/>
-      <c r="AH272" s="5" t="n"/>
-      <c r="AI272" s="5" t="n"/>
-      <c r="AJ272" s="5" t="n"/>
-      <c r="AK272" s="5" t="n"/>
-      <c r="AL272" s="5" t="n"/>
-      <c r="AM272" s="5" t="n"/>
+      <c r="AG272" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-i-3-1-biddle.md; 121st/142nd Pa Jul 3 slots sheet-only (flagged)</t>
+        </is>
+      </c>
+      <c r="AH272" s="5" t="inlineStr">
+        <is>
+          <t>Biddle w Jul 1; Rowley register commander; Col. T.B. Gates (20th NYSM) commanded the 2-regiment front element Jul 3, reporting direct to Doubleday (or-27-1-gates)</t>
+        </is>
+      </c>
+      <c r="AI272" s="5" t="inlineStr">
+        <is>
+          <t>no Jul 3 primary; build 460 remnant (compilation, flagged); Jul 1 wreck 898 of ~1,350-1,500 explains scale</t>
+        </is>
+      </c>
+      <c r="AJ272" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 ~17:00 'last and lowest of the ridges' between the roads; [C/E] Jul 3 front line = 80th NY + 151st Pa with the Vermonters (or-27-1-doubleday p.258); j3-02 bars (4482,4569)+(4625,4515); j3-03 (4591,4559) +-120m</t>
+        </is>
+      </c>
+      <c r="AK272" s="5" t="inlineStr">
+        <is>
+          <t>[D] THE CLIMAX LEG: 'by the right flank up to the foot of the bluff, delivering our fire as we marched' then two regiments to the fence - a firing flank-march toward the Copse (~200-400m)</t>
+        </is>
+      </c>
+      <c r="AL272" s="5" t="inlineStr">
+        <is>
+          <t>[D] fire on the march; volley 'at very short range, who now completely broke'; large prisoner haul; 2 colors left on the ground (or-27-1-gates)</t>
+        </is>
+      </c>
+      <c r="AM272" s="5" t="inlineStr">
+        <is>
+          <t>return 898 (80NY 170, 121Pa 179, 142Pa 211, 151Pa 337); DAY SPLIT NOT PRIMARY-SEPARABLE (Gates's 170 = the 80th's battle total, not a Jul 3 figure) - the T4 blocker, recorded honestly</t>
+        </is>
+      </c>
       <c r="AN272" s="5" t="n"/>
-      <c r="AO272" s="5" t="n"/>
+      <c r="AO272" s="5" t="inlineStr">
+        <is>
+          <t>T3 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
@@ -32049,20 +32193,56 @@
           <t>reg-us-ii-3-1</t>
         </is>
       </c>
-      <c r="AB279" s="5" t="n"/>
+      <c r="AB279" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (WITH CAUTION: three regiments are NOT on the II Corps front July 3)</t>
+        </is>
+      </c>
       <c r="AC279" s="5" t="n"/>
       <c r="AD279" s="5" t="n"/>
       <c r="AE279" s="5" t="n"/>
       <c r="AF279" s="5" t="n"/>
-      <c r="AG279" s="5" t="n"/>
-      <c r="AH279" s="5" t="n"/>
-      <c r="AI279" s="5" t="n"/>
-      <c r="AJ279" s="5" t="n"/>
-      <c r="AK279" s="5" t="n"/>
-      <c r="AL279" s="5" t="n"/>
-      <c r="AM279" s="5" t="n"/>
+      <c r="AG279" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-3-1-carroll.md; AUTHORING FLAG: any July 3 render placing these three regiments at the II Corps front contradicts the primary</t>
+        </is>
+      </c>
+      <c r="AH279" s="5" t="inlineStr">
+        <is>
+          <t>Col. S.S. Carroll; 14th Ind (Coons), 4th Oh (Carpenter), 7th WV (Lockwood); report written July 5 AT Two Taverns (earliest-dated Union brigade report fetched)</t>
+        </is>
+      </c>
+      <c r="AI279" s="5" t="inlineStr">
+        <is>
+          <t>no primary; build 640 (compilation, flagged)</t>
+        </is>
+      </c>
+      <c r="AJ279" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jul 2 ~08:00 between Woodruff and Taneytown road; [D vs CA-J2E-3] Jul 2 ~20:00 -&gt; East Cemetery Hill, HELD THROUGH JULY 5 (j2-05 script label (5100,5624) +-150m; residual bars (4671,5265))</t>
+        </is>
+      </c>
+      <c r="AK279" s="5" t="inlineStr">
+        <is>
+          <t>[D vs CA-J2E-3] the night rush, 3 regiments, 14th Ind leading, guided by Howard's aide; no return leg Jul 3</t>
+        </is>
+      </c>
+      <c r="AL279" s="5" t="inlineStr">
+        <is>
+          <t>[D] ECH night fight among Wiedrich/Ricketts guns (or-27-2-hays opposite); [A window] Jul 3 'exposed to a great deal of cross-firing' on the hill (ED-44-class under-fire state); ledger 252 prisoners/113 wounded/37 buried/349 arms</t>
+        </is>
+      </c>
+      <c r="AM279" s="5" t="inlineStr">
+        <is>
+          <t>return 211: 14th Ind 31, 4th Oh 31, 8th Oh 102 (own row), 7th WV 47; episode split Jul-2-night + Jul-3-crossfire dominant (no per-day primary)</t>
+        </is>
+      </c>
       <c r="AN279" s="5" t="n"/>
-      <c r="AO279" s="5" t="n"/>
+      <c r="AO279" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
@@ -32669,20 +32849,56 @@
           <t>reg-us-i-3-2</t>
         </is>
       </c>
-      <c r="AB284" s="5" t="n"/>
+      <c r="AB284" s="5" t="inlineStr">
+        <is>
+          <t>attested-static (sheet grain)</t>
+        </is>
+      </c>
       <c r="AC284" s="5" t="n"/>
       <c r="AD284" s="5" t="n"/>
       <c r="AE284" s="5" t="n"/>
       <c r="AF284" s="5" t="n"/>
-      <c r="AG284" s="5" t="n"/>
-      <c r="AH284" s="5" t="n"/>
-      <c r="AI284" s="5" t="n"/>
-      <c r="AJ284" s="5" t="n"/>
-      <c r="AK284" s="5" t="n"/>
-      <c r="AL284" s="5" t="n"/>
-      <c r="AM284" s="5" t="n"/>
+      <c r="AG284" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-i-3-2-stone.md; NO brigade/regimental report fetched for Jul 2-3 - 150th Pa regimental history is the upgrade route (standing list)</t>
+        </is>
+      </c>
+      <c r="AH284" s="5" t="inlineStr">
+        <is>
+          <t>Stone w Jul 1 -&gt; Wister w Jul 1 -&gt; Col. E.L. Dana (143rd Pa) through the battle's end; 143rd/149th/150th Pa</t>
+        </is>
+      </c>
+      <c r="AI284" s="5" t="inlineStr">
+        <is>
+          <t>no primary; build 465 remnant (compilation, flagged)</t>
+        </is>
+      </c>
+      <c r="AJ284" s="5" t="inlineStr">
+        <is>
+          <t>[C/E] Jul 3 second/third lines behind the Vermont/Gates front (or-27-1-doubleday p.258); j3-02 STONE. (4636,4453); j3-03 STONE'S BRIG. (4755,4466) +-120m, SHALER adjacent - static across both drawn states</t>
+        </is>
+      </c>
+      <c r="AK284" s="5" t="inlineStr">
+        <is>
+          <t>none attested Jul 2-3 (sheet states agree; no report-level stillness statement - negative at sheet grain only)</t>
+        </is>
+      </c>
+      <c r="AL284" s="5" t="inlineStr">
+        <is>
+          <t>[E] present under the cannonade's overs; NO fire window attested Jul 3 (consistent negative)</t>
+        </is>
+      </c>
+      <c r="AM284" s="5" t="inlineStr">
+        <is>
+          <t>return 853 (143Pa 253, 149Pa 336, 150Pa 264); Jul 1 overwhelmingly dominant [D]; build 0 in-window decay consistent</t>
+        </is>
+      </c>
       <c r="AN284" s="5" t="n"/>
-      <c r="AO284" s="5" t="n"/>
+      <c r="AO284" s="5" t="inlineStr">
+        <is>
+          <t>T3 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dossier upgrades (Hall, Harrow, Rittenhouse, Stone/Dana), index pass-5 section, overlay (66 units), master table regen
58 rows now carry audited T-levels. Hall/Harrow July 2 arcs closed
both-sided (T4 full-arc); Rittenhouse T3 with the return-row 13 find
and terminal MOLLUS disposition; Stone/Dana T4 full-arc via the 150th
Pa history (static-July-2 reading corrected by the primary).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -15461,20 +15461,56 @@
           <t>reg-csa-1c-mcl-3</t>
         </is>
       </c>
-      <c r="AB137" s="5" t="n"/>
+      <c r="AB137" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC137" s="5" t="n"/>
       <c r="AD137" s="5" t="n"/>
       <c r="AE137" s="5" t="n"/>
       <c r="AF137" s="5" t="n"/>
-      <c r="AG137" s="5" t="n"/>
-      <c r="AH137" s="5" t="n"/>
-      <c r="AI137" s="5" t="n"/>
-      <c r="AJ137" s="5" t="n"/>
-      <c r="AK137" s="5" t="n"/>
-      <c r="AL137" s="5" t="n"/>
-      <c r="AM137" s="5" t="n"/>
+      <c r="AG137" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-mcl-3-barksdale.md</t>
+        </is>
+      </c>
+      <c r="AH137" s="5" t="inlineStr">
+        <is>
+          <t>Barksdale's bde (13/17/18/21 MS); Barksdale mw at Plum Run ~19:00 (tablet + Hall's 20-yards receiving-side pin, compatible ~100 m grain), d. July 3 Hummelbaugh farm -&gt; Humphreys. NO OR REPORT at any echelon (verified-negative class)</t>
+        </is>
+      </c>
+      <c r="AI137" s="5" t="inlineStr">
+        <is>
+          <t>tablet 'Present 1,598' (compilation, hop flagged); no primary</t>
+        </is>
+      </c>
+      <c r="AJ137" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet] Warfield line from ~15:00; [E drawn j2-03 17:00] rgt numbers with advance arrows POISED not advanced (2923,3865) - drawn state contradicts the tablet's 'Advanced at 5 P.M.'; [E drawn j2-04 19:00] TWO ELEMENTS: main body vs Willard at Plum Run (4053,4080), 21st MS at Trostle/Bigelow (3617,3643) with WATSON (4093,3607)</t>
+        </is>
+      </c>
+      <c r="AK137" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J2A-9 ~18:15] step-off via Lamar order + drums pin + Alexander's 20-min ladder interval; the battery-extraction delay (McLaws); [B] ~600 m to the orchard then divergent axes; Plum Run collapse 19:00-19:15</t>
+        </is>
+      </c>
+      <c r="AL137" s="5" t="inlineStr">
+        <is>
+          <t>[D] the salient breach with Kershaw's 8th SC flank fire; 21st MS took Bigelow's 9th MA + Watson's I/5th US 'unable to bring off'; July 3 artillery support at the orchard (ED-44 adjacent)</t>
+        </is>
+      </c>
+      <c r="AM137" s="5" t="inlineStr">
+        <is>
+          <t>tablet ITEMIZES the return's pooled missing: 105/550/92 = 747 EXACT match (first tablet-closes-ED-49-gap case); ~804 B&amp;M variant carried; split concentrated 18:15-19:15</t>
+        </is>
+      </c>
       <c r="AN137" s="5" t="n"/>
-      <c r="AO137" s="5" t="n"/>
+      <c r="AO137" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -16577,20 +16613,56 @@
           <t>reg-csa-1c-mcl-1</t>
         </is>
       </c>
-      <c r="AB146" s="5" t="n"/>
+      <c r="AB146" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC146" s="5" t="n"/>
       <c r="AD146" s="5" t="n"/>
       <c r="AE146" s="5" t="n"/>
       <c r="AF146" s="5" t="n"/>
-      <c r="AG146" s="5" t="n"/>
-      <c r="AH146" s="5" t="n"/>
-      <c r="AI146" s="5" t="n"/>
-      <c r="AJ146" s="5" t="n"/>
-      <c r="AK146" s="5" t="n"/>
-      <c r="AL146" s="5" t="n"/>
-      <c r="AM146" s="5" t="n"/>
+      <c r="AG146" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-mcl-1-kershaw.md; ED-55 candidate exemplar (wing report-clock skew +90)</t>
+        </is>
+      </c>
+      <c r="AH146" s="5" t="inlineStr">
+        <is>
+          <t>Kershaw's bde (2/3/7/8/15 SC + 3d SC Bn); Kershaw unwounded; De Saussure k, McLeod mw, Kennedy/Bland/Miller w (all July 2)</t>
+        </is>
+      </c>
+      <c r="AI146" s="5" t="inlineStr">
+        <is>
+          <t>tablet 'Present about 1800' (compilation); no report statement</t>
+        </is>
+      </c>
+      <c r="AJ146" s="5" t="inlineStr">
+        <is>
+          <t>[C report +90] the stone wall 'about 3 p.m.' stated; [E drawn] KERSHAW advance line (3941,3263) at 17:00 j2-03; stony-hill W edge (3308,3336) at 19:00 j2-04; July 2 dark Peach Orchard -&gt; July 3 13:00 original wall (tablet+report)</t>
+        </is>
+      </c>
+      <c r="AK146" s="5" t="inlineStr">
+        <is>
+          <t>[trigger first-class] CABELL'S THREE-GUN SIGNAL step-off; Longstreet on foot to the road; [D] Barksdale's drums heard at the road (the ladder interval, Alexander: 20+ min); Wheatfield oscillation; nightfall withdrawal</t>
+        </is>
+      </c>
+      <c r="AL146" s="5" t="inlineStr">
+        <is>
+          <t>[D] stony hill fight at 30 paces; Caldwell's two-line counterattack; the Wofford resweep to the mountain's foot; July 3 Peach Orchard skirmish only</t>
+        </is>
+      </c>
+      <c r="AM146" s="5" t="inlineStr">
+        <is>
+          <t>THE CLEAN CASE: report = return = tablet 115/483/32 = 630 (2nd SC row blank - itemization gap flagged)</t>
+        </is>
+      </c>
       <c r="AN146" s="5" t="n"/>
-      <c r="AO146" s="5" t="n"/>
+      <c r="AO146" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -17021,20 +17093,56 @@
           <t>reg-csa-1c-hood-1</t>
         </is>
       </c>
-      <c r="AB149" s="5" t="n"/>
+      <c r="AB149" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC149" s="5" t="n"/>
       <c r="AD149" s="5" t="n"/>
       <c r="AE149" s="5" t="n"/>
       <c r="AF149" s="5" t="n"/>
-      <c r="AG149" s="5" t="n"/>
-      <c r="AH149" s="5" t="n"/>
-      <c r="AI149" s="5" t="n"/>
-      <c r="AJ149" s="5" t="n"/>
-      <c r="AK149" s="5" t="n"/>
-      <c r="AL149" s="5" t="n"/>
-      <c r="AM149" s="5" t="n"/>
+      <c r="AG149" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-hood-1-law.md; contributes CSA side of ED-53 candidate (step-off ~16:30 +-15)</t>
+        </is>
+      </c>
+      <c r="AH149" s="5" t="inlineStr">
+        <is>
+          <t>Law's bde (4/15/44/47/48 AL); Law to DIVISION at the step-off (Hood w) -&gt; Sheffield; Feagin w; no brigade report by Law (verified negative - five regimental reports are the OR base)</t>
+        </is>
+      </c>
+      <c r="AI149" s="5" t="inlineStr">
+        <is>
+          <t>tablet ~1,500 (compilation); 15th AL 'about five hundred' primary (oates-1905); the 22-man water detail captured entire pre-fight</t>
+        </is>
+      </c>
+      <c r="AJ149" s="5" t="inlineStr">
+        <is>
+          <t>[C] step-off line 50 yd W of tablet; [E drawn j2-03] 15 Ala bar (4345,2343) vs VINCENT'S SPUR, 44 Ala (3795,2538) at Plum Run; night line Round Top west foot (j2-05 drawn)</t>
+        </is>
+      </c>
+      <c r="AK149" s="5" t="inlineStr">
+        <is>
+          <t>[B] New Guilford 25 mi 03:30-04:00 -&gt; 12:00-14:00 (three-way arrival spread carried); [A vs CA-J2A-3 ~16:30] assault leg; Oates's Round Top excursion [D]; dusk withdrawal</t>
+        </is>
+      </c>
+      <c r="AL149" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J2A-6] the five-charges fight (attacker's own count = Chamberlain's); Devil's Den taken 'in less than an hour' (Law, tier-B input); July 3 skirmish + Farnsworth repulse 17:00 [C tablet]</t>
+        </is>
+      </c>
+      <c r="AM149" s="5" t="inlineStr">
+        <is>
+          <t>return 74/276/146-pooled=496 (ED-49); 15th AL report 161 vs row 83 and 4th AL 87 vs 66 (rule-4 exemplars); ~400 prisoners receiving-side cross-check</t>
+        </is>
+      </c>
       <c r="AN149" s="5" t="n"/>
-      <c r="AO149" s="5" t="n"/>
+      <c r="AO149" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -18049,20 +18157,56 @@
           <t>reg-csa-1c-hood-2</t>
         </is>
       </c>
-      <c r="AB157" s="5" t="n"/>
+      <c r="AB157" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC157" s="5" t="n"/>
       <c r="AD157" s="5" t="n"/>
       <c r="AE157" s="5" t="n"/>
       <c r="AF157" s="5" t="n"/>
-      <c r="AG157" s="5" t="n"/>
-      <c r="AH157" s="5" t="n"/>
-      <c r="AI157" s="5" t="n"/>
-      <c r="AJ157" s="5" t="n"/>
-      <c r="AK157" s="5" t="n"/>
-      <c r="AL157" s="5" t="n"/>
-      <c r="AM157" s="5" t="n"/>
+      <c r="AG157" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-hood-2-robertson.md</t>
+        </is>
+      </c>
+      <c r="AH157" s="5" t="inlineStr">
+        <is>
+          <t>Texas bde (1/4/5 TX + 3 AR); Robertson w late evening July 2 -&gt; Work; six field-officer w pins July 2; Price AAG lost July 3 morning</t>
+        </is>
+      </c>
+      <c r="AI157" s="5" t="inlineStr">
+        <is>
+          <t>tablet ~1,100 (compilation); no primary statement</t>
+        </is>
+      </c>
+      <c r="AJ157" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet] arrived ~16:00, left ordered on the pike - ABANDONED by his decision to close on Law (primary); [E drawn j2-03] TX bars in Plum Run valley; July 3 Big Round Top NW spur (tablet)</t>
+        </is>
+      </c>
+      <c r="AK157" s="5" t="inlineStr">
+        <is>
+          <t>[B] half-mile open-ground assault leg under Smith's canister; the 4th/5th TX right-drift to Law; 1st TX battery-hill sequence</t>
+        </is>
+      </c>
+      <c r="AL157" s="5" t="inlineStr">
+        <is>
+          <t>[B] over-an-hour Devil's Den contest; 3 of 6 Smith's guns (CROSS-CREDIT conflict with Law's 44th/48th - carried); July 3 continuous skirmishing (primary)</t>
+        </is>
+      </c>
+      <c r="AM157" s="5" t="inlineStr">
+        <is>
+          <t>return 84/393/120-pooled=597 (ED-49; 1st TX row transcription inconsistency flagged); tablet ~540 variant</t>
+        </is>
+      </c>
       <c r="AN157" s="5" t="n"/>
-      <c r="AO157" s="5" t="n"/>
+      <c r="AO157" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -26688,7 +26832,7 @@
       <c r="AF235" s="5" t="n"/>
       <c r="AG235" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-btty-rittenhouse.md; rittenhouse-mollus-1887 = the T-ceiling item</t>
+          <t>Dossier: reconstruction/dossiers/us-btty-rittenhouse.md; rittenhouse-mollus-1887 = the T-ceiling item; pass-5: MOLLUS round 4 TERMINAL (library/CDL); summit anchor refined to (4200,2600) +-80</t>
         </is>
       </c>
       <c r="AH235" s="5" t="inlineStr">
@@ -26718,13 +26862,13 @@
       </c>
       <c r="AM235" s="5" t="inlineStr">
         <is>
-          <t>14 (1 off + 8 men k, 5 w, tablet; ~19% of 73); Jul 2 dominates [D]; brigade frame 44 total (Martin)</t>
+          <t>return row 7/6/0=13 (p. 180, landed pass 5) vs tablet 14 - ED-52 adopts the return; episode split July 2 dominant (Hazlett mw)</t>
         </is>
       </c>
       <c r="AN235" s="5" t="n"/>
       <c r="AO235" s="5" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T3</t>
         </is>
       </c>
     </row>
@@ -31284,7 +31428,7 @@
       <c r="AF273" s="5" t="n"/>
       <c r="AG273" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-ii-2-3-hall.md; p.438 extraction gap + 'Should be Arnold's' footnote -&gt; ED-40 candidate</t>
+          <t>Dossier: reconstruction/dossiers/us-ii-2-3-hall.md; p.438 extraction gap + 'Should be Arnold's' footnote -&gt; ED-40 candidate; pass-5: July 2 arc closed both-sided (csa-1c-mcl-3-barksdale.md pairing; Barksdale-pin compatibility note)</t>
         </is>
       </c>
       <c r="AH273" s="5" t="inlineStr">
@@ -31320,7 +31464,7 @@
       <c r="AN273" s="5" t="n"/>
       <c r="AO273" s="5" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T4 full-arc (T5-grade window via V2 claims)</t>
         </is>
       </c>
     </row>
@@ -33852,7 +33996,7 @@
       <c r="AF292" s="5" t="n"/>
       <c r="AG292" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-i-3-2-stone.md; NO brigade/regimental report fetched for Jul 2-3 - 150th Pa regimental history is the upgrade route (standing list)</t>
+          <t>Dossier: reconstruction/dossiers/us-i-3-2-stone.md; NO brigade/regimental report fetched for Jul 2-3 - 150th Pa regimental history is the upgrade route (standing list); pass-5: 150th Pa history standing fetch LANDED - static July 2 reading corrected, named July 3 morning losses</t>
         </is>
       </c>
       <c r="AH292" s="5" t="inlineStr">
@@ -33862,7 +34006,7 @@
       </c>
       <c r="AI292" s="5" t="inlineStr">
         <is>
-          <t>no primary; build 465 remnant (compilation, flagged)</t>
+          <t>150th Pa 'aggregate for duty ... one hundred and nine' July 2 morning (chamberlin-150pa-1895, primary-adjacent); build 465 brigade remnant consistent</t>
         </is>
       </c>
       <c r="AJ292" s="5" t="inlineStr">
@@ -33872,7 +34016,7 @@
       </c>
       <c r="AK292" s="5" t="inlineStr">
         <is>
-          <t>none attested Jul 2-3 (sheet states agree; no report-level stillness statement - negative at sheet grain only)</t>
+          <t>[C ~18:00] July 2 double-quick down the Taneytown road to Humphreys's rear; 149th+150th to the Emmitsburg road recovering TWO GUNS (Doubleday concurring); night picket left of Codori; [C 07:00-08:00] July 3 relief under fire</t>
         </is>
       </c>
       <c r="AL292" s="5" t="inlineStr">
@@ -33888,7 +34032,7 @@
       <c r="AN292" s="5" t="n"/>
       <c r="AO292" s="5" t="inlineStr">
         <is>
-          <t>T3 full-arc</t>
+          <t>T4 full-arc</t>
         </is>
       </c>
     </row>
@@ -34497,20 +34641,56 @@
           <t>reg-us-v-2-3</t>
         </is>
       </c>
-      <c r="AB297" s="5" t="n"/>
+      <c r="AB297" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC297" s="5" t="n"/>
       <c r="AD297" s="5" t="n"/>
       <c r="AE297" s="5" t="n"/>
       <c r="AF297" s="5" t="n"/>
-      <c r="AG297" s="5" t="n"/>
-      <c r="AH297" s="5" t="n"/>
-      <c r="AI297" s="5" t="n"/>
-      <c r="AJ297" s="5" t="n"/>
-      <c r="AK297" s="5" t="n"/>
-      <c r="AL297" s="5" t="n"/>
-      <c r="AM297" s="5" t="n"/>
+      <c r="AG297" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-v-2-3-weed.md; paired battery us-btty-rittenhouse.md</t>
+        </is>
+      </c>
+      <c r="AH297" s="5" t="inlineStr">
+        <is>
+          <t>Weed's bde (140/146 NY, 91/155 PA); Weed mw on the summit near the battery, d. ~21:00 ('dead as Julius Caesar', Farley) -&gt; Garrard; O'Rorke mw at the head of the 140th; Hazlett pin paired (one primary)</t>
+        </is>
+      </c>
+      <c r="AI297" s="5" t="inlineStr">
+        <is>
+          <t>no brigade primary (open; compilation tier)</t>
+        </is>
+      </c>
+      <c r="AJ297" s="5" t="inlineStr">
+        <is>
+          <t>[D] the Sickles-diversion + Sykes double-quick recall (or-27-1-sykes); [E drawn j2-03] WEED bar at the summit (4169,2640) +-62 m with the signal station; night stone wall half-way down the slope (primary)</t>
+        </is>
+      </c>
+      <c r="AK297" s="5" t="inlineStr">
+        <is>
+          <t>[B] 140th's summit rush 300-400 m at the double, in by companies without loading (Farley); brigade following under Weed</t>
+        </is>
+      </c>
+      <c r="AL297" s="5" t="inlineStr">
+        <is>
+          <t>[D] the 17:30-18:30 crisis fire on the 16th MI right; summit hold under Devil's Den sharpshooter fire; July 3 held (battery window on the paired dossier)</t>
+        </is>
+      </c>
+      <c r="AM297" s="5" t="inlineStr">
+        <is>
+          <t>return: 140th NY 133 exact; brigade 200, division 1,029; three regiment rows digit-noisy (flagged); pins O'Rorke early / Weed late / Hazlett after Weed</t>
+        </is>
+      </c>
       <c r="AN297" s="5" t="n"/>
-      <c r="AO297" s="5" t="n"/>
+      <c r="AO297" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
@@ -35004,7 +35184,7 @@
       <c r="AF301" s="5" t="n"/>
       <c r="AG301" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-ii-2-1-harrow.md; division-sum gap 3,580 vs 3,773 recorded</t>
+          <t>Dossier: reconstruction/dossiers/us-ii-2-1-harrow.md; division-sum gap 3,580 vs 3,773 recorded; pass-5: July 2 evening counterattack leg both-sided (1st MN bracketed after CA-J2A-9, before sunset ED-31)</t>
         </is>
       </c>
       <c r="AH301" s="5" t="inlineStr">
@@ -35040,7 +35220,7 @@
       <c r="AN301" s="5" t="n"/>
       <c r="AO301" s="5" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T4 full-arc</t>
         </is>
       </c>
     </row>
@@ -36517,20 +36697,56 @@
           <t>reg-us-v-1-3</t>
         </is>
       </c>
-      <c r="AB313" s="5" t="n"/>
+      <c r="AB313" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover; July 3 ED-44 class)</t>
+        </is>
+      </c>
       <c r="AC313" s="5" t="n"/>
       <c r="AD313" s="5" t="n"/>
       <c r="AE313" s="5" t="n"/>
       <c r="AF313" s="5" t="n"/>
-      <c r="AG313" s="5" t="n"/>
-      <c r="AH313" s="5" t="n"/>
-      <c r="AI313" s="5" t="n"/>
-      <c r="AJ313" s="5" t="n"/>
-      <c r="AK313" s="5" t="n"/>
-      <c r="AL313" s="5" t="n"/>
-      <c r="AM313" s="5" t="n"/>
+      <c r="AG313" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-v-1-3-vincent.md; Warren letters = CA-J2A-4 primary base</t>
+        </is>
+      </c>
+      <c r="AH313" s="5" t="inlineStr">
+        <is>
+          <t>Vincent's bde (20 ME/16 MI/44 NY/83 PA); Vincent mw July 2 (16th MI crisis; d. July 7) -&gt; Rice; Linscott mw 21:00</t>
+        </is>
+      </c>
+      <c r="AI313" s="5" t="inlineStr">
+        <is>
+          <t>'about 1,000 muskets' - the brigade commander's own statement (primary, or-27-1-rice-vincent)</t>
+        </is>
+      </c>
+      <c r="AJ313" s="5" t="inlineStr">
+        <is>
+          <t>[C +45] extreme left 'about 4 p.m.' stated; line 20ME|83PA|44NY|16MI; [E drawn j2-03] VINCENT'S SPUR label (4256,2309), 16 MICH (4158,2503); [C 21:00] 20th ME ON Great Round Top - DRAWN on j2-05; July 3 relieved to the CENTER as reserve (primary - ED-54 candidate placement rule)</t>
+        </is>
+      </c>
+      <c r="AK313" s="5" t="inlineStr">
+        <is>
+          <t>[D+B] the self-diverted rush to the hill (~700 m at the double); the 20th ME left-refuse + right-wheel charge; the 21:00 night ascent (~200 men, no firing)</t>
+        </is>
+      </c>
+      <c r="AL313" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J2A-6] the defense 16:45-19:00; ammunition crisis (brigade-attested); 'now 8 o clock in the evening' repulse-complete clock (best Union primary end-clock of the phase); 500+ prisoners/1,000 muskets</t>
+        </is>
+      </c>
+      <c r="AM313" s="5" t="inlineStr">
+        <is>
+          <t>return exact-grain: 20 ME 125, 16 MI 60, 44 NY 111, 83 PA 55 = 352 (ED-52 basis; 20th ME narrative 130-136 carried not promoted); single-window brigade (July 3 lossless per Rice)</t>
+        </is>
+      </c>
       <c r="AN313" s="5" t="n"/>
-      <c r="AO313" s="5" t="n"/>
+      <c r="AO313" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Audit d6: sources +13 (145), standing-fetch dispositions, overlay +13 (79 units), master table regenerated (79 audited rows), bundle metadata recompiled
Weed digit-noise re-read CLOSED (aggregates firm 133/28/19/19);
Rittenhouse round-5 negative (terminal stands); Busey/Pfanz retries
negative (dispositions re-confirmed). ED-21 stagingSeed pin held.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -15337,20 +15337,56 @@
           <t>reg-csa-1c-hood-3</t>
         </is>
       </c>
-      <c r="AB136" s="5" t="n"/>
+      <c r="AB136" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC136" s="5" t="n"/>
       <c r="AD136" s="5" t="n"/>
       <c r="AE136" s="5" t="n"/>
       <c r="AF136" s="5" t="n"/>
-      <c r="AG136" s="5" t="n"/>
-      <c r="AH136" s="5" t="n"/>
-      <c r="AI136" s="5" t="n"/>
-      <c r="AJ136" s="5" t="n"/>
-      <c r="AK136" s="5" t="n"/>
-      <c r="AL136" s="5" t="n"/>
-      <c r="AM136" s="5" t="n"/>
+      <c r="AG136" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-hood-3-anderson.md; White's report is a consolidation (one hop above regimental layer, carried)</t>
+        </is>
+      </c>
+      <c r="AH136" s="5" t="inlineStr">
+        <is>
+          <t>G.T. Anderson's bde (7/8/9/11/59 GA); ANDERSON W in the second advance (marker (3529,2729) = check point) -&gt; Luffman register succession; report filed by Col. W. W. White (7th GA) - the report chain attests the churn</t>
+        </is>
+      </c>
+      <c r="AI136" s="5" t="inlineStr">
+        <is>
+          <t>tablet 'Present about 1800'; 7th GA detached to the cavalry flank pre-fight (named EC2 subtraction, ~4/5 engaged)</t>
+        </is>
+      </c>
+      <c r="AJ136" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet] formed ~16:00 division left; [E drawn j2-03] 'ANDERSON'S GA' advancing (3269,2902) + Rose Woods red line (3549,2849); third-advance end = woodland to Plum Run border; July 3 = the Emmitsburg Rd cavalry flank (NOT a Wheatfield hold)</t>
+        </is>
+      </c>
+      <c r="AK136" s="5" t="inlineStr">
+        <is>
+          <t>[D structure] THREE ADVANCES stated (stone fence taken / outflanked-retired / Anderson w / third 'half an hour in the ravine' - wave-4 duration input)</t>
+        </is>
+      </c>
+      <c r="AL136" s="5" t="inlineStr">
+        <is>
+          <t>[D] wave-1 stone-fence fight vs de Trobriand (both-sided); wave-3 receiving (Kelly tablet NAMES this brigade); July 3 Farnsworth-front actions</t>
+        </is>
+      </c>
+      <c r="AM136" s="5" t="inlineStr">
+        <is>
+          <t>tablet total = return total EXACT 671 (105/512/[54 pooled]); White's composition agrees at class; July2/3 split unstated (flagged)</t>
+        </is>
+      </c>
       <c r="AN136" s="5" t="n"/>
-      <c r="AO136" s="5" t="n"/>
+      <c r="AO136" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -15621,20 +15657,56 @@
           <t>reg-csa-1c-hood-4</t>
         </is>
       </c>
-      <c r="AB138" s="5" t="n"/>
+      <c r="AB138" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover; July 2-3 holder)</t>
+        </is>
+      </c>
       <c r="AC138" s="5" t="n"/>
       <c r="AD138" s="5" t="n"/>
       <c r="AE138" s="5" t="n"/>
       <c r="AF138" s="5" t="n"/>
-      <c r="AG138" s="5" t="n"/>
-      <c r="AH138" s="5" t="n"/>
-      <c r="AI138" s="5" t="n"/>
-      <c r="AJ138" s="5" t="n"/>
-      <c r="AK138" s="5" t="n"/>
-      <c r="AL138" s="5" t="n"/>
-      <c r="AM138" s="5" t="n"/>
+      <c r="AG138" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-hood-4-benning.md; third claimant in the guns cross-credit - ED-56 convergent-capture candidate; count/type agreement with Smith across the lines</t>
+        </is>
+      </c>
+      <c r="AH138" s="5" t="inlineStr">
+        <is>
+          <t>Benning's bde (2/15/17/20 GA); Benning unwounded; Cols. Jones (20GA) k + Harris (2GA) k in the Den fight</t>
+        </is>
+      </c>
+      <c r="AI138" s="5" t="inlineStr">
+        <is>
+          <t>tablet 'Present about 1500' (compilation, hop flagged)</t>
+        </is>
+      </c>
+      <c r="AJ138" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet] formed ~400yd behind the first line (2785,2269); [A vs CA-J2A-5] Devil's Den taken ~17:30 AND HELD to July 3 late day (advance marker (3697,2461)); [E drawn j2-04+j2-05] red line holding the Den across two sheets - drawn-state continuity</t>
+        </is>
+      </c>
+      <c r="AK138" s="5" t="inlineStr">
+        <is>
+          <t>[D first-person] THE WRONG-BRIGADE FOLLOW ('In truth, it was Robertson's') - the ladder's best-documented formation error; [B] 600-800yd ascent under fire 15-25 min; [D] the 15th GA mistaken-orders withdrawal disaster July 3</t>
+        </is>
+      </c>
+      <c r="AL138" s="5" t="inlineStr">
+        <is>
+          <t>[D] Den fight intermixed with 1st TX; gun-shelf enumeration matches Union battery dossiers gun-for-gun; overnight+July 3 hold under fire; McLaws-withdrawn-from-my-left exposure note</t>
+        </is>
+      </c>
+      <c r="AM138" s="5" t="inlineStr">
+        <is>
+          <t>three readings carried: report floor 'not less than 400', return 76/299/[122 pooled]=497 (adopted basis), tablet 509; loss SPREAD over the 2-day hold (not a single spike); 15th GA July 3 component unquantified (flagged)</t>
+        </is>
+      </c>
       <c r="AN138" s="5" t="n"/>
-      <c r="AO138" s="5" t="n"/>
+      <c r="AO138" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -18317,20 +18389,56 @@
           <t>reg-csa-1c-mcl-2</t>
         </is>
       </c>
-      <c r="AB158" s="5" t="n"/>
+      <c r="AB158" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC158" s="5" t="n"/>
       <c r="AD158" s="5" t="n"/>
       <c r="AE158" s="5" t="n"/>
       <c r="AF158" s="5" t="n"/>
-      <c r="AG158" s="5" t="n"/>
-      <c r="AH158" s="5" t="n"/>
-      <c r="AI158" s="5" t="n"/>
-      <c r="AJ158" s="5" t="n"/>
-      <c r="AK158" s="5" t="n"/>
-      <c r="AL158" s="5" t="n"/>
-      <c r="AM158" s="5" t="n"/>
+      <c r="AG158" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-mcl-2-semmes.md</t>
+        </is>
+      </c>
+      <c r="AH158" s="5" t="inlineStr">
+        <is>
+          <t>Semmes's bde (10/50/51/53 GA); SEMMES MW 'in the ravine near the Loop' (tablet verbatim; advance marker (3357,2864) = check point), d. July 10 -&gt; Bryan. NO OR REPORT at any echelon (verified-negative - the Barksdale class)</t>
+        </is>
+      </c>
+      <c r="AI158" s="5" t="inlineStr">
+        <is>
+          <t>tablet 'Present about 1200' (compilation, hop flagged); no primary</t>
+        </is>
+      </c>
+      <c r="AJ158" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J2A-7] Kershaw's support slot (Alexander ladder attack 3); [C tablet] Rose Hill/ravine/Loop fight; wave-4 sweep to Plum Run; July 3 the woodland S of Wheatfield to 13:00 (Benning's exposed-left note cross-bears the extraction)</t>
+        </is>
+      </c>
+      <c r="AK158" s="5" t="inlineStr">
+        <is>
+          <t>[D trigger] committal = Kershaw's 'Semmes brought up' (supported unit's primary); [B] 400m ravine advance</t>
+        </is>
+      </c>
+      <c r="AL158" s="5" t="inlineStr">
+        <is>
+          <t>[D] ravine fight vs Kelly/Zook/Brooke prongs (both-sided); July 3 woodland occupancy (ED-44 adjacent)</t>
+        </is>
+      </c>
+      <c r="AM158" s="5" t="inlineStr">
+        <is>
+          <t>tablet total = return total EXACT 430 (55/284/[91 pooled]); the SECOND tablet-corroborates-pooled-scope case after Barksdale; split: waves 2-4 ~all</t>
+        </is>
+      </c>
       <c r="AN158" s="5" t="n"/>
-      <c r="AO158" s="5" t="n"/>
+      <c r="AO158" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc (thin - no-report class)</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -18948,7 +19056,7 @@
       <c r="AF163" s="5" t="n"/>
       <c r="AG163" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/csa-3c-and-1-wilcox.md; CA-J3A-10 executor</t>
+          <t>Dossier: reconstruction/dossiers/csa-3c-and-1-wilcox.md; CA-J3A-10 executor; July 2 arc extended backward pass 6 (CA-J2A-10 executor leg)</t>
         </is>
       </c>
       <c r="AH163" s="5" t="inlineStr">
@@ -18963,12 +19071,12 @@
       </c>
       <c r="AJ163" s="5" t="inlineStr">
         <is>
-          <t>[D] before sunrise: line parallel to Emmitsburg pike ~200 yd W, Alexander's guns in front; j3-01 label ~(3100,4400)+-120 (04:00-08:00 window = exact bracket); farthest advance = ravine below McGilvery crest (build displacement understates - flag)</t>
+          <t>[D] before sunrise: line parallel to Emmitsburg pike ~200 yd W, Alexander's guns in front; j3-01 label ~(3100,4400)+-120 (04:00-08:00 window = exact bracket); farthest advance = ravine below McGilvery crest (build displacement understates - flag); PASS-6 BACKWARD-EXTENSION: [A vs CA-J2A-10] July 2 evening advance (pike crossing, two lines broken, 2+6 guns claimed, the ravine climb); [E drawn j2-04] WILCOX ALA (4112,4368) opposite '1 Minn' (4230,4282) - the sheet draws BOTH sides of the charge moment</t>
         </is>
       </c>
       <c r="AK163" s="5" t="inlineStr">
         <is>
-          <t>[A vs CA-J3A-6 +20-30 min] the DELAYED LAUNCH (three staff officers in succession; Alexander concurs; Lang sequences after repulse - one envelope); halt at ravine awaiting artillery that had no ammunition; withdrew on own judgment</t>
+          <t>[A vs CA-J3A-6 +20-30 min] the DELAYED LAUNCH (three staff officers in succession; Alexander concurs; Lang sequences after repulse - one envelope); halt at ravine awaiting artillery that had no ammunition; withdrew on own judgment; PASS-6: [D duration] the thirty-minute unsupported stand + withdrawal; the third-line-at-the-double-quick = the 1st MN charge from the receiving side (both-sided with or-27-1-coates-1mn)</t>
         </is>
       </c>
       <c r="AL163" s="5" t="inlineStr">
@@ -19097,20 +19205,56 @@
           <t>reg-csa-1c-mcl-4</t>
         </is>
       </c>
-      <c r="AB164" s="5" t="n"/>
+      <c r="AB164" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC164" s="5" t="n"/>
       <c r="AD164" s="5" t="n"/>
       <c r="AE164" s="5" t="n"/>
       <c r="AF164" s="5" t="n"/>
-      <c r="AG164" s="5" t="n"/>
-      <c r="AH164" s="5" t="n"/>
-      <c r="AI164" s="5" t="n"/>
-      <c r="AJ164" s="5" t="n"/>
-      <c r="AK164" s="5" t="n"/>
-      <c r="AL164" s="5" t="n"/>
-      <c r="AM164" s="5" t="n"/>
+      <c r="AG164" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-mcl-4-wofford.md; tablet clock 'about 6 P.M.' is a NEAR-ZERO skew exemplar - the wing's tablet skew is heterogeneous (ED-58 discussion)</t>
+        </is>
+      </c>
+      <c r="AH164" s="5" t="inlineStr">
+        <is>
+          <t>Wofford's bde (16/18/24 GA, Cobb's + Phillips Legions); Wofford unwounded; NO OR REPORT (verified-negative)</t>
+        </is>
+      </c>
+      <c r="AI164" s="5" t="inlineStr">
+        <is>
+          <t>tablet 'Present about 1350' (compilation, hop flagged)</t>
+        </is>
+      </c>
+      <c r="AJ164" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet] formed 100yd W of tablet (2652,3802); the Wheatfield-Rd sweep axis; farthest = LRT foot; [A vs CA-J2A-11] FELL BACK AT SUNSET (19:29 astronomical pin - the ladder's only document-grade end clock); [E drawn j2-05] red bars w/ withdrawal arrows on the Wheatfield's W ravine slope, '...FORD GA' label class (legibility partial, flagged) opposite McCandless (4011,3016)/Nevin (4290,3119)</t>
+        </is>
+      </c>
+      <c r="AK164" s="5" t="inlineStr">
+        <is>
+          <t>[B] ~1200m road-axis sweep 15-20 min; trigger both-sided (Kershaw's 'Wofford coming in in splendid style' + Fraser's flanked-right + Alexander's attack-4 ladder)</t>
+        </is>
+      </c>
+      <c r="AL164" s="5" t="inlineStr">
+        <is>
+          <t>[D] wave-4 flank sweep to the mountain's foot; the Crawford/McCandless collision; July 3 orchard-ridge artillery support</t>
+        </is>
+      </c>
+      <c r="AM164" s="5" t="inlineStr">
+        <is>
+          <t>CONFLICT: tablet itemizes 36/207/112=355 vs return 30/192/[112 pooled]=334 - missing agrees EXACTLY, k/w disagree; no own report to resolve; EC6 carries '334-355, missing 112 firm', NO promotion</t>
+        </is>
+      </c>
       <c r="AN164" s="5" t="n"/>
-      <c r="AO164" s="5" t="n"/>
+      <c r="AO164" s="5" t="inlineStr">
+        <is>
+          <t>T3 full-arc (EC6 conflicted)</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -20949,20 +21093,56 @@
           <t>reg-us-iii-b3</t>
         </is>
       </c>
-      <c r="AB183" s="5" t="n"/>
+      <c r="AB183" s="5" t="inlineStr">
+        <is>
+          <t>unauthored (not-yet-cast)</t>
+        </is>
+      </c>
       <c r="AC183" s="5" t="n"/>
       <c r="AD183" s="5" t="n"/>
       <c r="AE183" s="5" t="n"/>
       <c r="AF183" s="5" t="n"/>
-      <c r="AG183" s="5" t="n"/>
-      <c r="AH183" s="5" t="n"/>
-      <c r="AI183" s="5" t="n"/>
-      <c r="AJ183" s="5" t="n"/>
-      <c r="AK183" s="5" t="n"/>
-      <c r="AL183" s="5" t="n"/>
-      <c r="AM183" s="5" t="n"/>
+      <c r="AG183" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-smith.md; THE GUNS CROSS-CREDIT closed both-sided - exactly 3 Parrotts lost, CSA count/type agrees; ED-56 convergent-capture candidate</t>
+        </is>
+      </c>
+      <c r="AH183" s="5" t="inlineStr">
+        <is>
+          <t>Smith's 4th NY Independent (6x 10-pdr Parrott); Smith unwounded; 2 k named</t>
+        </is>
+      </c>
+      <c r="AI183" s="5" t="inlineStr">
+        <is>
+          <t>six guns, two elements (4 forward + 2 rear); personnel compilation-tier</t>
+        </is>
+      </c>
+      <c r="AJ183" s="5" t="inlineStr">
+        <is>
+          <t>[C report] forward guns on the Devil's Den hill (mon (3787,2551)); rear section 150yd back in Plum Run valley (mon (4016,2802)); [E drawn j2-03] 'Smith' drawn as a SEPARATE rear element (4016,2946) - two-element drawn state</t>
+        </is>
+      </c>
+      <c r="AK183" s="5" t="inlineStr">
+        <is>
+          <t>[D] forward guns attested-static to loss (kept firing rather than signal retreat); captain's shift to the rear section at the fall</t>
+        </is>
+      </c>
+      <c r="AL183" s="5" t="inlineStr">
+        <is>
+          <t>[C +90] duel from stated 14:30; munition ladder case-&gt;shell-&gt;canister (range-attesting); 140 ROUNDS EXPENDED (expenditure ledger, ED-42); oblique gully fire</t>
+        </is>
+      </c>
+      <c r="AM183" s="5" t="inlineStr">
+        <is>
+          <t>return 13 adopted (2/10/1) vs report 12 named (ED-52); concentrated in the forward fight</t>
+        </is>
+      </c>
       <c r="AN183" s="5" t="n"/>
-      <c r="AO183" s="5" t="n"/>
+      <c r="AO183" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -32301,20 +32481,56 @@
           <t>reg-us-iii-1-2</t>
         </is>
       </c>
-      <c r="AB279" s="5" t="n"/>
+      <c r="AB279" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 defender)</t>
+        </is>
+      </c>
       <c r="AC279" s="5" t="n"/>
       <c r="AD279" s="5" t="n"/>
       <c r="AE279" s="5" t="n"/>
       <c r="AF279" s="5" t="n"/>
-      <c r="AG279" s="5" t="n"/>
-      <c r="AH279" s="5" t="n"/>
-      <c r="AI279" s="5" t="n"/>
-      <c r="AJ279" s="5" t="n"/>
-      <c r="AK279" s="5" t="n"/>
-      <c r="AL279" s="5" t="n"/>
-      <c r="AM279" s="5" t="n"/>
+      <c r="AG279" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-iii-1-2-ward.md; tablet's 'forced back 4-5 P.M.' is a UNION early-tablet exemplar (ED-58 candidate)</t>
+        </is>
+      </c>
+      <c r="AH279" s="5" t="inlineStr">
+        <is>
+          <t>Ward's bde (20IN/3ME/4ME/86NY/124NY/99PA/1-2USSS); Wheeler (20IN) k, Van Horne Ellis (124NY) k (monument check point), Walker (4ME) w</t>
+        </is>
+      </c>
+      <c r="AI279" s="5" t="inlineStr">
+        <is>
+          <t>~1,500 effectives PRIMARY (Ward) - loss 781 = 52%, worst Union brigade ratio on the southern field</t>
+        </is>
+      </c>
+      <c r="AJ279" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet] Houck's Ridge line, left on the rocky eminence; tablet (3764,2670) OSM 19.7m; [E drawn j2-03] Ward's Brig + 86NY/124NY/99P bars (3841-3856,2665-2795)</t>
+        </is>
+      </c>
+      <c r="AK279" s="5" t="inlineStr">
+        <is>
+          <t>[D duration] 90-min oscillating stone-wall fight - TWO-SIDED agreement with the 48th AL's hour-and-a-half; [A vs CA-J2A-5] forced off as the Den fell</t>
+        </is>
+      </c>
+      <c r="AL279" s="5" t="inlineStr">
+        <is>
+          <t>[D] held-fire-to-200yd volley discipline record; 'nearly two hours' front</t>
+        </is>
+      </c>
+      <c r="AM279" s="5" t="inlineStr">
+        <is>
+          <t>return 781 adopted (report 'nearly 800' carried, ED-52); 4th ME row column-noise flagged (144-class); ~all July 2</t>
+        </is>
+      </c>
       <c r="AN279" s="5" t="n"/>
-      <c r="AO279" s="5" t="n"/>
+      <c r="AO279" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
@@ -32709,20 +32925,56 @@
           <t>reg-us-ii-1-4</t>
         </is>
       </c>
-      <c r="AB282" s="5" t="n"/>
+      <c r="AB282" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC282" s="5" t="n"/>
       <c r="AD282" s="5" t="n"/>
       <c r="AE282" s="5" t="n"/>
       <c r="AF282" s="5" t="n"/>
-      <c r="AG282" s="5" t="n"/>
-      <c r="AH282" s="5" t="n"/>
-      <c r="AI282" s="5" t="n"/>
-      <c r="AJ282" s="5" t="n"/>
-      <c r="AK282" s="5" t="n"/>
-      <c r="AL282" s="5" t="n"/>
-      <c r="AM282" s="5" t="n"/>
+      <c r="AG282" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-1-4-brooke.md</t>
+        </is>
+      </c>
+      <c r="AH282" s="5" t="inlineStr">
+        <is>
+          <t>Brooke's bde (27CT/2DE/64NY/53PA/145PA); Brooke 'severely bruised' (register w); Merwin (27CT) k</t>
+        </is>
+      </c>
+      <c r="AI282" s="5" t="inlineStr">
+        <is>
+          <t>no primary (negative); ~850 compilation hop-flagged; return 389 = ~46% - proportionally heaviest in the division</t>
+        </is>
+      </c>
+      <c r="AJ282" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J2A-8 +20-30min] FARTHEST ADVANCE tablet ON the Rose-ravine crest (3403,2913, OSM delta 56m flagged); [E drawn j2-04] CALDWELL'S DIV/Brooke's Brig labels at the apex (3487-3503,3230-3274)</t>
+        </is>
+      </c>
+      <c r="AK282" s="5" t="inlineStr">
+        <is>
+          <t>[D] passage-of-lines thru Cross; [B] 500m contested sweep 12-20 min; [D first-person] flanks-turned withdrawal 'unless I retired all would be killed or captured'</t>
+        </is>
+      </c>
+      <c r="AL282" s="5" t="inlineStr">
+        <is>
+          <t>[D] continuous fire fight; unsupported at the crest (negative-evidence class on support)</t>
+        </is>
+      </c>
+      <c r="AM282" s="5" t="inlineStr">
+        <is>
+          <t>return 389 (2DE 84, 64NY 98, 53PA 80, 145PA 90, 27CT 37); split: waves 3-4 carry ~all (deepest position = longest exposure)</t>
+        </is>
+      </c>
       <c r="AN282" s="5" t="n"/>
-      <c r="AO282" s="5" t="n"/>
+      <c r="AO282" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
@@ -34517,20 +34769,56 @@
           <t>reg-us-ii-1-3</t>
         </is>
       </c>
-      <c r="AB296" s="5" t="n"/>
+      <c r="AB296" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC296" s="5" t="n"/>
       <c r="AD296" s="5" t="n"/>
       <c r="AE296" s="5" t="n"/>
       <c r="AF296" s="5" t="n"/>
-      <c r="AG296" s="5" t="n"/>
-      <c r="AH296" s="5" t="n"/>
-      <c r="AI296" s="5" t="n"/>
-      <c r="AJ296" s="5" t="n"/>
-      <c r="AK296" s="5" t="n"/>
-      <c r="AL296" s="5" t="n"/>
-      <c r="AM296" s="5" t="n"/>
+      <c r="AG296" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-1-3-zook.md</t>
+        </is>
+      </c>
+      <c r="AH296" s="5" t="inlineStr">
+        <is>
+          <t>Zook's bde (52NY/57NY/66NY/140PA); Zook mw at the advance's start (statue on Wheatfield Rd = check point) -&gt; Fraser; Col. Roberts (140PA) k</t>
+        </is>
+      </c>
+      <c r="AI296" s="5" t="inlineStr">
+        <is>
+          <t>no primary (negative); ~975 compilation hop-flagged</t>
+        </is>
+      </c>
+      <c r="AJ296" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J2A-8] 'most advanced position on the crest of a small hill' (stony hill N crest); tablet (3576,3138) OSM delta 54m FLAGGED</t>
+        </is>
+      </c>
+      <c r="AK296" s="5" t="inlineStr">
+        <is>
+          <t>[D] committed right prong; stated line-order 140PA-66NY-52NY-57NY (the batch's only one); retreat when 'fresh troops' flanked both wings (= Wofford axis, both-sided)</t>
+        </is>
+      </c>
+      <c r="AL296" s="5" t="inlineStr">
+        <is>
+          <t>[D] wave-3 crest fight 18:15-18:45</t>
+        </is>
+      </c>
+      <c r="AM296" s="5" t="inlineStr">
+        <is>
+          <t>return 358 (140th PA 241 = 67% of brigade loss - the right-flank/Wofford-axis intensity shape); no report total (negative)</t>
+        </is>
+      </c>
       <c r="AN296" s="5" t="n"/>
-      <c r="AO296" s="5" t="n"/>
+      <c r="AO296" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
@@ -35184,7 +35472,7 @@
       <c r="AF301" s="5" t="n"/>
       <c r="AG301" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-ii-2-1-harrow.md; division-sum gap 3,580 vs 3,773 recorded; pass-5: July 2 evening counterattack leg both-sided (1st MN bracketed after CA-J2A-9, before sunset ED-31)</t>
+          <t>Dossier: reconstruction/dossiers/us-ii-2-1-harrow.md; division-sum gap 3,580 vs 3,773 recorded; pass-5: July 2 evening counterattack leg both-sided (1st MN bracketed after CA-J2A-9, before sunset ED-31); 1st MN regiment-grain upgrade pass 6</t>
         </is>
       </c>
       <c r="AH301" s="5" t="inlineStr">
@@ -35204,7 +35492,7 @@
       </c>
       <c r="AK301" s="5" t="inlineStr">
         <is>
-          <t>[C Jul 2] 15MA+82NY to Emmitsburg Rd + retire; [D] 1MN charge; [A vs CA-J3A-9] incline-right to the Copse [B: 2-5 min]</t>
+          <t>[C Jul 2] 15MA+82NY to Emmitsburg Rd + retire; [D] 1MN charge; [A vs CA-J3A-9] incline-right to the Copse [B: 2-5 min]; PASS-6: the 1st MN moment closed BOTH-SIDED at regiment grain (Coates primary + Wilcox p. 618 receiving side + j2-04 drawn pair; monument 232-of-330 ledger vs return 224, ED-52)</t>
         </is>
       </c>
       <c r="AL301" s="5" t="inlineStr">
@@ -35457,20 +35745,56 @@
           <t>reg-us-ii-1-2</t>
         </is>
       </c>
-      <c r="AB303" s="5" t="n"/>
+      <c r="AB303" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC303" s="5" t="n"/>
       <c r="AD303" s="5" t="n"/>
       <c r="AE303" s="5" t="n"/>
       <c r="AF303" s="5" t="n"/>
-      <c r="AG303" s="5" t="n"/>
-      <c r="AH303" s="5" t="n"/>
-      <c r="AI303" s="5" t="n"/>
-      <c r="AJ303" s="5" t="n"/>
-      <c r="AK303" s="5" t="n"/>
-      <c r="AL303" s="5" t="n"/>
-      <c r="AM303" s="5" t="n"/>
+      <c r="AG303" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-1-2-kelly.md</t>
+        </is>
+      </c>
+      <c r="AH303" s="5" t="inlineStr">
+        <is>
+          <t>Irish Bde (28MA/63NY/69NY/88NY/116PA); Kelly unwounded. Tablet NAMES its opponent (G.T. Anderson's bde) - tablet-layer both-siding</t>
+        </is>
+      </c>
+      <c r="AI303" s="5" t="inlineStr">
+        <is>
+          <t>530 into action PRIMARY (Kelly)</t>
+        </is>
+      </c>
+      <c r="AJ303" s="5" t="inlineStr">
+        <is>
+          <t>[A vs CA-J2A-8] stony hill ('very large rocks'); tablet (3526,3160) + Celtic cross (3574,3111)</t>
+        </is>
+      </c>
+      <c r="AK303" s="5" t="inlineStr">
+        <is>
+          <t>[C +70] 'about 5 p.m.' move; [B] wheat+wood advance 10-15 min; [D] withdrawal under flank pressure thru 'terrific fire'</t>
+        </is>
+      </c>
+      <c r="AL303" s="5" t="inlineStr">
+        <is>
+          <t>[D] 45-MINUTE duration primary for the stony-hill fight; prisoners taken</t>
+        </is>
+      </c>
+      <c r="AM303" s="5" t="inlineStr">
+        <is>
+          <t>return 198 adopted vs report 202 carried (ED-52 exemplar); 28th MA carries the missing (35) in the withdrawal</t>
+        </is>
+      </c>
       <c r="AN303" s="5" t="n"/>
-      <c r="AO303" s="5" t="n"/>
+      <c r="AO303" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
@@ -36201,20 +36525,56 @@
           <t>reg-us-ii-1-1</t>
         </is>
       </c>
-      <c r="AB309" s="5" t="n"/>
+      <c r="AB309" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC309" s="5" t="n"/>
       <c r="AD309" s="5" t="n"/>
       <c r="AE309" s="5" t="n"/>
       <c r="AF309" s="5" t="n"/>
-      <c r="AG309" s="5" t="n"/>
-      <c r="AH309" s="5" t="n"/>
-      <c r="AI309" s="5" t="n"/>
-      <c r="AJ309" s="5" t="n"/>
-      <c r="AK309" s="5" t="n"/>
-      <c r="AL309" s="5" t="n"/>
-      <c r="AM309" s="5" t="n"/>
+      <c r="AG309" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-ii-1-1-cross.md</t>
+        </is>
+      </c>
+      <c r="AH309" s="5" t="inlineStr">
+        <is>
+          <t>Cross's bde (5NH/61NY/81PA/148PA); Cross mw 'early in this engagement' wave-3 opening ~18:15-18:30 -&gt; McKeen. 5th NH monument = fall-vicinity check point</t>
+        </is>
+      </c>
+      <c r="AI309" s="5" t="inlineStr">
+        <is>
+          <t>780 muskets PRIMARY (McKeen) - the batch's cleanest strength+loss pairing</t>
+        </is>
+      </c>
+      <c r="AJ309" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet] II Corps line 10:00; [A vs CA-J2A-8] stone wall E of Wheatfield (tablet (3865,2994), OSM xcheck 15m); [D] farthest = wheat's far end +400yd; [E drawn j2-04] 'Cross Brig' bar (3862,3088)</t>
+        </is>
+      </c>
+      <c r="AK309" s="5" t="inlineStr">
+        <is>
+          <t>[A] division move ~18:00 (stated '5 p.m.' class, +60-70 early); [B] 400yd wheat advance 8-15 min; [D] Brooke passage-of-lines relief; withdrawal with division</t>
+        </is>
+      </c>
+      <c r="AL309" s="5" t="inlineStr">
+        <is>
+          <t>[D] wave-3 assault fire; ammunition exhaustion = relief trigger; July 3 breastworks, not assaulted</t>
+        </is>
+      </c>
+      <c r="AM309" s="5" t="inlineStr">
+        <is>
+          <t>report=return EXACT 330 (59/259/12 stated vs 57/260/13 block; composition drift carried); split: wave 3 dominant, Cross pins the spike's front edge</t>
+        </is>
+      </c>
       <c r="AN309" s="5" t="n"/>
-      <c r="AO309" s="5" t="n"/>
+      <c r="AO309" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
@@ -37549,20 +37909,56 @@
           <t>reg-us-v-1-2</t>
         </is>
       </c>
-      <c r="AB319" s="5" t="n"/>
+      <c r="AB319" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 twice-committed)</t>
+        </is>
+      </c>
       <c r="AC319" s="5" t="n"/>
       <c r="AD319" s="5" t="n"/>
       <c r="AE319" s="5" t="n"/>
       <c r="AF319" s="5" t="n"/>
-      <c r="AG319" s="5" t="n"/>
-      <c r="AH319" s="5" t="n"/>
-      <c r="AI319" s="5" t="n"/>
-      <c r="AJ319" s="5" t="n"/>
-      <c r="AK319" s="5" t="n"/>
-      <c r="AL319" s="5" t="n"/>
-      <c r="AM319" s="5" t="n"/>
+      <c r="AG319" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-v-1-2-sweitzer.md</t>
+        </is>
+      </c>
+      <c r="AH319" s="5" t="inlineStr">
+        <is>
+          <t>Sweitzer's bde (9MA detached/32MA/4MI/62PA); Jeffords (4MI) mw with the colors at the fence (monument check point); Lowry (62PA) k</t>
+        </is>
+      </c>
+      <c r="AI319" s="5" t="inlineStr">
+        <is>
+          <t>no primary (negative); ~1,010 incl. detached 9th MA (~420) - two-scope range carried</t>
+        </is>
+      </c>
+      <c r="AJ319" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet] first position woods at Wheatfield W (tablet (3670,2996) OSM-primary; j2-03 bar (3514,3077)); [A vs CA-J2A-8] SECOND position = the stone fence; j2-04 draws 'Sweitzer's Brigade' ON the fence (3706,2988) = 40m-class agreement with the 4th MI monument (3678,3012)</t>
+        </is>
+      </c>
+      <c r="AK319" s="5" t="inlineStr">
+        <is>
+          <t>[D] conditional first withdrawal (Prescott exchange); [D trigger] THE SECOND ADVANCE at Caldwell's personal request (both-command-sided); [D] caught-in-rear crisis + fighting extraction</t>
+        </is>
+      </c>
+      <c r="AL319" s="5" t="inlineStr">
+        <is>
+          <t>[D] the fence fight front-and-rear ~18:45-19:10; friendly-fire misread moment (smoke record)</t>
+        </is>
+      </c>
+      <c r="AM319" s="5" t="inlineStr">
+        <is>
+          <t>return 427 (4MI 165, 62PA 175; 121 c/m concentrate in the cut-off pair - capture-pocket shape); no report total (negative)</t>
+        </is>
+      </c>
       <c r="AN319" s="5" t="n"/>
-      <c r="AO319" s="5" t="n"/>
+      <c r="AO319" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
@@ -37673,20 +38069,56 @@
           <t>reg-us-v-1-1</t>
         </is>
       </c>
-      <c r="AB320" s="5" t="n"/>
+      <c r="AB320" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC320" s="5" t="n"/>
       <c r="AD320" s="5" t="n"/>
       <c r="AE320" s="5" t="n"/>
       <c r="AF320" s="5" t="n"/>
-      <c r="AG320" s="5" t="n"/>
-      <c r="AH320" s="5" t="n"/>
-      <c r="AI320" s="5" t="n"/>
-      <c r="AJ320" s="5" t="n"/>
-      <c r="AK320" s="5" t="n"/>
-      <c r="AL320" s="5" t="n"/>
-      <c r="AM320" s="5" t="n"/>
+      <c r="AG320" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-v-1-1-tilton.md; subject of the de Trobriand accusation - ED-59 candidate</t>
+        </is>
+      </c>
+      <c r="AH320" s="5" t="inlineStr">
+        <is>
+          <t>Tilton's bde (18MA/22MA/1MI/118PA); Tilton unwounded</t>
+        </is>
+      </c>
+      <c r="AI320" s="5" t="inlineStr">
+        <is>
+          <t>654 into action (Barnes PRIMARY) vs 'only 474' post-fight (two-scope, flagged not averaged)</t>
+        </is>
+      </c>
+      <c r="AJ320" s="5" t="inlineStr">
+        <is>
+          <t>[C +75] stony hill woods S of Rose's house; tablet (3480,3138) OSM-primary; [E drawn j2-03] BARNES' DIV (3394,3301) + Tilton bar (3436,3204) pre-withdrawal; July 3 = LRT garrison relief (interlocks ED-54)</t>
+        </is>
+      </c>
+      <c r="AK320" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet] Baltimore Pike -&gt; Third Corps support after 16:00; [D first-person] withdrawal on personally-reconnoitered Rose-house-axis outflanking (the ED-59 causal core)</t>
+        </is>
+      </c>
+      <c r="AL320" s="5" t="inlineStr">
+        <is>
+          <t>[D] twice repulsed Kershaw's left (wave 2)</t>
+        </is>
+      </c>
+      <c r="AM320" s="5" t="inlineStr">
+        <is>
+          <t>return 125 adopted vs report 109 carried (ED-52); ~all in the wave-2 stand</t>
+        </is>
+      </c>
       <c r="AN320" s="5" t="n"/>
-      <c r="AO320" s="5" t="n"/>
+      <c r="AO320" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
@@ -37921,20 +38353,56 @@
           <t>reg-us-iii-1-3</t>
         </is>
       </c>
-      <c r="AB322" s="5" t="n"/>
+      <c r="AB322" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (July 2 mover)</t>
+        </is>
+      </c>
       <c r="AC322" s="5" t="n"/>
       <c r="AD322" s="5" t="n"/>
       <c r="AE322" s="5" t="n"/>
       <c r="AF322" s="5" t="n"/>
-      <c r="AG322" s="5" t="n"/>
-      <c r="AH322" s="5" t="n"/>
-      <c r="AI322" s="5" t="n"/>
-      <c r="AJ322" s="5" t="n"/>
-      <c r="AK322" s="5" t="n"/>
-      <c r="AL322" s="5" t="n"/>
-      <c r="AM322" s="5" t="n"/>
+      <c r="AG322" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-iii-1-3-detrobriand.md; carries the ED-59-candidate withdrawal accusation vs Tilton/Sweitzer</t>
+        </is>
+      </c>
+      <c r="AH322" s="5" t="inlineStr">
+        <is>
+          <t>de Trobriand's bde (17ME/3MI/5MI/40NY/110PA); Pierce (3MI) w-amp, Pulford (5MI) w, Jones (110PA) w</t>
+        </is>
+      </c>
+      <c r="AI322" s="5" t="inlineStr">
+        <is>
+          <t>no primary (negative); ~1,387 compilation hop-flagged</t>
+        </is>
+      </c>
+      <c r="AJ322" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet 'between 2 and 3 P.M.'] the apex-of-the-angle deployment; tablet (3659,3049) OSM delta 0.9m - the register's cleanest agreement; 17th ME wall (3633,2965); [E drawn j2-03] Winslow in the field NE (3734,3141), line bar (3604,2997)</t>
+        </is>
+      </c>
+      <c r="AK322" s="5" t="inlineStr">
+        <is>
+          <t>[D] contraction onto the ravine-wall line; [D trigger] 'our ammunition was just exhausted' when Caldwell relieved (wave-2/3 seam)</t>
+        </is>
+      </c>
+      <c r="AL322" s="5" t="inlineStr">
+        <is>
+          <t>[D] wave-1 defense vs Anderson (5th MI half-loss stand, both-sided with White's three advances)</t>
+        </is>
+      </c>
+      <c r="AM322" s="5" t="inlineStr">
+        <is>
+          <t>report=return EXACT 490 (40th NY's 150 tactically belongs to Ward's front - cross-charge noted); split: waves 1-2 dominate</t>
+        </is>
+      </c>
       <c r="AN322" s="5" t="n"/>
-      <c r="AO322" s="5" t="n"/>
+      <c r="AO322" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Audit d9: overlay +9 (113 units) + five pass-9 upgrade notes; master table regenerated (113 audited rows / 327 total)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -15905,20 +15905,56 @@
           <t>reg-csa-2c-rod-1</t>
         </is>
       </c>
-      <c r="AB140" s="5" t="n"/>
+      <c r="AB140" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC140" s="5" t="n"/>
       <c r="AD140" s="5" t="n"/>
       <c r="AE140" s="5" t="n"/>
       <c r="AF140" s="5" t="n"/>
-      <c r="AG140" s="5" t="n"/>
-      <c r="AH140" s="5" t="n"/>
-      <c r="AI140" s="5" t="n"/>
-      <c r="AJ140" s="5" t="n"/>
-      <c r="AK140" s="5" t="n"/>
-      <c r="AL140" s="5" t="n"/>
-      <c r="AM140" s="5" t="n"/>
+      <c r="AG140" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-2c-rod-1-daniel.md; 4 a.m. vs recap 5 a.m. intra-report pair carried</t>
+        </is>
+      </c>
+      <c r="AH140" s="5" t="inlineStr">
+        <is>
+          <t>Daniel's Bde, Rodes's Div (32/43/45/53 NC + 2nd NC Bn); Daniel throughout; Bond/Green w July 1 pins</t>
+        </is>
+      </c>
+      <c r="AI140" s="5" t="inlineStr">
+        <is>
+          <t>OPEN; July 1 cost 'nearly one-third' = July 3 at two-thirds-strength CLASS (his fraction, not a number)</t>
+        </is>
+      </c>
+      <c r="AJ140" s="5" t="inlineStr">
+        <is>
+          <t>[C] 1.30 a.m. off / 4 a.m. reported to Johnson; [D+drawn] j3-01 DANIEL (5754,5842) behind JONES (5721,5780); j3-02 (6035,5465) the left-flank move drawn; E Conf Ave tablet (formation-line semantics)</t>
+        </is>
+      </c>
+      <c r="AK140" s="5" t="inlineStr">
+        <is>
+          <t>[B] the 4-mile night march at ~0.7 m/s (physics-consistent); [D] into Jones's support; the costly staff-guided lateral leg; the Steuart co-charge</t>
+        </is>
+      </c>
+      <c r="AL140" s="5" t="inlineStr">
+        <is>
+          <t>THE ASSESSMENT PRIMARY ('could not have been carried by any force'); the co-charge both-sided (Daniel/Steuart/Kane); the holding phase to 15:00-16:00 + midnight skirmishers</t>
+        </is>
+      </c>
+      <c r="AM140" s="5" t="inlineStr">
+        <is>
+          <t>ANV return 916 (165/635/116) w/ regiment rows — the Second Corps' largest; July-1-dominant by his own fraction; no per-day numbers</t>
+        </is>
+      </c>
       <c r="AN140" s="5" t="n"/>
-      <c r="AO140" s="5" t="n"/>
+      <c r="AO140" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -16732,7 +16768,7 @@
       <c r="AF146" s="5" t="n"/>
       <c r="AG146" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/csa-2c-joh-4-jones.md; register commander note corrected (w July 2, not July 3)</t>
+          <t>Dossier: reconstruction/dossiers/csa-2c-joh-4-jones.md; register commander note corrected (w July 2, not July 3) | PASS 9: Daniel-supports-Dungan weld (the succession named by the supporting brigade); j3-01 drawn arrival pair.</t>
         </is>
       </c>
       <c r="AH146" s="5" t="inlineStr">
@@ -17816,7 +17852,7 @@
       <c r="AF153" s="5" t="n"/>
       <c r="AG153" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/csa-2c-joh-3-nicholls.md; the evening chain's first agreeing CSA clock (ED-62 core)</t>
+          <t>Dossier: reconstruction/dossiers/csa-2c-joh-3-nicholls.md; the evening chain's first agreeing CSA clock (ED-62 core) | PASS 9: morning-fire arc framed (program + seven hours + the Rodes wave on its left).</t>
         </is>
       </c>
       <c r="AH153" s="5" t="inlineStr">
@@ -17965,20 +18001,56 @@
           <t>reg-csa-2c-rod-5</t>
         </is>
       </c>
-      <c r="AB154" s="5" t="n"/>
+      <c r="AB154" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC154" s="5" t="n"/>
       <c r="AD154" s="5" t="n"/>
       <c r="AE154" s="5" t="n"/>
       <c r="AF154" s="5" t="n"/>
-      <c r="AG154" s="5" t="n"/>
-      <c r="AH154" s="5" t="n"/>
-      <c r="AI154" s="5" t="n"/>
-      <c r="AJ154" s="5" t="n"/>
-      <c r="AK154" s="5" t="n"/>
-      <c r="AL154" s="5" t="n"/>
-      <c r="AM154" s="5" t="n"/>
+      <c r="AG154" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-2c-rod-5-oneal.md; the skeleton's softest clock (wave 2) answered at executor grain</t>
+        </is>
+      </c>
+      <c r="AH154" s="5" t="inlineStr">
+        <is>
+          <t>O'Neal's (Rodes's old) Bde (3/5/6/12/26 AL); O'Neal (senior colonel, commission withheld); July 3 orders direct from Johnson</t>
+        </is>
+      </c>
+      <c r="AI154" s="5" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="AJ154" s="5" t="inlineStr">
+        <is>
+          <t>[C] 2 a.m. off / arrived at daylight; [D+drawn] j3-01 (6223,5804) NE arrival vs j3-02 (5721,5694) north-slope attack — the ~510 m drawn advance IS the 8 a.m. attack; E Conf Ave tablet</t>
+        </is>
+      </c>
+      <c r="AK154" s="5" t="inlineStr">
+        <is>
+          <t>[B] the same-route night march; [C 8 a.m.] the wave-2 attack (four named regiments); [D] fall back with the entire line -&gt; behind-the-hill hold till midnight</t>
+        </is>
+      </c>
+      <c r="AL154" s="5" t="inlineStr">
+        <is>
+          <t>THE CA-J3M-2 WAVE-2 EXECUTOR CLOCK ('did not actively engage the foe until 8 a.m.'); grape-range attestation; the three-hour murderous-fire hold</t>
+        </is>
+      </c>
+      <c r="AM154" s="5" t="inlineStr">
+        <is>
+          <t>ANV return 696 (73/430/193) w/ asterisked regimental counter-readings carried; July-1-heavy, July 3 in the 8-11 hold</t>
+        </is>
+      </c>
       <c r="AN154" s="5" t="n"/>
-      <c r="AO154" s="5" t="n"/>
+      <c r="AO154" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -18781,20 +18853,56 @@
           <t>reg-csa-2c-ear-2</t>
         </is>
       </c>
-      <c r="AB160" s="5" t="n"/>
+      <c r="AB160" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (command-note grain)</t>
+        </is>
+      </c>
       <c r="AC160" s="5" t="n"/>
       <c r="AD160" s="5" t="n"/>
       <c r="AE160" s="5" t="n"/>
       <c r="AF160" s="5" t="n"/>
-      <c r="AG160" s="5" t="n"/>
-      <c r="AH160" s="5" t="n"/>
-      <c r="AI160" s="5" t="n"/>
-      <c r="AJ160" s="5" t="n"/>
-      <c r="AK160" s="5" t="n"/>
-      <c r="AL160" s="5" t="n"/>
-      <c r="AM160" s="5" t="n"/>
+      <c r="AG160" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-2c-ear-2-smith.md; T2 ceiling accepted, not padded</t>
+        </is>
+      </c>
+      <c r="AH160" s="5" t="inlineStr">
+        <is>
+          <t>Smith's Bde, Early's Div (31/49/52 VA — three regiments); 'Extra Billy' Smith; Hoffman the later commander</t>
+        </is>
+      </c>
+      <c r="AI160" s="5" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="AJ160" s="5" t="inlineStr">
+        <is>
+          <t>[E] July 1-2 York-road flank guard (Early); [D+drawn] Johnson's extreme left near the creek (j3-01 SMITH VA (6324,5152); j3-02 (6107,5116)); E Conf Ave tablet</t>
+        </is>
+      </c>
+      <c r="AK160" s="5" t="inlineStr">
+        <is>
+          <t>[D] the by-daylight night detachment march (Early's order primary; no own clock)</t>
+        </is>
+      </c>
+      <c r="AL160" s="5" t="inlineStr">
+        <is>
+          <t>'his three regiments were engaged on the 3rd on the extreme left, under General Johnson's directions' (Early) — vs JOHNSON'S SILENCE (his July 3 paragraph names only Daniel/O'Neal): the echelon-asymmetry record; Hoffman report referral UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="AM160" s="5" t="inlineStr">
+        <is>
+          <t>not consulted this pass (Early-division return block holds the row; open at this grain)</t>
+        </is>
+      </c>
       <c r="AN160" s="5" t="n"/>
-      <c r="AO160" s="5" t="n"/>
+      <c r="AO160" s="5" t="inlineStr">
+        <is>
+          <t>T2 (command-note grain)</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -18916,7 +19024,7 @@
       <c r="AF161" s="5" t="n"/>
       <c r="AG161" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/csa-2c-joh-1-steuart.md; action clocks +75 profiled vs his own 11 p.m. ~0 - in-division heterogeneity documented</t>
+          <t>Dossier: reconstruction/dossiers/csa-2c-joh-1-steuart.md; action clocks +75 profiled vs his own 11 p.m. ~0 - in-division heterogeneity documented | PASS 9: the 10 a.m. charge BOTH-SIDED at three grains (Daniel co-charge / Kane 10.30 receiving / Colgrove prisoner ID).</t>
         </is>
       </c>
       <c r="AH161" s="5" t="inlineStr">
@@ -19076,7 +19184,7 @@
       <c r="AF162" s="5" t="n"/>
       <c r="AG162" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/csa-2c-joh-2-walker.md; Gregg cavalry companion flagged for the cavalry batch</t>
+          <t>Dossier: reconstruction/dossiers/csa-2c-joh-2-walker.md; Gregg cavalry companion flagged for the cavalry batch | PASS 9: wave-1 composition pin (Johnson's Stonewall-up verbatim); drawn-static WALKER labels across j3-01/j3-02.</t>
         </is>
       </c>
       <c r="AH162" s="5" t="inlineStr">
@@ -21081,20 +21189,56 @@
           <t>reg-us-xii-arty</t>
         </is>
       </c>
-      <c r="AB180" s="5" t="n"/>
+      <c r="AB180" s="5" t="inlineStr">
+        <is>
+          <t>not-yet-cast (group grain)</t>
+        </is>
+      </c>
       <c r="AC180" s="5" t="n"/>
       <c r="AD180" s="5" t="n"/>
       <c r="AE180" s="5" t="n"/>
       <c r="AF180" s="5" t="n"/>
-      <c r="AG180" s="5" t="n"/>
-      <c r="AH180" s="5" t="n"/>
-      <c r="AI180" s="5" t="n"/>
-      <c r="AJ180" s="5" t="n"/>
-      <c r="AK180" s="5" t="n"/>
-      <c r="AL180" s="5" t="n"/>
-      <c r="AM180" s="5" t="n"/>
+      <c r="AG180" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-xii-arty-muhlenberg.md; report-vs-tablet conflicts (20-vs-26 guns; 10:00-vs-10:30 end) carried on CA-J3M-1/4</t>
+        </is>
+      </c>
+      <c r="AH180" s="5" t="inlineStr">
+        <is>
+          <t>Muhlenberg (1st Lt, 4th US) commanding; F 4th US (Rugg), K 5th US (Kinzie), Knap's E PA (Atwell), M 1st NY (Winegar)</t>
+        </is>
+      </c>
+      <c r="AI180" s="5" t="inlineStr">
+        <is>
+          <t>20 guns in the July 3 program BY THE AUTHOR (10 rifles + 10 Napoleons) vs tablet 26 — Rigby A 1st MD reconciliation flagged, not adopted; personnel OPEN</t>
+        </is>
+      </c>
+      <c r="AJ180" s="5" t="inlineStr">
+        <is>
+          <t>[E] the pike/Powers/McAllister's program arc 600-800 yards out (four program-ground markers registered incl. Rigby); July 2 park negative (F + K 'remained in park')</t>
+        </is>
+      </c>
+      <c r="AK180" s="5" t="inlineStr">
+        <is>
+          <t>[C ~17:00 July 2] the Geary/Van Reed forward sections; otherwise attested-static</t>
+        </is>
+      </c>
+      <c r="AL180" s="5" t="inlineStr">
+        <is>
+          <t>THE CA-J3M-1 AUTHOR PRIMARY: 4.30 open / 15 min without intermission / 5.30 resume / 'until 10 a.m.'; Williams verbatim-class corroboration; the July 2 eight-gun thirty-minute Latimer duel received; NO rounds figures (verified negative)</t>
+        </is>
+      </c>
+      <c r="AM180" s="5" t="inlineStr">
+        <is>
+          <t>9 w aggregate (return p. 185) + the July 2 section losses itemized; July-2-weighted</t>
+        </is>
+      </c>
       <c r="AN180" s="5" t="n"/>
-      <c r="AO180" s="5" t="n"/>
+      <c r="AO180" s="5" t="inlineStr">
+        <is>
+          <t>T3 (group grain)</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -34333,20 +34477,56 @@
           <t>reg-us-xii-2-1</t>
         </is>
       </c>
-      <c r="AB289" s="5" t="n"/>
+      <c r="AB289" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC289" s="5" t="n"/>
       <c r="AD289" s="5" t="n"/>
       <c r="AE289" s="5" t="n"/>
       <c r="AF289" s="5" t="n"/>
-      <c r="AG289" s="5" t="n"/>
-      <c r="AH289" s="5" t="n"/>
-      <c r="AI289" s="5" t="n"/>
-      <c r="AJ289" s="5" t="n"/>
-      <c r="AK289" s="5" t="n"/>
-      <c r="AL289" s="5" t="n"/>
-      <c r="AM289" s="5" t="n"/>
+      <c r="AG289" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-xii-2-1-candy.md</t>
+        </is>
+      </c>
+      <c r="AH289" s="5" t="inlineStr">
+        <is>
+          <t>1st Bde 2nd Div XII (5/7/29/66 OH, 28/147 PA); Candy throughout</t>
+        </is>
+      </c>
+      <c r="AI289" s="5" t="inlineStr">
+        <is>
+          <t>OPEN (no primary; no hop)</t>
+        </is>
+      </c>
+      <c r="AJ289" s="5" t="inlineStr">
+        <is>
+          <t>[E] reserve hollow (j3-01 CANDY'S BRIG label (5620,5114); HQ pin w/ OSM duplicates flagged); [D] the 66th OH outside-the-works ground (mon-66oh, non-works-line semantics)</t>
+        </is>
+      </c>
+      <c r="AK289" s="5" t="inlineStr">
+        <is>
+          <t>[C 19:00-&gt;00:30] the wrong-road round trip ('supposed to be General Hancock's'; 28th PA 12.30 a.m. forward); [D] the 66th OH over-the-crest deployment; rotation legs</t>
+        </is>
+      </c>
+      <c r="AL289" s="5" t="inlineStr">
+        <is>
+          <t>the confusion confession; the 3.45 a.m. pre-program clock (profiled [-45,15]); the 66th OH enfilade; rotation service</t>
+        </is>
+      </c>
+      <c r="AM289" s="5" t="inlineStr">
+        <is>
+          <t>return brigade total 139 (division arithmetic closes 540=303+139+98); regiment rows the cheap residual</t>
+        </is>
+      </c>
       <c r="AN289" s="5" t="n"/>
-      <c r="AO289" s="5" t="n"/>
+      <c r="AO289" s="5" t="inlineStr">
+        <is>
+          <t>T3 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
@@ -34777,20 +34957,56 @@
           <t>reg-us-xii-1-3</t>
         </is>
       </c>
-      <c r="AB292" s="5" t="n"/>
+      <c r="AB292" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (the CA-J3M-3 executor)</t>
+        </is>
+      </c>
       <c r="AC292" s="5" t="n"/>
       <c r="AD292" s="5" t="n"/>
       <c r="AE292" s="5" t="n"/>
       <c r="AF292" s="5" t="n"/>
-      <c r="AG292" s="5" t="n"/>
-      <c r="AH292" s="5" t="n"/>
-      <c r="AI292" s="5" t="n"/>
-      <c r="AJ292" s="5" t="n"/>
-      <c r="AK292" s="5" t="n"/>
-      <c r="AL292" s="5" t="n"/>
-      <c r="AM292" s="5" t="n"/>
+      <c r="AG292" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-xii-1-3-colgrove.md; THE SPANGLER'S MEADOW TWO-POLE record -&gt; ED-64 candidate (5.30/6 a.m. executor pole vs Ruger ~10 a.m. + Bachelder 8-11 sheet)</t>
+        </is>
+      </c>
+      <c r="AH292" s="5" t="inlineStr">
+        <is>
+          <t>3rd Bde 1st Div XII (27 IN/2 MA/13 NJ/107 NY/3 WI); Ruger to div morning July 2, Colgrove up; MUDGE k in the charge (Morse succession primary)</t>
+        </is>
+      </c>
+      <c r="AI292" s="5" t="inlineStr">
+        <is>
+          <t>27th IN 339 PRIMARY (=monument exact); 2nd MA 294 EM + 22 officers (Cogswell + monument); other three OPEN</t>
+        </is>
+      </c>
+      <c r="AJ292" s="5" t="inlineStr">
+        <is>
+          <t>[A] the meadow's south works (mon-2ma START-line semantics; mon-27in; HQ pin); [D] the 27th IN advance marker (6115.9,4964.0) = 79 m north of main (the '90 yards'); j3-01 position vs j3-02 charge drawn states 59/69 m from the stones</t>
+        </is>
+      </c>
+      <c r="AK292" s="5" t="inlineStr">
+        <is>
+          <t>[C] the July 2 left-wing round trip (back 'about 10 p.m.'); [B] the 100-yard double-quick charge + the 27th's double-distance oblique; [C ~17:00] 13 NJ/107 NY to Gregg</t>
+        </is>
+      </c>
+      <c r="AL292" s="5" t="inlineStr">
+        <is>
+          <t>THE ORDER-CORRUPTION PAIR ('The general directs that you advance your line immediately' via Lt. Snow vs Ruger's skirmishers-first intent); the no-skirmish decision primary; charge-repulse-counter-repulse; ~100 prisoners</t>
+        </is>
+      </c>
+      <c r="AM292" s="5" t="inlineStr">
+        <is>
+          <t>return 279 (27 IN 110 / 2 MA 136 = 88% of it); Fesler's charge-vs-works itemized split (98 of 111 in the charge); the 110/111/112 and 130/135/136 component clusters ALL carried</t>
+        </is>
+      </c>
       <c r="AN292" s="5" t="n"/>
-      <c r="AO292" s="5" t="n"/>
+      <c r="AO292" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
@@ -36296,7 +36512,7 @@
       <c r="AF303" s="5" t="n"/>
       <c r="AG303" s="5" t="inlineStr">
         <is>
-          <t>Dossier: reconstruction/dossiers/us-xii-2-3-greene.md; CA-J2E-1 primary (6.30) + E-2 both-sided (w/ Nicholls 19:00) -&gt; ED-62 evidence</t>
+          <t>Dossier: reconstruction/dossiers/us-xii-2-3-greene.md; CA-J2E-1 primary (6.30) + E-2 both-sided (w/ Nicholls 19:00) -&gt; ED-62 evidence | PASS 9: July 3 morning frame hardened around the spine (Kane 3.30/seven-hours/10.30; Muhlenberg program; the Rodes wave opposite).</t>
         </is>
       </c>
       <c r="AH303" s="5" t="inlineStr">
@@ -36765,20 +36981,56 @@
           <t>reg-us-xii-2-2</t>
         </is>
       </c>
-      <c r="AB306" s="5" t="n"/>
+      <c r="AB306" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC306" s="5" t="n"/>
       <c r="AD306" s="5" t="n"/>
       <c r="AE306" s="5" t="n"/>
       <c r="AF306" s="5" t="n"/>
-      <c r="AG306" s="5" t="n"/>
-      <c r="AH306" s="5" t="n"/>
-      <c r="AI306" s="5" t="n"/>
-      <c r="AJ306" s="5" t="n"/>
-      <c r="AK306" s="5" t="n"/>
-      <c r="AL306" s="5" t="n"/>
-      <c r="AM306" s="5" t="n"/>
+      <c r="AG306" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-xii-2-2-kane.md; the morning chain's cleanest receiving-side ladder</t>
+        </is>
+      </c>
+      <c r="AH306" s="5" t="inlineStr">
+        <is>
+          <t>2nd Bde 2nd Div XII (29/109/111 PA); the Cobham-Kane-Cobham command passage (ambulance arrival 6 a.m. July 2)</t>
+        </is>
+      </c>
+      <c r="AI306" s="5" t="inlineStr">
+        <is>
+          <t>PRIMARY: 652 in action (Kane p. 848)</t>
+        </is>
+      </c>
+      <c r="AJ306" s="5" t="inlineStr">
+        <is>
+          <t>[A] works between Greene's right and Candy (mon-109pa/111pa/29pa chain + HQ pin, OSM 'Huey' mislabel flagged); j2-04 vacated vs j3-02 returned KANE labels</t>
+        </is>
+      </c>
+      <c r="AK306" s="5" t="inlineStr">
+        <is>
+          <t>[D] the wrong-object march; [B ~1 mile dark + two fire contacts] the groping return past Greene's right</t>
+        </is>
+      </c>
+      <c r="AL306" s="5" t="inlineStr">
+        <is>
+          <t>the night-discovery primary ('thus discovering that the enemy had entire possession of our works'); July 3: 3.30 attack, 'Johnson's division led, followed by Rodes''; SEVEN HOURS 'until about 10.30' + column-of-regiments last effort</t>
+        </is>
+      </c>
+      <c r="AM306" s="5" t="inlineStr">
+        <is>
+          <t>Kane 96 vs Cobham 98 = return 98 (killed exact 23 at all three); July-3-weighted (absent July 2 evening)</t>
+        </is>
+      </c>
       <c r="AN306" s="5" t="n"/>
-      <c r="AO306" s="5" t="n"/>
+      <c r="AO306" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
@@ -37173,20 +37425,56 @@
           <t>reg-us-xii-1-2</t>
         </is>
       </c>
-      <c r="AB309" s="5" t="n"/>
+      <c r="AB309" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC309" s="5" t="n"/>
       <c r="AD309" s="5" t="n"/>
       <c r="AE309" s="5" t="n"/>
       <c r="AF309" s="5" t="n"/>
-      <c r="AG309" s="5" t="n"/>
-      <c r="AH309" s="5" t="n"/>
-      <c r="AI309" s="5" t="n"/>
-      <c r="AJ309" s="5" t="n"/>
-      <c r="AK309" s="5" t="n"/>
-      <c r="AL309" s="5" t="n"/>
-      <c r="AM309" s="5" t="n"/>
+      <c r="AG309" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-xii-1-2-lockwood.md</t>
+        </is>
+      </c>
+      <c r="AH309" s="5" t="inlineStr">
+        <is>
+          <t>2nd (unattached) Bde 1st Div XII (1 MD PHB/1 MD ES/150 NY); Lockwood senior-but-new; ED-61 command-grain claimant (pass 8)</t>
+        </is>
+      </c>
+      <c r="AI309" s="5" t="inlineStr">
+        <is>
+          <t>OPEN; two-regiment July 2 vs three-regiment July 3 composition fact</t>
+        </is>
+      </c>
+      <c r="AJ309" s="5" t="inlineStr">
+        <is>
+          <t>[C] 8 a.m. July 2 arrival; [D] the July 2 evening McGilvery-line ground; [E] July 3 behind the left (HQ + three regimentals registered; 1st MD PHB at the meadow's NW woods)</t>
+        </is>
+      </c>
+      <c r="AK309" s="5" t="inlineStr">
+        <is>
+          <t>[B] the 1-mile double-quick July 2 (Maulsby); [C ~06:00] the woods deployment order; [C ~14:00] the left-center round trip (Ruger's brigade-numbering slip flagged)</t>
+        </is>
+      </c>
+      <c r="AL309" s="5" t="inlineStr">
+        <is>
+          <t>battery support at the program's edge; the 1st MD PHB woods engagement (the ~06:00 flank congestion fact in ED-64's conflation analysis)</t>
+        </is>
+      </c>
+      <c r="AM309" s="5" t="inlineStr">
+        <is>
+          <t>return 174 (1st MD PHB 104 = the woods fight's weight); no per-day primary</t>
+        </is>
+      </c>
       <c r="AN309" s="5" t="n"/>
-      <c r="AO309" s="5" t="n"/>
+      <c r="AO309" s="5" t="inlineStr">
+        <is>
+          <t>T3 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
@@ -37617,20 +37905,56 @@
           <t>reg-us-xii-1-1</t>
         </is>
       </c>
-      <c r="AB312" s="5" t="n"/>
+      <c r="AB312" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC312" s="5" t="n"/>
       <c r="AD312" s="5" t="n"/>
       <c r="AE312" s="5" t="n"/>
       <c r="AF312" s="5" t="n"/>
-      <c r="AG312" s="5" t="n"/>
-      <c r="AH312" s="5" t="n"/>
-      <c r="AI312" s="5" t="n"/>
-      <c r="AJ312" s="5" t="n"/>
-      <c r="AK312" s="5" t="n"/>
-      <c r="AL312" s="5" t="n"/>
-      <c r="AM312" s="5" t="n"/>
+      <c r="AG312" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-xii-1-1-mcdougall.md; the July 2/3 seam's Union-decision record</t>
+        </is>
+      </c>
+      <c r="AH312" s="5" t="inlineStr">
+        <is>
+          <t>1st Bde 1st Div XII (5 CT/20 CT/3 MD/123 NY/145 NY/46 PA); McDougall throughout</t>
+        </is>
+      </c>
+      <c r="AI312" s="5" t="inlineStr">
+        <is>
+          <t>OPEN (no primary; no hop)</t>
+        </is>
+      </c>
+      <c r="AJ312" s="5" t="inlineStr">
+        <is>
+          <t>[E] lower-hill works chain (HQ + five regimentals registered; 5th CT node NEGATIVE); j2-04 vacated label; j3-01 rally-ground read (5991,4530)</t>
+        </is>
+      </c>
+      <c r="AK312" s="5" t="inlineStr">
+        <is>
+          <t>[D] the 1.5-mile round trip; THE STOPPED NIGHT APPROACH (skirmisher discovery, no night assault, arms-down); [D] the 123rd NY works reoccupation (CA-J3M-4 executor)</t>
+        </is>
+      </c>
+      <c r="AL312" s="5" t="inlineStr">
+        <is>
+          <t>the 20th CT woods fight under friendly overhead artillery (FRIENDLY-FIRE record); July 4 reconnaissance detachment</t>
+        </is>
+      </c>
+      <c r="AM312" s="5" t="inlineStr">
+        <is>
+          <t>return 80 (20th CT 28 the woods cost); friendly-fire component unnumbered (flagged)</t>
+        </is>
+      </c>
       <c r="AN312" s="5" t="n"/>
-      <c r="AO312" s="5" t="n"/>
+      <c r="AO312" s="5" t="inlineStr">
+        <is>
+          <t>T3 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Wave A1: bundle metadata recompile (inputs.battle hash; payload byte-identical, ED-21 stagingSeed pin held d470c469) + master table regenerated (16 rows' build metrics)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -8130,29 +8130,29 @@
         <v>432</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>432</v>
+        <v>418</v>
       </c>
       <c r="H80" s="3">
         <f>IF(F80=0,0,1-G80/F80)</f>
         <v/>
       </c>
       <c r="I80" s="2" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M80" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O80" s="2" t="n">
         <v>0</v>
@@ -8191,7 +8191,7 @@
       </c>
       <c r="X80" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T0</t>
         </is>
       </c>
       <c r="Y80" s="2" t="inlineStr">
@@ -8287,32 +8287,32 @@
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>240</v>
+        <v>338</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>240</v>
+        <v>293</v>
       </c>
       <c r="H81" s="3">
         <f>IF(F81=0,0,1-G81/F81)</f>
         <v/>
       </c>
       <c r="I81" s="2" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L81" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M81" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O81" s="2" t="n">
         <v>0</v>
@@ -8351,7 +8351,7 @@
       </c>
       <c r="X81" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T0</t>
         </is>
       </c>
       <c r="Y81" s="2" t="inlineStr">
@@ -9214,29 +9214,29 @@
         <v>480</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>480</v>
+        <v>433</v>
       </c>
       <c r="H87" s="3">
         <f>IF(F87=0,0,1-G87/F87)</f>
         <v/>
       </c>
       <c r="I87" s="2" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L87" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M87" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O87" s="2" t="n">
         <v>0</v>
@@ -9275,7 +9275,7 @@
       </c>
       <c r="X87" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T0</t>
         </is>
       </c>
       <c r="Y87" s="2" t="inlineStr">
@@ -17227,17 +17227,17 @@
         </is>
       </c>
       <c r="F149" s="2" t="n">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="G149" s="2" t="n">
-        <v>300</v>
+        <v>245</v>
       </c>
       <c r="H149" s="3">
         <f>IF(F149=0,0,1-G149/F149)</f>
         <v/>
       </c>
       <c r="I149" s="2" t="n">
-        <v>400</v>
+        <v>155</v>
       </c>
       <c r="J149" s="2" t="n">
         <v>6</v>
@@ -17255,10 +17255,10 @@
         <v>6</v>
       </c>
       <c r="O149" s="2" t="n">
-        <v>990.4</v>
+        <v>1448.8</v>
       </c>
       <c r="P149" s="2" t="n">
-        <v>170</v>
+        <v>264.8</v>
       </c>
       <c r="Q149" s="2" t="inlineStr">
         <is>
@@ -19483,26 +19483,26 @@
         </is>
       </c>
       <c r="F164" s="2" t="n">
-        <v>1777</v>
+        <v>1200</v>
       </c>
       <c r="G164" s="2" t="n">
-        <v>1577</v>
+        <v>996</v>
       </c>
       <c r="H164" s="3">
         <f>IF(F164=0,0,1-G164/F164)</f>
         <v/>
       </c>
       <c r="I164" s="2" t="n">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="J164" s="2" t="n">
         <v>6</v>
       </c>
       <c r="K164" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L164" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M164" s="2" t="n">
         <v>0</v>
@@ -19511,10 +19511,10 @@
         <v>6</v>
       </c>
       <c r="O164" s="2" t="n">
-        <v>1011</v>
+        <v>1619</v>
       </c>
       <c r="P164" s="2" t="n">
-        <v>170.1</v>
+        <v>270.7</v>
       </c>
       <c r="Q164" s="2" t="inlineStr">
         <is>
@@ -24063,7 +24063,7 @@
         </is>
       </c>
       <c r="S209" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T209" s="2" t="n">
         <v>0</v>
@@ -24998,14 +24998,14 @@
         <v>114</v>
       </c>
       <c r="G216" s="2" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H216" s="3">
         <f>IF(F216=0,0,1-G216/F216)</f>
         <v/>
       </c>
       <c r="I216" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J216" s="2" t="n">
         <v>4</v>
@@ -25566,29 +25566,29 @@
         <v>103</v>
       </c>
       <c r="G220" s="2" t="n">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="H220" s="3">
         <f>IF(F220=0,0,1-G220/F220)</f>
         <v/>
       </c>
       <c r="I220" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J220" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K220" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L220" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M220" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N220" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O220" s="2" t="n">
         <v>0</v>
@@ -25607,7 +25607,7 @@
         </is>
       </c>
       <c r="S220" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T220" s="2" t="n">
         <v>0</v>
@@ -25938,29 +25938,29 @@
         <v>149</v>
       </c>
       <c r="G223" s="2" t="n">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="H223" s="3">
         <f>IF(F223=0,0,1-G223/F223)</f>
         <v/>
       </c>
       <c r="I223" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J223" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K223" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L223" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M223" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N223" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O223" s="2" t="n">
         <v>806.6</v>
@@ -25979,7 +25979,7 @@
         </is>
       </c>
       <c r="S223" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T223" s="2" t="n">
         <v>0</v>
@@ -26387,7 +26387,7 @@
         </is>
       </c>
       <c r="S226" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T226" s="2" t="n">
         <v>0</v>
@@ -27090,29 +27090,29 @@
         <v>116</v>
       </c>
       <c r="G232" s="2" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H232" s="3">
         <f>IF(F232=0,0,1-G232/F232)</f>
         <v/>
       </c>
       <c r="I232" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J232" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K232" s="2" t="n">
         <v>2</v>
       </c>
       <c r="L232" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M232" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N232" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O232" s="2" t="n">
         <v>1578.9</v>
@@ -27291,7 +27291,7 @@
         </is>
       </c>
       <c r="S233" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T233" s="2" t="n">
         <v>0</v>
@@ -28143,7 +28143,7 @@
         </is>
       </c>
       <c r="S239" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T239" s="2" t="n">
         <v>0</v>
@@ -28763,7 +28763,7 @@
         </is>
       </c>
       <c r="S244" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T244" s="2" t="n">
         <v>0</v>
@@ -33459,17 +33459,17 @@
         </is>
       </c>
       <c r="F282" s="2" t="n">
-        <v>209</v>
+        <v>164</v>
       </c>
       <c r="G282" s="2" t="n">
-        <v>170</v>
+        <v>118</v>
       </c>
       <c r="H282" s="3">
         <f>IF(F282=0,0,1-G282/F282)</f>
         <v/>
       </c>
       <c r="I282" s="2" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="J282" s="2" t="n">
         <v>3</v>
@@ -39472,10 +39472,10 @@
         <v>710</v>
       </c>
       <c r="J322" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K322" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L322" s="2" t="n">
         <v>3</v>
@@ -39484,13 +39484,13 @@
         <v>0</v>
       </c>
       <c r="N322" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O322" s="2" t="n">
-        <v>0</v>
+        <v>70.2</v>
       </c>
       <c r="P322" s="2" t="n">
-        <v>0</v>
+        <v>70.2</v>
       </c>
       <c r="Q322" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Audit d11: overlay +7 new (130 units) / 25 updated cells (the EC2 sweep — Rodes June-30 return primaries + B&M-repro hops both sides; the cell-closure notes); master table regenerated (329 rows, 130 audited T-levels); index pass-11 section; dossier cast-status lines corrected to in-build (all seven are July 3 build rows)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -14310,7 +14310,7 @@
       </c>
       <c r="AI130" s="5" t="inlineStr">
         <is>
-          <t>1,650 (ED-9, no primary); crossing party ~150 (T5)</t>
+          <t>1,650 (ED-9, no primary); crossing party ~150 (T5) ; p11 sweep: B&amp;M-repro 2,055 (hop) beside ED-9 1,650 - divergent, both carried, no primary</t>
         </is>
       </c>
       <c r="AJ130" s="5" t="inlineStr">
@@ -15126,7 +15126,7 @@
       </c>
       <c r="AI135" s="5" t="inlineStr">
         <is>
-          <t>1,575 (ED-9/stone-sentinels, no primary; negative - no morning report survives)</t>
+          <t>1,575 (ED-9/stone-sentinels, no primary; negative - no morning report survives) ; p11 sweep: B&amp;M-repro 1,634 (hop) beside ED-9 1,575</t>
         </is>
       </c>
       <c r="AJ135" s="5" t="inlineStr">
@@ -15606,7 +15606,7 @@
       </c>
       <c r="AI138" s="5" t="inlineStr">
         <is>
-          <t>tablet 'Present 1,598' (compilation, hop flagged); no primary</t>
+          <t>tablet 'Present 1,598' (compilation, hop flagged); no primary ; p11 sweep: B&amp;M-repro 1,620 (Barksdale; hop) beside tablet 1,598</t>
         </is>
       </c>
       <c r="AJ138" s="5" t="inlineStr">
@@ -15926,7 +15926,7 @@
       </c>
       <c r="AI140" s="5" t="inlineStr">
         <is>
-          <t>OPEN; July 1 cost 'nearly one-third' = July 3 at two-thirds-strength CLASS (his fraction, not a number)</t>
+          <t>OPEN; July 1 cost 'nearly one-third' = July 3 at two-thirds-strength CLASS (his fraction, not a number) ; p11: June-30 return PRIMARY 171+2,123=2,294 (p. 564) beside his 'about 2,200' report figure; B&amp;M-repro 2,162 (hop)</t>
         </is>
       </c>
       <c r="AJ140" s="5" t="inlineStr">
@@ -16065,20 +16065,56 @@
           <t>reg-csa-2c-rod-3</t>
         </is>
       </c>
-      <c r="AB141" s="5" t="n"/>
+      <c r="AB141" s="5" t="inlineStr">
+        <is>
+          <t>unauthored</t>
+        </is>
+      </c>
       <c r="AC141" s="5" t="n"/>
       <c r="AD141" s="5" t="n"/>
       <c r="AE141" s="5" t="n"/>
       <c r="AF141" s="5" t="n"/>
-      <c r="AG141" s="5" t="n"/>
-      <c r="AH141" s="5" t="n"/>
-      <c r="AI141" s="5" t="n"/>
-      <c r="AJ141" s="5" t="n"/>
-      <c r="AK141" s="5" t="n"/>
-      <c r="AL141" s="5" t="n"/>
-      <c r="AM141" s="5" t="n"/>
+      <c r="AG141" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-2c-rod-3-doles.md; CA-J1P-1/3 + CA-J2E context</t>
+        </is>
+      </c>
+      <c r="AH141" s="5" t="inlineStr">
+        <is>
+          <t>Doles throughout (the one uninjured Rodes brigade commander); Winn k + Lumpkin severely w (July 1)</t>
+        </is>
+      </c>
+      <c r="AI141" s="5" t="inlineStr">
+        <is>
+          <t>PRIMARY 'went into action with 131 officers and 1,238 enlisted men; total, 1,369' + June-30 return 128+1,275=1,403 (p. 564); B&amp;M-repro 1,323 (hop) carried</t>
+        </is>
+      </c>
+      <c r="AJ141" s="5" t="inlineStr">
+        <is>
+          <t>[C ~13:00] the left-of-division formation in the plain; the skirmisher hill (3.30 referent ambiguity recorded); the east-west street line July 1-2; [C ~20:00 Jul 2] within 100 yd of Cemetery Hill -&gt; the dirt road 300 yd back, held to 1 a.m. July 4</t>
+        </is>
+      </c>
+      <c r="AK141" s="5" t="inlineStr">
+        <is>
+          <t>[D] the left-flank moves vs the knoll; the Gordon-conjunction attack; the 157th NY front-change + plain pursuit; the failed college cut-off (pace-class negative); the July 2 evening column with Ramseur/Iverson</t>
+        </is>
+      </c>
+      <c r="AL141" s="5" t="inlineStr">
+        <is>
+          <t>The knoll rock-fence assault; THE 157th NY DESTRUCTION both-sided; THE FRIENDLY-FIRE APPENDIX (the two-gun brass battery at Rodes's HQ hill); July 2-4 heavy skirmishing</t>
+        </is>
+      </c>
+      <c r="AM141" s="5" t="inlineStr">
+        <is>
+          <t>Report=return EXACT 24/124/31 = 179 (regiment rows 45/49/17/68 both ledgers); July-1-dominant shape</t>
+        </is>
+      </c>
       <c r="AN141" s="5" t="n"/>
-      <c r="AO141" s="5" t="n"/>
+      <c r="AO141" s="5" t="inlineStr">
+        <is>
+          <t>T4 (full arc)</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -16210,7 +16246,7 @@
       </c>
       <c r="AI142" s="5" t="inlineStr">
         <is>
-          <t>PRIMARY 'about 1,200 men' (one regiment detached); tablet class pending</t>
+          <t>PRIMARY 'about 1,200 men' (one regiment detached); tablet class pending ; p11 sweep: B&amp;M-repro 1,813 (hop) beside the 1,200-engaged primary (one regiment detached)</t>
         </is>
       </c>
       <c r="AJ142" s="5" t="inlineStr">
@@ -16230,7 +16266,7 @@
       </c>
       <c r="AM142" s="5" t="inlineStr">
         <is>
-          <t>his 350 k&amp;w (40 k) vs return 380 (71 k) - the k conflict carried; 'nearly 300 buried'; the 1,800-prisoner inspector credit (not adopted); 26th Ga 11 = the structural control row</t>
+          <t>his 350 k&amp;w (40 k) vs return 380 (71 k) - the k conflict carried; 'nearly 300 buried'; the 1,800-prisoner inspector credit (not adopted); 26th Ga 11 = the structural control row ; p11: 13th Ga row closed at arithmetic grade (103 = 20/83/0); Guild k&amp;w ledger 65/258=323 noted (third count set)</t>
         </is>
       </c>
       <c r="AN142" s="5" t="n"/>
@@ -16370,7 +16406,7 @@
       </c>
       <c r="AI143" s="5" t="inlineStr">
         <is>
-          <t>OPEN (hop flagged); July 1 loss pre-shrinks the line (his own figures); tablet 'Present about 1200' (pass-10 hop; k/w cells = return exact)</t>
+          <t>OPEN (hop flagged); July 1 loss pre-shrinks the line (his own figures); tablet 'Present about 1200' (pass-10 hop; k/w cells = return exact) ; p11 sweep: B&amp;M-repro 1,295 (hop)</t>
         </is>
       </c>
       <c r="AJ143" s="5" t="inlineStr">
@@ -16530,7 +16566,7 @@
       </c>
       <c r="AI144" s="5" t="inlineStr">
         <is>
-          <t>tablet 'Present about 900' (pass-10 hop); no report primary</t>
+          <t>tablet 'Present about 900' (pass-10 hop); no report primary ; p11 sweep: B&amp;M-repro 1,244 (hop) beside the tablet ~900 - both hops, un-averaged</t>
         </is>
       </c>
       <c r="AJ144" s="5" t="inlineStr">
@@ -16550,7 +16586,7 @@
       </c>
       <c r="AM144" s="5" t="inlineStr">
         <is>
-          <t>return 345 (6th NC 172 / 21st 111 / 57th 62 - COLUMN-NOISE '623' cell caught by row arithmetic); no per-day primary - split flagged reconstruction</t>
+          <t>return 345 (6th NC 172 / 21st 111 / 57th 62 - COLUMN-NOISE '623' cell caught by row arithmetic); no per-day primary - split flagged reconstruction ; p11: 57th NC = 62 adopted at quadruple-arithmetic grade (printed '623' both channels; ED-71 candidate)</t>
         </is>
       </c>
       <c r="AN144" s="5" t="n"/>
@@ -16690,7 +16726,7 @@
       </c>
       <c r="AI145" s="5" t="inlineStr">
         <is>
-          <t>tablet '820 of 1,470' (adjudicated class); no report primary</t>
+          <t>tablet '820 of 1,470' (adjudicated class); no report primary ; CLOSED p11: June-30 return PRIMARY 114+1,350=1,464 (p. 564) beside tablet 1,470 + B&amp;M-repro 1,384 (hop) - un-averaged</t>
         </is>
       </c>
       <c r="AJ145" s="5" t="inlineStr">
@@ -16710,7 +16746,7 @@
       </c>
       <c r="AM145" s="5" t="inlineStr">
         <is>
-          <t>return (p. 342) 820 = 130/382/308 (m POOLED - the capture mass; single-cell OCR flag on w); THE SINGLE-SPIKE EXEMPLAR - one line, one field, minutes-scale; 12th NC 56 bounds the residue</t>
+          <t>return (p. 342) 820 = 130/382/308 (m POOLED - the capture mass; single-cell OCR flag on w); THE SINGLE-SPIKE EXEMPLAR - one line, one field, minutes-scale; 12th NC 56 bounds the residue ; p11 re-read: printed total row 130/328/308/820 fails own arithmetic (766 vs 820) both channels; 382 reconciliation-only; regiment rows digit-read (ED-71 candidate)</t>
         </is>
       </c>
       <c r="AN145" s="5" t="n"/>
@@ -16850,7 +16886,7 @@
       </c>
       <c r="AI146" s="5" t="inlineStr">
         <is>
-          <t>OPEN (no primary; no hop taken - flagged); tablet 'Present 1600' (pass-10 hop)</t>
+          <t>OPEN (no primary; no hop taken - flagged); tablet 'Present 1600' (pass-10 hop) ; p11 sweep: B&amp;M-repro 1,520 (hop) beside tablet ~1,600</t>
         </is>
       </c>
       <c r="AJ146" s="5" t="inlineStr">
@@ -17010,7 +17046,7 @@
       </c>
       <c r="AI147" s="5" t="inlineStr">
         <is>
-          <t>tablet 'Present about 1800' (compilation); no report statement</t>
+          <t>tablet 'Present about 1800' (compilation); no report statement ; p11 sweep: B&amp;M-repro 2,183 (hop) beside tablet ~1,800 - divergent hops, both carried</t>
         </is>
       </c>
       <c r="AJ147" s="5" t="inlineStr">
@@ -17665,7 +17701,7 @@
       </c>
       <c r="AL151" s="5" t="inlineStr">
         <is>
-          <t>[A window + B] '&gt;= one hour under a most galling fire' (his duration) / 'two hours' (Engelhard) - both carried; climax: '800 guns' combined two-brigade strength pin at the works</t>
+          <t>[A window + B] '&gt;= one hour under a most galling fire' (his duration) / 'two hours' (Engelhard) - both carried; climax: '800 guns' combined two-brigade strength pin at the works ; p11 back-extension: Scales's July 1 narrative in full - the Davis rescue, the pass-through of the ammunition-exhausted first line, the 75-yd halt, the ten-minutes-to-breakthrough pin, Perrin both-siding</t>
         </is>
       </c>
       <c r="AM151" s="5" t="inlineStr">
@@ -17934,7 +17970,7 @@
       </c>
       <c r="AI153" s="5" t="inlineStr">
         <is>
-          <t>OPEN (no primary; no hop taken - flagged); tablet 'Present about 1100' (pass-10 hop)</t>
+          <t>OPEN (no primary; no hop taken - flagged); tablet 'Present about 1100' (pass-10 hop) ; p11 sweep: B&amp;M-repro 1,104 (hop) - agrees with tablet ~1,100</t>
         </is>
       </c>
       <c r="AJ153" s="5" t="inlineStr">
@@ -18094,7 +18130,7 @@
       </c>
       <c r="AI154" s="5" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN ; p11: June-30 return PRIMARY 138+1,656=1,794 (p. 564, Rodes' old brigade row); B&amp;M-repro 1,688 (hop)</t>
         </is>
       </c>
       <c r="AJ154" s="5" t="inlineStr">
@@ -18233,20 +18269,56 @@
           <t>reg-csa-3c-pen-1</t>
         </is>
       </c>
-      <c r="AB155" s="5" t="n"/>
+      <c r="AB155" s="5" t="inlineStr">
+        <is>
+          <t>unauthored</t>
+        </is>
+      </c>
       <c r="AC155" s="5" t="n"/>
       <c r="AD155" s="5" t="n"/>
       <c r="AE155" s="5" t="n"/>
       <c r="AF155" s="5" t="n"/>
-      <c r="AG155" s="5" t="n"/>
-      <c r="AH155" s="5" t="n"/>
-      <c r="AI155" s="5" t="n"/>
-      <c r="AJ155" s="5" t="n"/>
-      <c r="AK155" s="5" t="n"/>
-      <c r="AL155" s="5" t="n"/>
-      <c r="AM155" s="5" t="n"/>
+      <c r="AG155" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-pen-1-perrin.md; CA-J1P-5 executor; feeds ED-70 candidate</t>
+        </is>
+      </c>
+      <c r="AH155" s="5" t="inlineStr">
+        <is>
+          <t>Perrin (14th SC) commanding McGowan's brigade from June 5; five regimental commanders named; division succession (Pender mw Jul 2 ~sunset -&gt; Lane) recorded</t>
+        </is>
+      </c>
+      <c r="AI155" s="5" t="inlineStr">
+        <is>
+          <t>No report figure (negative); B&amp;M-repro 1,882 (hop); the 1st SC Rifles LEFT AS TRAIN GUARD (named detachment primary) bounds engaged below the hop</t>
+        </is>
+      </c>
+      <c r="AJ155" s="5" t="inlineStr">
+        <is>
+          <t>[C ~08:00] the march order behind Heth; the deploy 3 mi out; the two bounds ([C ~15:00]; [C after 16:00] the Pender assault order); the fence-&gt;grove-&gt;barricade-&gt;stone-wall-&gt;town axis (both-sided artifacts: Paul's barricade, Gamble's wall, Wainwright's thirty pieces)</t>
+        </is>
+      </c>
+      <c r="AK155" s="5" t="inlineStr">
+        <is>
+          <t>[C after-16:00] THE ASSAULT LEG: pass-through of Pettigrew's exhausted line, the ravine dress, the hold-fire order, the two oblique splits, the town entry</t>
+        </is>
+      </c>
+      <c r="AL155" s="5" t="inlineStr">
+        <is>
+          <t>CA-J1P-5 EXECUTOR: 'the most destructive fire of musketry I have ever been exposed to'; Scales halted / 'Lane did not move upon my right at all' (both both-sided); 'hundreds of prisoners, two field-pieces'; Hill's corps ledger + halt decision</t>
+        </is>
+      </c>
+      <c r="AM155" s="5" t="inlineStr">
+        <is>
+          <t>Return p. 344: 100/477/0 = 577 (division 1,690 printed-exact); the two-left-regiments halving statement; July-1-dominant</t>
+        </is>
+      </c>
       <c r="AN155" s="5" t="n"/>
-      <c r="AO155" s="5" t="n"/>
+      <c r="AO155" s="5" t="inlineStr">
+        <is>
+          <t>T4 (July 1 grain; full arc T3)</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -18502,7 +18574,7 @@
       </c>
       <c r="AI157" s="5" t="inlineStr">
         <is>
-          <t>OPEN (no primary)</t>
+          <t>OPEN (no primary) ; CLOSED p11: June-30 return PRIMARY 119+971=1,090 (p. 564); B&amp;M-repro 1,027 (hop)</t>
         </is>
       </c>
       <c r="AJ157" s="5" t="inlineStr">
@@ -18822,7 +18894,7 @@
       </c>
       <c r="AI159" s="5" t="inlineStr">
         <is>
-          <t>tablet 'Present about 1200' (compilation, hop flagged); no primary</t>
+          <t>tablet 'Present about 1200' (compilation, hop flagged); no primary ; p11 sweep: B&amp;M-repro 1,334 (Semmes; hop) beside tablet ~1,200</t>
         </is>
       </c>
       <c r="AJ159" s="5" t="inlineStr">
@@ -18982,7 +19054,7 @@
       </c>
       <c r="AI160" s="5" t="inlineStr">
         <is>
-          <t>three-regiment structure primary (13th/58th VA detached, Hoffman); tablet 'Present about 800' (pass-10 hop)</t>
+          <t>three-regiment structure primary (13th/58th VA detached, Hoffman); tablet 'Present about 800' (pass-10 hop) ; p11 sweep: B&amp;M-repro 806 (hop) - agrees with the tablet ~800</t>
         </is>
       </c>
       <c r="AJ160" s="5" t="inlineStr">
@@ -19142,7 +19214,7 @@
       </c>
       <c r="AI161" s="5" t="inlineStr">
         <is>
-          <t>OPEN (no primary; no hop taken - flagged); tablet 'Present about 1700' (pass-10 hop)</t>
+          <t>OPEN (no primary; no hop taken - flagged); tablet 'Present about 1700' (pass-10 hop) ; p11 sweep: B&amp;M-repro 2,121 (hop) beside tablet ~1,700 - divergent hops, both carried</t>
         </is>
       </c>
       <c r="AJ161" s="5" t="inlineStr">
@@ -19302,7 +19374,7 @@
       </c>
       <c r="AI162" s="5" t="inlineStr">
         <is>
-          <t>OPEN; Terry's 4th VA 'three-fourths' fraction primary carried w/ scope flag (vs return 86); tablet 'Present about 1450' (pass-10 hop)</t>
+          <t>OPEN; Terry's 4th VA 'three-fourths' fraction primary carried w/ scope flag (vs return 86); tablet 'Present about 1450' (pass-10 hop) ; p11 sweep: B&amp;M-repro 1,323 (hop)</t>
         </is>
       </c>
       <c r="AJ162" s="5" t="inlineStr">
@@ -19746,7 +19818,7 @@
       </c>
       <c r="AI165" s="5" t="inlineStr">
         <is>
-          <t>tablet 'Present about 1350' (compilation, hop flagged)</t>
+          <t>tablet 'Present about 1350' (compilation, hop flagged) ; p11 sweep: B&amp;M-repro 1,398 (hop) - agrees with tablet ~1,350</t>
         </is>
       </c>
       <c r="AJ165" s="5" t="inlineStr">
@@ -29689,7 +29761,7 @@
       </c>
       <c r="AL250" s="5" t="inlineStr">
         <is>
-          <t>THE CA-J1M-2 EXECUTOR ('checking and retarding... several hours'; Buford: 'held its own for more than two hours'); the afternoon carbine stand ('saved a division of our infantry'); 'commenced the fight in the morning and close it in the evening'</t>
+          <t>THE CA-J1M-2 EXECUTOR ('checking and retarding... several hours'; Buford: 'held its own for more than two hours'); the afternoon carbine stand ('saved a division of our infantry'); 'commenced the fight in the morning and close it in the evening' ; p11: the afternoon stand's CSA half CLOSED (Lane's Hudson-40 detail + Perrin's 'Lane did not move') - the saved-a-division claim now three-report convergent</t>
         </is>
       </c>
       <c r="AM250" s="5" t="inlineStr">
@@ -29886,7 +29958,7 @@
       </c>
       <c r="AI252" s="5" t="inlineStr">
         <is>
-          <t>OPEN (no primary; B&amp;M-class reading not located)</t>
+          <t>OPEN (no primary; B&amp;M-class reading not located) ; CLOSED-at-hop p11: B&amp;M-repro 1,148 (the pass-10 'not located' now located)</t>
         </is>
       </c>
       <c r="AJ252" s="5" t="inlineStr">
@@ -33821,20 +33893,56 @@
           <t>reg-us-i-2-2</t>
         </is>
       </c>
-      <c r="AB284" s="5" t="n"/>
+      <c r="AB284" s="5" t="inlineStr">
+        <is>
+          <t>unauthored</t>
+        </is>
+      </c>
       <c r="AC284" s="5" t="n"/>
       <c r="AD284" s="5" t="n"/>
       <c r="AE284" s="5" t="n"/>
       <c r="AF284" s="5" t="n"/>
-      <c r="AG284" s="5" t="n"/>
-      <c r="AH284" s="5" t="n"/>
-      <c r="AI284" s="5" t="n"/>
-      <c r="AJ284" s="5" t="n"/>
-      <c r="AK284" s="5" t="n"/>
-      <c r="AL284" s="5" t="n"/>
-      <c r="AM284" s="5" t="n"/>
+      <c r="AG284" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-i-2-2-baxter.md; CA-J1P-2 Union receiving executor</t>
+        </is>
+      </c>
+      <c r="AH284" s="5" t="inlineStr">
+        <is>
+          <t>Baxter uninjured; Bates w x2, Wheelock captured/escaped, Lt. Thomas k in the streets; Coulter+11th Pa transferred out to 1st Bde</t>
+        </is>
+      </c>
+      <c r="AI284" s="5" t="inlineStr">
+        <is>
+          <t>No brigade primary (negative); B&amp;M-repro 1,452 (hop); division frame 'less than 2,500' (Robinson) CONFLICTS with the two-brigade B&amp;M sum 2,989 - both carried</t>
+        </is>
+      </c>
+      <c r="AJ284" s="5" t="inlineStr">
+        <is>
+          <t>[C 11:00] arrival; the two front-changes to the Oak Ridge crest (the pass-10 drawn wall bar = this line); [C ~17:00] the Emmitsburg-road line; [C Jul 2 10:00] relieved by Webb; the July 2-3 support ladder (six clocked moves); [C Jul 3 ~13:00] Cemetery Hill right-front under the cannonade ~2 h, then Hays's right</t>
+        </is>
+      </c>
+      <c r="AK284" s="5" t="inlineStr">
+        <is>
+          <t>[D] the relief hand-off ~15:00+ (Coulter's after-3, ammunition exhausted); the town retreat under fire; the clocked July 2-3 ladder</t>
+        </is>
+      </c>
+      <c r="AL284" s="5" t="inlineStr">
+        <is>
+          <t>THE IVERSON REPULSE RECEIVING RECORD: the deadly fire, the charge (88th Pa two flags + 97th NY one), the 12th Mass flank fire 'great influence upon its surrender'; Coulter 12:30 general-firing pin; division 'three flags and about 1,000 prisoners'; the Northrup conduct record</t>
+        </is>
+      </c>
+      <c r="AM284" s="5" t="inlineStr">
+        <is>
+          <t>Return p. 174 rows (not digit-re-read); division 'lost considerably more than half' of &lt;2,500 (primary); shape: the Oak Ridge window + the town capture spike; July 3 'considerable loss' skirmish clear (unquantified)</t>
+        </is>
+      </c>
       <c r="AN284" s="5" t="n"/>
-      <c r="AO284" s="5" t="n"/>
+      <c r="AO284" s="5" t="inlineStr">
+        <is>
+          <t>T4 (July 1 grain; full arc T3)</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
@@ -34126,7 +34234,7 @@
       </c>
       <c r="AI286" s="5" t="inlineStr">
         <is>
-          <t>no Jul 3 primary; build 460 remnant (compilation, flagged); Jul 1 wreck 898 of ~1,350-1,500 explains scale</t>
+          <t>no Jul 3 primary; build 460 remnant (compilation, flagged); Jul 1 wreck 898 of ~1,350-1,500 explains scale ; p11 back-extension: July 1 PRIMARY 1,287 in / 440 k&amp;w + 457 m / 390 left (dated July 2) - the day split lands; B&amp;M-repro 1,361 (hop)</t>
         </is>
       </c>
       <c r="AJ286" s="5" t="inlineStr">
@@ -34152,7 +34260,7 @@
       <c r="AN286" s="5" t="n"/>
       <c r="AO286" s="5" t="inlineStr">
         <is>
-          <t>T3 full-arc</t>
+          <t>T4 (July 1 grain; July 3 T3) - p11 upgrade</t>
         </is>
       </c>
     </row>
@@ -35545,20 +35653,56 @@
           <t>reg-us-xi-2-1</t>
         </is>
       </c>
-      <c r="AB295" s="5" t="n"/>
+      <c r="AB295" s="5" t="inlineStr">
+        <is>
+          <t>unauthored</t>
+        </is>
+      </c>
       <c r="AC295" s="5" t="n"/>
       <c r="AD295" s="5" t="n"/>
       <c r="AE295" s="5" t="n"/>
       <c r="AF295" s="5" t="n"/>
-      <c r="AG295" s="5" t="n"/>
-      <c r="AH295" s="5" t="n"/>
-      <c r="AI295" s="5" t="n"/>
-      <c r="AJ295" s="5" t="n"/>
-      <c r="AK295" s="5" t="n"/>
-      <c r="AL295" s="5" t="n"/>
-      <c r="AM295" s="5" t="n"/>
+      <c r="AG295" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-xi-2-1-coster.md</t>
+        </is>
+      </c>
+      <c r="AH295" s="5" t="inlineStr">
+        <is>
+          <t>Coster; NO report at any brigade echelon (verified negative - the third XI no-report brigade)</t>
+        </is>
+      </c>
+      <c r="AI295" s="5" t="inlineStr">
+        <is>
+          <t>No primary (negative); B&amp;M-repro 1,156 (hop); the brickyard force = three regiments (73rd Pa stayed on the hill)</t>
+        </is>
+      </c>
+      <c r="AJ295" s="5" t="inlineStr">
+        <is>
+          <t>[C ~14:00 via von Steinwehr] Cemetery Hill NE supporting Wiedrich (+ the stone-church regiment); [D] the brickyard line NE of town; the fall-back with the brick-house stopper; the hill's NE front July 2-3</t>
+        </is>
+      </c>
+      <c r="AK295" s="5" t="inlineStr">
+        <is>
+          <t>[D] the through-town commitment to the brickyard; the covered fall-back</t>
+        </is>
+      </c>
+      <c r="AL295" s="5" t="inlineStr">
+        <is>
+          <t>The brickyard delaying action (division grain + BOTH-SIDED by Hays/Avery pass 10); the brick-house stopper</t>
+        </is>
+      </c>
+      <c r="AM295" s="5" t="inlineStr">
+        <is>
+          <t>Return p. 183: 252/200/111/34 = 597 aggregate-exact (m column row-forced 313, noisy); the minutes-scale single-spike wreck second only to Iverson's</t>
+        </is>
+      </c>
       <c r="AN295" s="5" t="n"/>
-      <c r="AO295" s="5" t="n"/>
+      <c r="AO295" s="5" t="inlineStr">
+        <is>
+          <t>T2 (honestly thin; the fight T3 via the attackers)</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
@@ -35669,20 +35813,56 @@
           <t>reg-us-i-2-1</t>
         </is>
       </c>
-      <c r="AB296" s="5" t="n"/>
+      <c r="AB296" s="5" t="inlineStr">
+        <is>
+          <t>unauthored</t>
+        </is>
+      </c>
       <c r="AC296" s="5" t="n"/>
       <c r="AD296" s="5" t="n"/>
       <c r="AE296" s="5" t="n"/>
       <c r="AF296" s="5" t="n"/>
-      <c r="AG296" s="5" t="n"/>
-      <c r="AH296" s="5" t="n"/>
-      <c r="AI296" s="5" t="n"/>
-      <c r="AJ296" s="5" t="n"/>
-      <c r="AK296" s="5" t="n"/>
-      <c r="AL296" s="5" t="n"/>
-      <c r="AM296" s="5" t="n"/>
+      <c r="AG296" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-i-2-1-paul.md; the ED-52 Union day-split exemplar</t>
+        </is>
+      </c>
+      <c r="AH296" s="5" t="inlineStr">
+        <is>
+          <t>THE CASCADE: Paul severely w -&gt; Leonard w -&gt; Root w -&gt; Coulter (assigned on Cemetery Hill, w himself July 3) - five commanders; three Paul staff missing</t>
+        </is>
+      </c>
+      <c r="AI296" s="5" t="inlineStr">
+        <is>
+          <t>No brigade primary (negative); B&amp;M-repro 1,537 (hop); 16th Me ~275 literature-class NOT hopped</t>
+        </is>
+      </c>
+      <c r="AJ296" s="5" t="inlineStr">
+        <is>
+          <t>[D] the seminary rail-barricade (Paul entrenching - the artifact Perrin stormed, both-sided); the Oak Ridge relief slots; the 16th Maine sacrifice hill; Cemetery Hill; the Baxter-parallel July 2-3 ladder</t>
+        </is>
+      </c>
+      <c r="AK296" s="5" t="inlineStr">
+        <is>
+          <t>[D ~15:00] the relief insertion (Coulter-clocked); the 16th Me detachment + three-stage collapse; the town retreat</t>
+        </is>
+      </c>
+      <c r="AL296" s="5" t="inlineStr">
+        <is>
+          <t>The repeated-attacks repulse record (division grain); the 16th Maine hold-as-long-as-there-is-a-man order VERBATIM; July 2 dark gauntlet run; July 3 arrival at the repulse</t>
+        </is>
+      </c>
+      <c r="AM296" s="5" t="inlineStr">
+        <is>
+          <t>THE DAY-SPLIT PRIMARY: 776/28/14/3 = 821 (Coulter's table, excl. 11th Pa Jul 1); 16th Me July 1 223 (162 m = the pocket)</t>
+        </is>
+      </c>
       <c r="AN296" s="5" t="n"/>
-      <c r="AO296" s="5" t="n"/>
+      <c r="AO296" s="5" t="inlineStr">
+        <is>
+          <t>T3 (July 1 grain; full arc T2)</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
@@ -35989,7 +36169,7 @@
       </c>
       <c r="AL298" s="5" t="inlineStr">
         <is>
-          <t>[E] present under the cannonade's overs; NO fire window attested Jul 3 (consistent negative)</t>
+          <t>[E] present under the cannonade's overs; NO fire window attested Jul 3 (consistent negative) ; p11 back-extension: Roy Stone's report in full - the 11:00 / 12-1 Oak Hill enfilade / 1.30 grand-advance clock ladder (ED-69 candidate primary); the RR-cut episode; the cascade in action; 'nearly two-thirds... fell'</t>
         </is>
       </c>
       <c r="AM298" s="5" t="inlineStr">
@@ -36722,7 +36902,7 @@
       </c>
       <c r="AM303" s="5" t="inlineStr">
         <is>
-          <t>return: 140th NY 133 exact; brigade 200, division 1,029; three regiment rows digit-noisy (flagged); pins O'Rorke early / Weed late / Hazlett after Weed</t>
+          <t>return: 140th NY 133 exact; brigade 200, division 1,029; three regiment rows digit-noisy (flagged); pins O'Rorke early / Weed late / Hazlett after Weed ; p11 re-read: 140th NY digit-exact 1+25/5+84/18=133; brigade total row internally perfect 40/142/18=200; small rows off-by-one open (199 vs 200)</t>
         </is>
       </c>
       <c r="AN303" s="5" t="n"/>
@@ -37141,7 +37321,7 @@
       </c>
       <c r="AH306" s="5" t="inlineStr">
         <is>
-          <t>Ames -&gt; division (Barlow w July 1) -&gt; HARRIS commanding the bde from late July 1; Fowler (17th CT) k July 1; Noble took over July 4</t>
+          <t>Ames -&gt; division (Barlow w July 1) -&gt; HARRIS commanding the bde from late July 1; Fowler (17th CT) k July 1; Noble took over July 4 ; p11: the structured Barlow-Gordon record added (contemporary layer adopted - the July 7 letter + Gordon's OR pin; the 1903 memoir NO status)</t>
         </is>
       </c>
       <c r="AI306" s="5" t="inlineStr">
@@ -37765,20 +37945,56 @@
           <t>reg-us-xi-3-2</t>
         </is>
       </c>
-      <c r="AB310" s="5" t="n"/>
+      <c r="AB310" s="5" t="inlineStr">
+        <is>
+          <t>unauthored</t>
+        </is>
+      </c>
       <c r="AC310" s="5" t="n"/>
       <c r="AD310" s="5" t="n"/>
       <c r="AE310" s="5" t="n"/>
       <c r="AF310" s="5" t="n"/>
-      <c r="AG310" s="5" t="n"/>
-      <c r="AH310" s="5" t="n"/>
-      <c r="AI310" s="5" t="n"/>
-      <c r="AJ310" s="5" t="n"/>
-      <c r="AK310" s="5" t="n"/>
-      <c r="AL310" s="5" t="n"/>
-      <c r="AM310" s="5" t="n"/>
+      <c r="AG310" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-xi-3-2-krzyzanowski.md; CA-J1P-3 receiving center</t>
+        </is>
+      </c>
+      <c r="AH310" s="5" t="inlineStr">
+        <is>
+          <t>Krzyzanowski (no own report - verified negative); Col. J.S. Robinson (82nd OH) severely w; 26th WI Boebel w -&gt; Fuchs -&gt; Jacobs</t>
+        </is>
+      </c>
+      <c r="AI310" s="5" t="inlineStr">
+        <is>
+          <t>82nd OH PRIMARY 312 PFD (-&gt;220 Jul 11 bracket); no brigade primary; B&amp;M-repro 1,403 (hop)</t>
+        </is>
+      </c>
+      <c r="AJ310" s="5" t="inlineStr">
+        <is>
+          <t>[C ~14:00 secondhand] arrival + the line north of town (82nd OH left, 26th WI right); [C ~16:00] the Cemetery Hill stone-fence rally; the cemetery-building position Jul 2-5</t>
+        </is>
+      </c>
+      <c r="AK310" s="5" t="inlineStr">
+        <is>
+          <t>[D] the forward commitment; the division-ordered fall-back through town; the ~16:00 rally</t>
+        </is>
+      </c>
+      <c r="AL310" s="5" t="inlineStr">
+        <is>
+          <t>The open-field stand vs Gordon/Doles converging (both-sided); the town gauntlet; July 2-3 attested-quiet (26th WI no-loss negative)</t>
+        </is>
+      </c>
+      <c r="AM310" s="5" t="inlineStr">
+        <is>
+          <t>Return p. 183 digit-exact: 20/140/181/111/217 = 669; 82nd OH report=return EXACT 181; July 1 near-total</t>
+        </is>
+      </c>
       <c r="AN310" s="5" t="n"/>
-      <c r="AO310" s="5" t="n"/>
+      <c r="AO310" s="5" t="inlineStr">
+        <is>
+          <t>T3 (July 1 grain; full arc T2)</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
@@ -38710,7 +38926,7 @@
       </c>
       <c r="AI316" s="5" t="inlineStr">
         <is>
-          <t>24th Mich PRIMARY 496; brigade aggregate open</t>
+          <t>24th Mich PRIMARY 496; brigade aggregate open ; p11 sweep: B&amp;M-repro 1,829 brigade hop beside the 24th Mich 496 primary</t>
         </is>
       </c>
       <c r="AJ316" s="5" t="inlineStr">
@@ -40450,7 +40666,7 @@
       </c>
       <c r="AI328" s="5" t="inlineStr">
         <is>
-          <t>no primary (negative); ~1,387 compilation hop-flagged</t>
+          <t>no primary (negative); ~1,387 compilation hop-flagged ; p11: the 1,387 hop CONFIRMED at the sweep source</t>
         </is>
       </c>
       <c r="AJ328" s="5" t="inlineStr">
@@ -40465,7 +40681,7 @@
       </c>
       <c r="AL328" s="5" t="inlineStr">
         <is>
-          <t>[D] wave-1 defense vs Anderson (5th MI half-loss stand, both-sided with White's three advances)</t>
+          <t>[D] wave-1 defense vs Anderson (5th MI half-loss stand, both-sided with White's three advances) ; p11 clock re-read: 'About 2 p. m.' line-of-battle formation = the tablet's 2-3 P.M. (report=tablet pair; profile upgraded)</t>
         </is>
       </c>
       <c r="AM328" s="5" t="inlineStr">
@@ -40589,20 +40805,56 @@
           <t>reg-us-xi-3-1</t>
         </is>
       </c>
-      <c r="AB329" s="5" t="n"/>
+      <c r="AB329" s="5" t="inlineStr">
+        <is>
+          <t>unauthored</t>
+        </is>
+      </c>
       <c r="AC329" s="5" t="n"/>
       <c r="AD329" s="5" t="n"/>
       <c r="AE329" s="5" t="n"/>
       <c r="AF329" s="5" t="n"/>
-      <c r="AG329" s="5" t="n"/>
-      <c r="AH329" s="5" t="n"/>
-      <c r="AI329" s="5" t="n"/>
-      <c r="AJ329" s="5" t="n"/>
-      <c r="AK329" s="5" t="n"/>
-      <c r="AL329" s="5" t="n"/>
-      <c r="AM329" s="5" t="n"/>
+      <c r="AG329" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-xi-3-1-schimmelfennig.md; Dobke 1:30 feeds ED-69</t>
+        </is>
+      </c>
+      <c r="AH329" s="5" t="inlineStr">
+        <is>
+          <t>THE CASCADE UP: Howard-&gt;field, Schurz-&gt;corps, Schimmelfennig-&gt;division (cut off in town Jul 1-4), von Amsberg-&gt;brigade at commitment</t>
+        </is>
+      </c>
+      <c r="AI329" s="5" t="inlineStr">
+        <is>
+          <t>No brigade primary (negative); B&amp;M-repro 1,670 (hop); 45th NY one-third-assembled fraction; Schurz 'hardly over 6,000' division frame</t>
+        </is>
+      </c>
+      <c r="AJ329" s="5" t="inlineStr">
+        <is>
+          <t>[C 11:00-11:30] the I-Corps-right deploy (45th NY skirmish line, Dilger rear, 61st OH right); the open-field line under Oak Hill fire; [D ~16:00] the seminary cover halt; the town maze; Cemetery Hill stone fence</t>
+        </is>
+      </c>
+      <c r="AK329" s="5" t="inlineStr">
+        <is>
+          <t>[C] double-quick through town to deploy; the 16:00 retreat + THE ALLEY-TRAP town leg (~100 escaped); the July 2 night mile to the Culp's stone wall</t>
+        </is>
+      </c>
+      <c r="AL329" s="5" t="inlineStr">
+        <is>
+          <t>[C 13:30 early-lean] the flank fire + surrender event (the O'Neal/Iverson front from the XI side); the 157th NY vs Doles episode both-sided; the cross-corps retreat-cover order</t>
+        </is>
+      </c>
+      <c r="AM329" s="5" t="inlineStr">
+        <is>
+          <t>Return p. 183 digit-exact: 112/224/307/54/110 = 807 (rows sum); missing 453 = the town pockets</t>
+        </is>
+      </c>
       <c r="AN329" s="5" t="n"/>
-      <c r="AO329" s="5" t="n"/>
+      <c r="AO329" s="5" t="inlineStr">
+        <is>
+          <t>T3 (July 1 grain; full arc T2)</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
@@ -40734,7 +40986,7 @@
       </c>
       <c r="AI330" s="5" t="inlineStr">
         <is>
-          <t>OPEN; three-regiment knoll line (structural)</t>
+          <t>OPEN; three-regiment knoll line (structural) ; p11 sweep: B&amp;M-repro 1,118 (hop)</t>
         </is>
       </c>
       <c r="AJ330" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Overlay d13: +9 units; master table regenerated (330 rows, 150 audited)
Appends the pass-13 overlay entries (Randol, Pennington, Henry's and
Lane's Sumter battalions, V Corps Artillery/Martin's, Mahone, Posey,
Thomas, the Provost Guard) and regenerates the master table. No new
register rows this pass (all nine were existing register entries);
audited-unit count moves 141 -> 150.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -7321,20 +7321,56 @@
           <t>reg-csa-1c-bn-henry</t>
         </is>
       </c>
-      <c r="AB74" s="5" t="n"/>
+      <c r="AB74" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC74" s="5" t="n"/>
       <c r="AD74" s="5" t="n"/>
       <c r="AE74" s="5" t="n"/>
       <c r="AF74" s="5" t="n"/>
-      <c r="AG74" s="5" t="n"/>
-      <c r="AH74" s="5" t="n"/>
-      <c r="AI74" s="5" t="n"/>
-      <c r="AJ74" s="5" t="n"/>
-      <c r="AK74" s="5" t="n"/>
-      <c r="AL74" s="5" t="n"/>
-      <c r="AM74" s="5" t="n"/>
+      <c r="AG74" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-1c-bn-henry.md; closes the First Corps battalion arc's one gap (pass-12 triage)</t>
+        </is>
+      </c>
+      <c r="AH74" s="5" t="inlineStr">
+        <is>
+          <t>Maj. Mathis W. Henry; 4 batteries (Latham/Branch, Bachman/German, Garden/Palmetto, Reilly/Rowan); own report fetch-verified (No. 463, pp. 427-428)</t>
+        </is>
+      </c>
+      <c r="AI74" s="5" t="inlineStr">
+        <is>
+          <t>OPEN — no personnel total in report or tablet</t>
+        </is>
+      </c>
+      <c r="AJ74" s="5" t="inlineStr">
+        <is>
+          <t>[C report-primary] July 2 pm, 2 of 4 batteries (Reilly/Latham) engaged 'on the right of our line'; July 3 whole battalion; July-2/3 SCF-adjacent fire</t>
+        </is>
+      </c>
+      <c r="AK74" s="5" t="inlineStr">
+        <is>
+          <t>Reilly's/Latham's into line July 2 (16:00); Bachman's/Garden's join by July 3</t>
+        </is>
+      </c>
+      <c r="AL74" s="5" t="inlineStr">
+        <is>
+          <t>1,500 rounds report=tablet exact; TWO battery markers (Latham's, Garden's) independently credit ~17:00 fire vs Farnsworth's charge — new CA-SCF-2 CSA-side corroboration (now 5 sources)</t>
+        </is>
+      </c>
+      <c r="AM74" s="5" t="inlineStr">
+        <is>
+          <t>Report=tablet digit-exact: K4/W23 (no M/C stated)</t>
+        </is>
+      </c>
       <c r="AN74" s="5" t="n"/>
-      <c r="AO74" s="5" t="n"/>
+      <c r="AO74" s="5" t="inlineStr">
+        <is>
+          <t>T4 (battalion grain, ED-36 pattern)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -8885,20 +8921,56 @@
           <t>reg-csa-3c-bn-lane</t>
         </is>
       </c>
-      <c r="AB84" s="5" t="n"/>
+      <c r="AB84" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC84" s="5" t="n"/>
       <c r="AD84" s="5" t="n"/>
       <c r="AE84" s="5" t="n"/>
       <c r="AF84" s="5" t="n"/>
-      <c r="AG84" s="5" t="n"/>
-      <c r="AH84" s="5" t="n"/>
-      <c r="AI84" s="5" t="n"/>
-      <c r="AJ84" s="5" t="n"/>
-      <c r="AK84" s="5" t="n"/>
-      <c r="AL84" s="5" t="n"/>
-      <c r="AM84" s="5" t="n"/>
+      <c r="AG84" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-bn-lane.md; closes the Third Corps battalion arc's one gap (pass-12 triage)</t>
+        </is>
+      </c>
+      <c r="AH84" s="5" t="inlineStr">
+        <is>
+          <t>Maj. John Lane; 3 batteries (Ross/A, Patterson/B, Wingfield/C); own report fetch-verified (No. 548, pp. 635-636) — Capt. Wingfield w July 3</t>
+        </is>
+      </c>
+      <c r="AI84" s="5" t="inlineStr">
+        <is>
+          <t>OPEN — no personnel total in report or tablet</t>
+        </is>
+      </c>
+      <c r="AJ84" s="5" t="inlineStr">
+        <is>
+          <t>[C report-primary] ridge east of town, '~1,400 yards' from Cemetery Hill; Patterson's battery detached to Wilcox's brigade July 2 am — cross-reference to csa-3c-and-1-wilcox.md and CA-J2A-10</t>
+        </is>
+      </c>
+      <c r="AK84" s="5" t="inlineStr">
+        <is>
+          <t>Patterson's detachment leg (named trigger + destination activity); remainder static on the ridge</t>
+        </is>
+      </c>
+      <c r="AL84" s="5" t="inlineStr">
+        <is>
+          <t>Ross's/Wingfield's markers both name CA-J3A-1 cannonade participation — new geographic witnesses from Anderson's front</t>
+        </is>
+      </c>
+      <c r="AM84" s="5" t="inlineStr">
+        <is>
+          <t>DOUBLE digit-exact 3-way cross-check: battery-marker sums = battalion tablet on BOTH rounds (1,082) and casualties (30); Lane's OWN report gives a conflicting total (29) — ED-74 candidate proposed</t>
+        </is>
+      </c>
       <c r="AN84" s="5" t="n"/>
-      <c r="AO84" s="5" t="n"/>
+      <c r="AO84" s="5" t="inlineStr">
+        <is>
+          <t>T4 (battalion grain, own-report primary)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -18005,20 +18077,56 @@
           <t>reg-csa-3c-and-2</t>
         </is>
       </c>
-      <c r="AB152" s="5" t="n"/>
+      <c r="AB152" s="5" t="inlineStr">
+        <is>
+          <t>attested-static</t>
+        </is>
+      </c>
       <c r="AC152" s="5" t="n"/>
       <c r="AD152" s="5" t="n"/>
       <c r="AE152" s="5" t="n"/>
       <c r="AF152" s="5" t="n"/>
-      <c r="AG152" s="5" t="n"/>
-      <c r="AH152" s="5" t="n"/>
-      <c r="AI152" s="5" t="n"/>
-      <c r="AJ152" s="5" t="n"/>
-      <c r="AK152" s="5" t="n"/>
-      <c r="AL152" s="5" t="n"/>
-      <c r="AM152" s="5" t="n"/>
+      <c r="AG152" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-and-2-mahone.md; the famous CSA non-participation; cross-refs Wright's/Lang's dossiers (the neighbors that advanced)</t>
+        </is>
+      </c>
+      <c r="AH152" s="5" t="inlineStr">
+        <is>
+          <t>Brig. Gen. William Mahone throughout; own report fetch-verified (dated July 10, 1863)</t>
+        </is>
+      </c>
+      <c r="AI152" s="5" t="inlineStr">
+        <is>
+          <t>Report=tablet digit-exact: Present 1,500</t>
+        </is>
+      </c>
+      <c r="AJ152" s="5" t="inlineStr">
+        <is>
+          <t>[C report-primary] 'immediately in front of the enemy, in support of Pegram's batteries' — cross-ref csa-3c-bn-pegram.md; arrived forenoon July 2, unchanged through July 4</t>
+        </is>
+      </c>
+      <c r="AK152" s="5" t="inlineStr">
+        <is>
+          <t>NONE — the defining fact is the absence of a July 2 advance leg</t>
+        </is>
+      </c>
+      <c r="AL152" s="5" t="inlineStr">
+        <is>
+          <t>Skirmish line only both days, report=tablet corroborating; report is SILENT on why the brigade did not advance to support Wright's/Posey's requests — first-class negative</t>
+        </is>
+      </c>
+      <c r="AM152" s="5" t="inlineStr">
+        <is>
+          <t>Report=tablet digit-exact: K8/W55/M39 = 102, mainly from shelling while stationary</t>
+        </is>
+      </c>
       <c r="AN152" s="5" t="n"/>
-      <c r="AO152" s="5" t="n"/>
+      <c r="AO152" s="5" t="inlineStr">
+        <is>
+          <t>T4 (own-report primary, negative-evidence class)</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -18609,20 +18717,56 @@
           <t>reg-csa-3c-and-5</t>
         </is>
       </c>
-      <c r="AB156" s="5" t="n"/>
+      <c r="AB156" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC156" s="5" t="n"/>
       <c r="AD156" s="5" t="n"/>
       <c r="AE156" s="5" t="n"/>
       <c r="AF156" s="5" t="n"/>
-      <c r="AG156" s="5" t="n"/>
-      <c r="AH156" s="5" t="n"/>
-      <c r="AI156" s="5" t="n"/>
-      <c r="AJ156" s="5" t="n"/>
-      <c r="AK156" s="5" t="n"/>
-      <c r="AL156" s="5" t="n"/>
-      <c r="AM156" s="5" t="n"/>
+      <c r="AG156" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-and-5-posey.md; the PARTIAL-advance case between Mahone's none and Wright's/Lang's full advance</t>
+        </is>
+      </c>
+      <c r="AH156" s="5" t="inlineStr">
+        <is>
+          <t>Brig. Gen. Carnot Posey throughout; own report fetch-verified (dated July 29, 1863)</t>
+        </is>
+      </c>
+      <c r="AI156" s="5" t="inlineStr">
+        <is>
+          <t>CONFLICT: tablet 1,150 vs web-research 1,320 — not resolved</t>
+        </is>
+      </c>
+      <c r="AJ156" s="5" t="inlineStr">
+        <is>
+          <t>[C report-primary] open field w/ woods both flanks; advance '200-300 yds beyond the barn and house, which were burned' = the Bliss farm — NEW cross-ref to csa-3c-pen-3-thomas.md; withdrew to rear of Pegram's battery</t>
+        </is>
+      </c>
+      <c r="AK156" s="5" t="inlineStr">
+        <is>
+          <t>FOUR-STAGE piecemeal commitment (48th/19th, then 16th, then 12th) — Posey's own report blames this for the advance's failure to cohere</t>
+        </is>
+      </c>
+      <c r="AL156" s="5" t="inlineStr">
+        <is>
+          <t>Skirmish-grain success (pushed Union pickets back, drove artillerists off guns briefly) but never joined the main Cemetery Ridge assault</t>
+        </is>
+      </c>
+      <c r="AM156" s="5" t="inlineStr">
+        <is>
+          <t>CONFLICT: tablet K12/W71=83 vs web-research K15/W68=83 — same total, different split, not resolved</t>
+        </is>
+      </c>
       <c r="AN156" s="5" t="n"/>
-      <c r="AO156" s="5" t="n"/>
+      <c r="AO156" s="5" t="inlineStr">
+        <is>
+          <t>T4 (own-report primary, partial-advance class)</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -19693,20 +19837,56 @@
           <t>reg-csa-3c-pen-3</t>
         </is>
       </c>
-      <c r="AB163" s="5" t="n"/>
+      <c r="AB163" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC163" s="5" t="n"/>
       <c r="AD163" s="5" t="n"/>
       <c r="AE163" s="5" t="n"/>
       <c r="AF163" s="5" t="n"/>
-      <c r="AG163" s="5" t="n"/>
-      <c r="AH163" s="5" t="n"/>
-      <c r="AI163" s="5" t="n"/>
-      <c r="AJ163" s="5" t="n"/>
-      <c r="AK163" s="5" t="n"/>
-      <c r="AL163" s="5" t="n"/>
-      <c r="AM163" s="5" t="n"/>
+      <c r="AG163" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-3c-pen-3-thomas.md; REGISTER CORRECTION — Thomas is Pender's Division per reg-csa-3c-pen-3, not Anderson's, despite the task's framing (noted, not silently fixed)</t>
+        </is>
+      </c>
+      <c r="AH163" s="5" t="inlineStr">
+        <is>
+          <t>Brig. Gen. Edward L. Thomas throughout; own report NOT directly fetched this pass (civilwarhome.com mirror confirmed dead) — attributed grade only</t>
+        </is>
+      </c>
+      <c r="AI163" s="5" t="inlineStr">
+        <is>
+          <t>CONFLICT: ~1,400 attributed vs tablet 'about 1200' — not resolved</t>
+        </is>
+      </c>
+      <c r="AJ163" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet] July 1 reserve then McMillan's Woods; July 2 22:00 to Long Lane, flanked by McGowan's/Perrin's brigade (left) and the Bliss House/Barn (right) — same farm as csa-3c-and-5-posey.md's EC3.2, new cross-ref</t>
+        </is>
+      </c>
+      <c r="AK163" s="5" t="inlineStr">
+        <is>
+          <t>Reserve-&gt;McMillan's Woods (sunset J1); artillery-support-&gt;Long Lane (22:00 J2); skirmish line-&gt;Seminary Ridge (after dark J3)</t>
+        </is>
+      </c>
+      <c r="AL163" s="5" t="inlineStr">
+        <is>
+          <t>July 1-2 reserve/artillery-support only; July 3 'severe skirmishing... most of the day' — NOT a quiet-flank case despite the task's framing</t>
+        </is>
+      </c>
+      <c r="AM163" s="5" t="inlineStr">
+        <is>
+          <t>Tablet: K34/W179/M57 = 270 — HIGHEST of the three brigades in this pass's batch (Mahone 102, Posey 83)</t>
+        </is>
+      </c>
       <c r="AN163" s="5" t="n"/>
-      <c r="AO163" s="5" t="n"/>
+      <c r="AO163" s="5" t="inlineStr">
+        <is>
+          <t>T3 (tablet + attributed-report grain)</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -21249,20 +21429,56 @@
           <t>reg-us-v-arty</t>
         </is>
       </c>
-      <c r="AB177" s="5" t="n"/>
+      <c r="AB177" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC177" s="5" t="n"/>
       <c r="AD177" s="5" t="n"/>
       <c r="AE177" s="5" t="n"/>
       <c r="AF177" s="5" t="n"/>
-      <c r="AG177" s="5" t="n"/>
-      <c r="AH177" s="5" t="n"/>
-      <c r="AI177" s="5" t="n"/>
-      <c r="AJ177" s="5" t="n"/>
-      <c r="AK177" s="5" t="n"/>
-      <c r="AL177" s="5" t="n"/>
-      <c r="AM177" s="5" t="n"/>
+      <c r="AG177" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-v-arty-martin.md; the pass-12-recommended Union corps-arty group, picked over III/VI on a reasoned (not exhaustive) source check</t>
+        </is>
+      </c>
+      <c r="AH177" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Augustus P. Martin; 5 batteries (Hazlett's/Rittenhouse's, Walcott's, Watson's, Gibbs's, Barnes's); own report fetch-verified (No. 221, pp. 659-661)</t>
+        </is>
+      </c>
+      <c r="AI177" s="5" t="inlineStr">
+        <is>
+          <t>937 men / 48 guns (tablet, search-summary grade, not page-verified)</t>
+        </is>
+      </c>
+      <c r="AJ177" s="5" t="inlineStr">
+        <is>
+          <t>[C report-primary] brigade arrival 16:00-17:00 July 2; Battery I 'not to be found' — reassigned by III Corps staff without record (cross-corps command friction)</t>
+        </is>
+      </c>
+      <c r="AK177" s="5" t="inlineStr">
+        <is>
+          <t>Brigade-wide arrival only; individual battery legs not authored beyond Rittenhouse's existing dossier</t>
+        </is>
+      </c>
+      <c r="AL177" s="5" t="inlineStr">
+        <is>
+          <t>Hazlett k ('shot in the head... died at 8 p.m.', upgrades the tablet-only pin on file); Battery I overrun then RETAKEN by Lt. Peeples w/ the Garibaldi Guards</t>
+        </is>
+      </c>
+      <c r="AM177" s="5" t="inlineStr">
+        <is>
+          <t>Report-primary brigade total: K9/W33/M2 = 44; Battery D's own component (7k/6w) not yet reconciled with us-btty-rittenhouse.md's existing EC6</t>
+        </is>
+      </c>
       <c r="AN177" s="5" t="n"/>
-      <c r="AO177" s="5" t="n"/>
+      <c r="AO177" s="5" t="inlineStr">
+        <is>
+          <t>T4 (brigade grain)</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -22449,20 +22665,56 @@
           <t>reg-us-ha-2-1</t>
         </is>
       </c>
-      <c r="AB189" s="5" t="n"/>
+      <c r="AB189" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC189" s="5" t="n"/>
       <c r="AD189" s="5" t="n"/>
       <c r="AE189" s="5" t="n"/>
       <c r="AF189" s="5" t="n"/>
-      <c r="AG189" s="5" t="n"/>
-      <c r="AH189" s="5" t="n"/>
-      <c r="AI189" s="5" t="n"/>
-      <c r="AJ189" s="5" t="n"/>
-      <c r="AK189" s="5" t="n"/>
-      <c r="AL189" s="5" t="n"/>
-      <c r="AM189" s="5" t="n"/>
+      <c r="AG189" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-randol.md; self-surfaced by pass-12's McIntosh tablet quote; closed pass 13</t>
+        </is>
+      </c>
+      <c r="AH189" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Alanson M. Randol throughout; split command July 3 (Chester's section w/ Custer's brigade, Kinney's section near Hanover Road); armament discrepancy flagged (tablet '4 12-Pdrs' vs horse-arty convention of 3-in rifles)</t>
+        </is>
+      </c>
+      <c r="AI189" s="5" t="inlineStr">
+        <is>
+          <t>Tablet: 84 men (report-adjacent, not a B&amp;M hop)</t>
+        </is>
+      </c>
+      <c r="AJ189" s="5" t="inlineStr">
+        <is>
+          <t>[C tablet] with 1st Brig 2nd Cav Div, not engaged July 1-2; PASS-13 SHEET-CROP: Chester's section (10569,5638) and Kinney's section (10354,5270), ~370 m apart — first drawn confirmation the tablet split is real</t>
+        </is>
+      </c>
+      <c r="AK189" s="5" t="inlineStr">
+        <is>
+          <t>Not authored — no trigger/timing for either section located</t>
+        </is>
+      </c>
+      <c r="AL189" s="5" t="inlineStr">
+        <is>
+          <t>Chester's section co-named in McIntosh's tablet as CA-ECF-2 co-executor (~14:00); Kinney's section 'remained near Hanover Road', no engagement claimed</t>
+        </is>
+      </c>
+      <c r="AM189" s="5" t="inlineStr">
+        <is>
+          <t>Tablet: 'suffered no casualties' — explicit zero, both sections combined</t>
+        </is>
+      </c>
       <c r="AN189" s="5" t="n"/>
-      <c r="AO189" s="5" t="n"/>
+      <c r="AO189" s="5" t="inlineStr">
+        <is>
+          <t>T3 (ECF grain, split-section)</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -24105,20 +24357,56 @@
           <t>reg-us-ha-1-4</t>
         </is>
       </c>
-      <c r="AB207" s="5" t="n"/>
+      <c r="AB207" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC207" s="5" t="n"/>
       <c r="AD207" s="5" t="n"/>
       <c r="AE207" s="5" t="n"/>
       <c r="AF207" s="5" t="n"/>
-      <c r="AG207" s="5" t="n"/>
-      <c r="AH207" s="5" t="n"/>
-      <c r="AI207" s="5" t="n"/>
-      <c r="AJ207" s="5" t="n"/>
-      <c r="AK207" s="5" t="n"/>
-      <c r="AL207" s="5" t="n"/>
-      <c r="AM207" s="5" t="n"/>
+      <c r="AG207" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-pennington.md; self-surfaced by pass-12's McIntosh tablet quote; closed pass 13</t>
+        </is>
+      </c>
+      <c r="AH207" s="5" t="inlineStr">
+        <is>
+          <t>Lieut. A. C. M. Pennington Jr. throughout; six 3-in rifles (no armament discrepancy); parent Robertson's report defers narrative to Custer's</t>
+        </is>
+      </c>
+      <c r="AI207" s="5" t="inlineStr">
+        <is>
+          <t>Tablet: 129 men</t>
+        </is>
+      </c>
+      <c r="AJ207" s="5" t="inlineStr">
+        <is>
+          <t>[C, shared w/ Custer's brigade] Hanover Rd/Low Dutch sector; PASS-13 SHEET-CROP: 'PENNINGTON/CLARK BAT.M' at (10072,5237), south of Custer's block; 'Clark' unidentified</t>
+        </is>
+      </c>
+      <c r="AK207" s="5" t="inlineStr">
+        <is>
+          <t>Inferred-by-attachment to Custer's brigade only</t>
+        </is>
+      </c>
+      <c r="AL207" s="5" t="inlineStr">
+        <is>
+          <t>July 2 Hunterstown; July 3 ~14:00 CA-ECF-2, report=tablet agreement ('engaged all day' / 'on the right of the Union Army') — the pass's second report=tablet pair</t>
+        </is>
+      </c>
+      <c r="AM207" s="5" t="inlineStr">
+        <is>
+          <t>Tablet: wounded 1 officer only (no enlisted figure stated)</t>
+        </is>
+      </c>
       <c r="AN207" s="5" t="n"/>
-      <c r="AO207" s="5" t="n"/>
+      <c r="AO207" s="5" t="inlineStr">
+        <is>
+          <t>T3 (ECF grain)</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -33121,20 +33409,56 @@
           <t>reg-us-hq-provost</t>
         </is>
       </c>
-      <c r="AB276" s="5" t="n"/>
+      <c r="AB276" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC276" s="5" t="n"/>
       <c r="AD276" s="5" t="n"/>
       <c r="AE276" s="5" t="n"/>
       <c r="AF276" s="5" t="n"/>
-      <c r="AG276" s="5" t="n"/>
-      <c r="AH276" s="5" t="n"/>
-      <c r="AI276" s="5" t="n"/>
-      <c r="AJ276" s="5" t="n"/>
-      <c r="AK276" s="5" t="n"/>
-      <c r="AL276" s="5" t="n"/>
-      <c r="AM276" s="5" t="n"/>
+      <c r="AG276" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-hq-provost-patrick.md; the cheap command-record closer named in the task; thinnest sourcing of this pass's command batch (only the 93rd NY tablet is fetch-verified)</t>
+        </is>
+      </c>
+      <c r="AH276" s="5" t="inlineStr">
+        <is>
+          <t>Brig. Gen. Marsena R. Patrick, Provost Marshal General; 93rd NY served as HQ guard (own tablet fetch-verified)</t>
+        </is>
+      </c>
+      <c r="AI276" s="5" t="inlineStr">
+        <is>
+          <t>93rd NY: 399 (tablet); whole command: 1,750 (attributed, not reconciled with the 399 figure)</t>
+        </is>
+      </c>
+      <c r="AJ276" s="5" t="inlineStr">
+        <is>
+          <t>[D attributed] Sheely Farm HQ; [C tablet] 93rd NY near the Leister House/Taneytown Rd — the two positions not reconciled into one command anchor</t>
+        </is>
+      </c>
+      <c r="AK276" s="5" t="inlineStr">
+        <is>
+          <t>Not authored — rear-area, non-maneuvering command</t>
+        </is>
+      </c>
+      <c r="AL276" s="5" t="inlineStr">
+        <is>
+          <t>Patrick's own diary quote (attributed): checked straggler disorder, organized a guard keeping ~2,000 CSA prisoners safe after the July 3 repulse — downstream CA-J3A-9/10 context</t>
+        </is>
+      </c>
+      <c r="AM276" s="5" t="inlineStr">
+        <is>
+          <t>1 killed, 4 wounded (attributed, whole command)</t>
+        </is>
+      </c>
       <c r="AN276" s="5" t="n"/>
-      <c r="AO276" s="5" t="n"/>
+      <c r="AO276" s="5" t="inlineStr">
+        <is>
+          <t>T2 (command record)</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dossier pass 15: overlay + master-table regeneration + index update
Overlay: +37 new units (164 -> 201) covering all pass-15 dossiers (3
non-battery, 20 needs-own-dossier, 13 static-park verifications, 1
bonus closer). Master table regenerated (330 rows, 201 audited
overlay units, up from 164). Index: pass-15 section added with the
full 37-dossier table and the register-clearance framing.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -4977,20 +4977,56 @@
           <t>reg-csa-cav-ha-7</t>
         </is>
       </c>
-      <c r="AB49" s="5" t="n"/>
+      <c r="AB49" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (attested-absent-from-combat)</t>
+        </is>
+      </c>
       <c r="AC49" s="5" t="n"/>
       <c r="AD49" s="5" t="n"/>
       <c r="AE49" s="5" t="n"/>
       <c r="AF49" s="5" t="n"/>
-      <c r="AG49" s="5" t="n"/>
-      <c r="AH49" s="5" t="n"/>
-      <c r="AI49" s="5" t="n"/>
-      <c r="AJ49" s="5" t="n"/>
-      <c r="AK49" s="5" t="n"/>
-      <c r="AL49" s="5" t="n"/>
-      <c r="AM49" s="5" t="n"/>
+      <c r="AG49" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/csa-cav-ha-mcclanahan.md; bonus closer, not part of the task's core 23; closes needs-own-dossier to true zero</t>
+        </is>
+      </c>
+      <c r="AH49" s="5" t="inlineStr">
+        <is>
+          <t>Capt. John H. McClanahan, w/ Imboden's semi-independent command; NOT part of Beckham's Stuart HA bn</t>
+        </is>
+      </c>
+      <c r="AI49" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="AJ49" s="5" t="inlineStr">
+        <is>
+          <t>CONFIRMED reached field margin only noon Jul3, retired w/ trains at night - never fought</t>
+        </is>
+      </c>
+      <c r="AK49" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="AL49" s="5" t="inlineStr">
+        <is>
+          <t>train-guard duty Jul1-3; post-battle Williamsport action flagged as out-of-scope context</t>
+        </is>
+      </c>
+      <c r="AM49" s="5" t="inlineStr">
+        <is>
+          <t>'No report nor details of losses made' (formal negative)</t>
+        </is>
+      </c>
       <c r="AN49" s="5" t="n"/>
-      <c r="AO49" s="5" t="n"/>
+      <c r="AO49" s="5" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -21805,20 +21841,56 @@
           <t>reg-us-vi-arty</t>
         </is>
       </c>
-      <c r="AB178" s="5" t="n"/>
+      <c r="AB178" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (command/frame grain)</t>
+        </is>
+      </c>
       <c r="AC178" s="5" t="n"/>
       <c r="AD178" s="5" t="n"/>
       <c r="AE178" s="5" t="n"/>
       <c r="AF178" s="5" t="n"/>
-      <c r="AG178" s="5" t="n"/>
-      <c r="AH178" s="5" t="n"/>
-      <c r="AI178" s="5" t="n"/>
-      <c r="AJ178" s="5" t="n"/>
-      <c r="AK178" s="5" t="n"/>
-      <c r="AL178" s="5" t="n"/>
-      <c r="AM178" s="5" t="n"/>
+      <c r="AG178" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-vi-arty-tompkins.md; tablet 9-bty/54-gun vs register 8/48 discrepancy unresolved</t>
+        </is>
+      </c>
+      <c r="AH178" s="5" t="inlineStr">
+        <is>
+          <t>8 batteries (McCartney/Cowan/Harn/Waterman/Adams/Williston/Butler/L.Martin); Col. C.H.Tompkins; NO brigade report - 5 batteries filed own numbered reports (238-242) addressed to Tompkins</t>
+        </is>
+      </c>
+      <c r="AI178" s="5" t="inlineStr">
+        <is>
+          <t>937 men/48 guns (search-stage)</t>
+        </is>
+      </c>
+      <c r="AJ178" s="5" t="inlineStr">
+        <is>
+          <t>Weickert farm reserve ground; Ziegler's Grove convergence (4 batteries) Jul3 post-repulse</t>
+        </is>
+      </c>
+      <c r="AK178" s="5" t="inlineStr">
+        <is>
+          <t>not authored - no consolidated report</t>
+        </is>
+      </c>
+      <c r="AL178" s="5" t="inlineStr">
+        <is>
+          <t>'not actively engaged' except Cowan's; McCartney arrived after repulse</t>
+        </is>
+      </c>
+      <c r="AM178" s="5" t="inlineStr">
+        <is>
+          <t>tablet 12 total, not reconciled vs per-battery (mostly zero) tablets</t>
+        </is>
+      </c>
       <c r="AN178" s="5" t="n"/>
-      <c r="AO178" s="5" t="n"/>
+      <c r="AO178" s="5" t="inlineStr">
+        <is>
+          <t>T2 command record</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -23041,20 +23113,56 @@
           <t>reg-us-ar-1r-2</t>
         </is>
       </c>
-      <c r="AB190" s="5" t="n"/>
+      <c r="AB190" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC190" s="5" t="n"/>
       <c r="AD190" s="5" t="n"/>
       <c r="AE190" s="5" t="n"/>
       <c r="AF190" s="5" t="n"/>
-      <c r="AG190" s="5" t="n"/>
-      <c r="AH190" s="5" t="n"/>
-      <c r="AI190" s="5" t="n"/>
-      <c r="AJ190" s="5" t="n"/>
-      <c r="AK190" s="5" t="n"/>
-      <c r="AL190" s="5" t="n"/>
-      <c r="AM190" s="5" t="n"/>
+      <c r="AG190" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-turnbull.md; TRIAGE CORRECTION - lost guns in combat, strongest contradiction of static-park</t>
+        </is>
+      </c>
+      <c r="AH190" s="5" t="inlineStr">
+        <is>
+          <t>Lt. John C. Turnbull, Batteries F&amp;K 3US; 6x12pdr</t>
+        </is>
+      </c>
+      <c r="AI190" s="5" t="inlineStr">
+        <is>
+          <t>145 men</t>
+        </is>
+      </c>
+      <c r="AJ190" s="5" t="inlineStr">
+        <is>
+          <t>[D Jul1] crest near Meade's HQ; [D Jul2] log house/Emmitsburg Rd w/Humphreys; [D Jul3] Taneytown Rd/Cemetery Hill</t>
+        </is>
+      </c>
+      <c r="AK190" s="5" t="inlineStr">
+        <is>
+          <t>[D] 3-position chain Jul1-3</t>
+        </is>
+      </c>
+      <c r="AL190" s="5" t="inlineStr">
+        <is>
+          <t>engaged Jul2, COMPELLED TO RETIRE, lost 4 guns+45 horses (recaptured)</t>
+        </is>
+      </c>
+      <c r="AM190" s="5" t="inlineStr">
+        <is>
+          <t>1off+8k/14w/1m = 24</t>
+        </is>
+      </c>
       <c r="AN190" s="5" t="n"/>
-      <c r="AO190" s="5" t="n"/>
+      <c r="AO190" s="5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -23217,20 +23325,56 @@
           <t>reg-us-ar-2v-1</t>
         </is>
       </c>
-      <c r="AB192" s="5" t="n"/>
+      <c r="AB192" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (attested-absent)</t>
+        </is>
+      </c>
       <c r="AC192" s="5" t="n"/>
       <c r="AD192" s="5" t="n"/>
       <c r="AE192" s="5" t="n"/>
       <c r="AF192" s="5" t="n"/>
-      <c r="AG192" s="5" t="n"/>
-      <c r="AH192" s="5" t="n"/>
-      <c r="AI192" s="5" t="n"/>
-      <c r="AJ192" s="5" t="n"/>
-      <c r="AK192" s="5" t="n"/>
-      <c r="AL192" s="5" t="n"/>
-      <c r="AM192" s="5" t="n"/>
+      <c r="AG192" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-brooker.md; TRIAGE CONFIRMED (the exception to this pass's corrections)</t>
+        </is>
+      </c>
+      <c r="AH192" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Albert F. Brooker, Battery B 1CT Heavy; 4x4.5in siege rifle</t>
+        </is>
+      </c>
+      <c r="AI192" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="AJ192" s="5" t="inlineStr">
+        <is>
+          <t>CONFIRMED never at Gettysburg - held at Westminster MD (siege ordnance unsuited to rapid movement)</t>
+        </is>
+      </c>
+      <c r="AK192" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="AL192" s="5" t="inlineStr">
+        <is>
+          <t>held at Westminster throughout</t>
+        </is>
+      </c>
+      <c r="AM192" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
       <c r="AN192" s="5" t="n"/>
-      <c r="AO192" s="5" t="n"/>
+      <c r="AO192" s="5" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -24521,20 +24665,56 @@
           <t>reg-us-ar-2v-2</t>
         </is>
       </c>
-      <c r="AB206" s="5" t="n"/>
+      <c r="AB206" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok (attested-absent)</t>
+        </is>
+      </c>
       <c r="AC206" s="5" t="n"/>
       <c r="AD206" s="5" t="n"/>
       <c r="AE206" s="5" t="n"/>
       <c r="AF206" s="5" t="n"/>
-      <c r="AG206" s="5" t="n"/>
-      <c r="AH206" s="5" t="n"/>
-      <c r="AI206" s="5" t="n"/>
-      <c r="AJ206" s="5" t="n"/>
-      <c r="AK206" s="5" t="n"/>
-      <c r="AL206" s="5" t="n"/>
-      <c r="AM206" s="5" t="n"/>
+      <c r="AG206" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-pratt.md; TRIAGE CONFIRMED; brigade's 8-casualty total therefore belongs entirely to Sterling's+Taft's batteries</t>
+        </is>
+      </c>
+      <c r="AH206" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Franklin A. Pratt, Battery M 1CT Heavy; 4x4.5in siege rifle</t>
+        </is>
+      </c>
+      <c r="AI206" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="AJ206" s="5" t="inlineStr">
+        <is>
+          <t>CONFIRMED never engaged - Westminster MD w/ Brooker's battery</t>
+        </is>
+      </c>
+      <c r="AK206" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="AL206" s="5" t="inlineStr">
+        <is>
+          <t>held at Westminster</t>
+        </is>
+      </c>
+      <c r="AM206" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
       <c r="AN206" s="5" t="n"/>
-      <c r="AO206" s="5" t="n"/>
+      <c r="AO206" s="5" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -24893,20 +25073,56 @@
           <t>reg-us-ar-4v-4</t>
         </is>
       </c>
-      <c r="AB209" s="5" t="n"/>
+      <c r="AB209" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC209" s="5" t="n"/>
       <c r="AD209" s="5" t="n"/>
       <c r="AE209" s="5" t="n"/>
       <c r="AF209" s="5" t="n"/>
-      <c r="AG209" s="5" t="n"/>
-      <c r="AH209" s="5" t="n"/>
-      <c r="AI209" s="5" t="n"/>
-      <c r="AJ209" s="5" t="n"/>
-      <c r="AK209" s="5" t="n"/>
-      <c r="AL209" s="5" t="n"/>
-      <c r="AM209" s="5" t="n"/>
+      <c r="AG209" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-ames.md; TRIAGE CORRECTION, closes the 13-battery sweep</t>
+        </is>
+      </c>
+      <c r="AH209" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Nelson Ames, Battery G 1NY; 6x12pdr Nap</t>
+        </is>
+      </c>
+      <c r="AI209" s="5" t="inlineStr">
+        <is>
+          <t>132 men</t>
+        </is>
+      </c>
+      <c r="AJ209" s="5" t="inlineStr">
+        <is>
+          <t>[A 15:00-17:30 Jul2] Peach Orchard w/ III Corps; [D Jul3] Cemetery Ridge w/ II Corps 1st Div</t>
+        </is>
+      </c>
+      <c r="AK209" s="5" t="inlineStr">
+        <is>
+          <t>[A] into Peach Orchard line; [D] relocate to II Corps ground</t>
+        </is>
+      </c>
+      <c r="AL209" s="5" t="inlineStr">
+        <is>
+          <t>3-5:30pm Peach Orchard fight (precisely timed)</t>
+        </is>
+      </c>
+      <c r="AM209" s="5" t="inlineStr">
+        <is>
+          <t>7w</t>
+        </is>
+      </c>
       <c r="AN209" s="5" t="n"/>
-      <c r="AO209" s="5" t="n"/>
+      <c r="AO209" s="5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -26437,20 +26653,56 @@
           <t>reg-us-ar-4v-1</t>
         </is>
       </c>
-      <c r="AB220" s="5" t="n"/>
+      <c r="AB220" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC220" s="5" t="n"/>
       <c r="AD220" s="5" t="n"/>
       <c r="AE220" s="5" t="n"/>
       <c r="AF220" s="5" t="n"/>
-      <c r="AG220" s="5" t="n"/>
-      <c r="AH220" s="5" t="n"/>
-      <c r="AI220" s="5" t="n"/>
-      <c r="AJ220" s="5" t="n"/>
-      <c r="AK220" s="5" t="n"/>
-      <c r="AL220" s="5" t="n"/>
-      <c r="AM220" s="5" t="n"/>
+      <c r="AG220" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-dow.md; TRIAGE CORRECTION</t>
+        </is>
+      </c>
+      <c r="AH220" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Edwin B. Dow, 6th Maine Battery(F); 4x12pdr Nap</t>
+        </is>
+      </c>
+      <c r="AI220" s="5" t="inlineStr">
+        <is>
+          <t>103 men</t>
+        </is>
+      </c>
+      <c r="AJ220" s="5" t="inlineStr">
+        <is>
+          <t>detached under McGilvery (Fitzhugh's own report)</t>
+        </is>
+      </c>
+      <c r="AK220" s="5" t="inlineStr">
+        <is>
+          <t>not authored beyond detachment</t>
+        </is>
+      </c>
+      <c r="AL220" s="5" t="inlineStr">
+        <is>
+          <t>Jul3 pre-charge cannonade duel</t>
+        </is>
+      </c>
+      <c r="AM220" s="5" t="inlineStr">
+        <is>
+          <t>13w (all attributed to the cannonade)</t>
+        </is>
+      </c>
       <c r="AN220" s="5" t="n"/>
-      <c r="AO220" s="5" t="n"/>
+      <c r="AO220" s="5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -26561,20 +26813,56 @@
           <t>reg-us-ar-3v-1</t>
         </is>
       </c>
-      <c r="AB221" s="5" t="n"/>
+      <c r="AB221" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC221" s="5" t="n"/>
       <c r="AD221" s="5" t="n"/>
       <c r="AE221" s="5" t="n"/>
       <c r="AF221" s="5" t="n"/>
-      <c r="AG221" s="5" t="n"/>
-      <c r="AH221" s="5" t="n"/>
-      <c r="AI221" s="5" t="n"/>
-      <c r="AJ221" s="5" t="n"/>
-      <c r="AK221" s="5" t="n"/>
-      <c r="AL221" s="5" t="n"/>
-      <c r="AM221" s="5" t="n"/>
+      <c r="AG221" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-edgell.md; matches Taft's-battery triage-mismatch pattern exactly</t>
+        </is>
+      </c>
+      <c r="AH221" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Frederick M. Edgell, 1st NH Battery; own report</t>
+        </is>
+      </c>
+      <c r="AI221" s="5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AJ221" s="5" t="inlineStr">
+        <is>
+          <t>[C ~14:30 Jul2] Cemetery Hill nr seminary; [D Jul3] relocated to cornfield nr Baltimore turnpike</t>
+        </is>
+      </c>
+      <c r="AK221" s="5" t="inlineStr">
+        <is>
+          <t>[C] into position; [D] relocation</t>
+        </is>
+      </c>
+      <c r="AL221" s="5" t="inlineStr">
+        <is>
+          <t>counter-battery fire; 105rds sub-total/353 total (2 scopes, not conflict)</t>
+        </is>
+      </c>
+      <c r="AM221" s="5" t="inlineStr">
+        <is>
+          <t>3w(1 serious)/3horses k</t>
+        </is>
+      </c>
       <c r="AN221" s="5" t="n"/>
-      <c r="AO221" s="5" t="n"/>
+      <c r="AO221" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -26685,20 +26973,56 @@
           <t>reg-us-ha-1-5</t>
         </is>
       </c>
-      <c r="AB222" s="5" t="n"/>
+      <c r="AB222" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC222" s="5" t="n"/>
       <c r="AD222" s="5" t="n"/>
       <c r="AE222" s="5" t="n"/>
       <c r="AF222" s="5" t="n"/>
-      <c r="AG222" s="5" t="n"/>
-      <c r="AH222" s="5" t="n"/>
-      <c r="AI222" s="5" t="n"/>
-      <c r="AJ222" s="5" t="n"/>
-      <c r="AK222" s="5" t="n"/>
-      <c r="AL222" s="5" t="n"/>
-      <c r="AM222" s="5" t="n"/>
+      <c r="AG222" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-elder.md; 3rd independent Union SCF corroboration (ED-72)</t>
+        </is>
+      </c>
+      <c r="AH222" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Samuel S. Elder, Battery E 4US; 4x3in rifle (sub-6-gun)</t>
+        </is>
+      </c>
+      <c r="AI222" s="5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AJ222" s="5" t="inlineStr">
+        <is>
+          <t>[C Jun29] detached to 3rd Cav Div; [D Jul3] Bushman Hill SW of Round Top; sheet-crop confirmed beside Farnsworth's Bde</t>
+        </is>
+      </c>
+      <c r="AK222" s="5" t="inlineStr">
+        <is>
+          <t>[C Jun29] detachment; [D Jul3] into position</t>
+        </is>
+      </c>
+      <c r="AL222" s="5" t="inlineStr">
+        <is>
+          <t>South Cavalry Field ~17:30, CA-SCF-2</t>
+        </is>
+      </c>
+      <c r="AM222" s="5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AN222" s="5" t="n"/>
-      <c r="AO222" s="5" t="n"/>
+      <c r="AO222" s="5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -26969,20 +27293,56 @@
           <t>reg-us-ha-2-2</t>
         </is>
       </c>
-      <c r="AB224" s="5" t="n"/>
+      <c r="AB224" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC224" s="5" t="n"/>
       <c r="AD224" s="5" t="n"/>
       <c r="AE224" s="5" t="n"/>
       <c r="AF224" s="5" t="n"/>
-      <c r="AG224" s="5" t="n"/>
-      <c r="AH224" s="5" t="n"/>
-      <c r="AI224" s="5" t="n"/>
-      <c r="AJ224" s="5" t="n"/>
-      <c r="AK224" s="5" t="n"/>
-      <c r="AL224" s="5" t="n"/>
-      <c r="AM224" s="5" t="n"/>
+      <c r="AG224" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-graham.md</t>
+        </is>
+      </c>
+      <c r="AH224" s="5" t="inlineStr">
+        <is>
+          <t>Capt. (bvt LtCol) William M. Graham, Battery K 1US; 6x3in rifle</t>
+        </is>
+      </c>
+      <c r="AI224" s="5" t="inlineStr">
+        <is>
+          <t>114 men (search-summary)</t>
+        </is>
+      </c>
+      <c r="AJ224" s="5" t="inlineStr">
+        <is>
+          <t>South Cavalry Field Jul3, left w/ cavalry, engaged Farnsworth's/Merritt's attacks</t>
+        </is>
+      </c>
+      <c r="AK224" s="5" t="inlineStr">
+        <is>
+          <t>not authored</t>
+        </is>
+      </c>
+      <c r="AL224" s="5" t="inlineStr">
+        <is>
+          <t>SCF action alongside Farnsworth's/Merritt's brigades</t>
+        </is>
+      </c>
+      <c r="AM224" s="5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AN224" s="5" t="n"/>
-      <c r="AO224" s="5" t="n"/>
+      <c r="AO224" s="5" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -27341,20 +27701,56 @@
           <t>reg-us-ar-3v-4</t>
         </is>
       </c>
-      <c r="AB227" s="5" t="n"/>
+      <c r="AB227" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC227" s="5" t="n"/>
       <c r="AD227" s="5" t="n"/>
       <c r="AE227" s="5" t="n"/>
       <c r="AF227" s="5" t="n"/>
-      <c r="AG227" s="5" t="n"/>
-      <c r="AH227" s="5" t="n"/>
-      <c r="AI227" s="5" t="n"/>
-      <c r="AJ227" s="5" t="n"/>
-      <c r="AK227" s="5" t="n"/>
-      <c r="AL227" s="5" t="n"/>
-      <c r="AM227" s="5" t="n"/>
+      <c r="AG227" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-hill.md; TRIAGE CORRECTION, per-day casualty date split</t>
+        </is>
+      </c>
+      <c r="AH227" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Wallace Hill, Battery C 1WV; 4x10pdr Parrott (sub-6-gun)</t>
+        </is>
+      </c>
+      <c r="AI227" s="5" t="inlineStr">
+        <is>
+          <t>124 men</t>
+        </is>
+      </c>
+      <c r="AJ227" s="5" t="inlineStr">
+        <is>
+          <t>Cemetery Hill, right on cemetery/left near stonewall by road</t>
+        </is>
+      </c>
+      <c r="AK227" s="5" t="inlineStr">
+        <is>
+          <t>not authored - single position only</t>
+        </is>
+      </c>
+      <c r="AL227" s="5" t="inlineStr">
+        <is>
+          <t>fought Jul2-3</t>
+        </is>
+      </c>
+      <c r="AM227" s="5" t="inlineStr">
+        <is>
+          <t>2k(named+dated: Braddock Jul2, Lacy Jul3)/2w</t>
+        </is>
+      </c>
       <c r="AN227" s="5" t="n"/>
-      <c r="AO227" s="5" t="n"/>
+      <c r="AO227" s="5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -27713,20 +28109,56 @@
           <t>reg-us-ar-1r-1</t>
         </is>
       </c>
-      <c r="AB230" s="5" t="n"/>
+      <c r="AB230" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC230" s="5" t="n"/>
       <c r="AD230" s="5" t="n"/>
       <c r="AE230" s="5" t="n"/>
       <c r="AF230" s="5" t="n"/>
-      <c r="AG230" s="5" t="n"/>
-      <c r="AH230" s="5" t="n"/>
-      <c r="AI230" s="5" t="n"/>
-      <c r="AJ230" s="5" t="n"/>
-      <c r="AK230" s="5" t="n"/>
-      <c r="AL230" s="5" t="n"/>
-      <c r="AM230" s="5" t="n"/>
+      <c r="AG230" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-eakin.md; corrects static-park triage</t>
+        </is>
+      </c>
+      <c r="AH230" s="5" t="inlineStr">
+        <is>
+          <t>Lt. Chandler P. Eakin (w Jul2), Lt. Philip D. Mason succ.; Battery H 1US; 6x12pdr</t>
+        </is>
+      </c>
+      <c r="AI230" s="5" t="inlineStr">
+        <is>
+          <t>153 men</t>
+        </is>
+      </c>
+      <c r="AJ230" s="5" t="inlineStr">
+        <is>
+          <t>Cemetery Hill facing Emmitsburg Rd</t>
+        </is>
+      </c>
+      <c r="AK230" s="5" t="inlineStr">
+        <is>
+          <t>not authored - no leg located</t>
+        </is>
+      </c>
+      <c r="AL230" s="5" t="inlineStr">
+        <is>
+          <t>engaged Jul2-3 (TRIAGE CORRECTION: was static-park, actually 2-day fight)</t>
+        </is>
+      </c>
+      <c r="AM230" s="5" t="inlineStr">
+        <is>
+          <t>1k/1off+7w/1m = 10 total</t>
+        </is>
+      </c>
       <c r="AN230" s="5" t="n"/>
-      <c r="AO230" s="5" t="n"/>
+      <c r="AO230" s="5" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
@@ -27837,20 +28269,56 @@
           <t>reg-us-ar-3v-2</t>
         </is>
       </c>
-      <c r="AB231" s="5" t="n"/>
+      <c r="AB231" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC231" s="5" t="n"/>
       <c r="AD231" s="5" t="n"/>
       <c r="AE231" s="5" t="n"/>
       <c r="AF231" s="5" t="n"/>
-      <c r="AG231" s="5" t="n"/>
-      <c r="AH231" s="5" t="n"/>
-      <c r="AI231" s="5" t="n"/>
-      <c r="AJ231" s="5" t="n"/>
-      <c r="AK231" s="5" t="n"/>
-      <c r="AL231" s="5" t="n"/>
-      <c r="AM231" s="5" t="n"/>
+      <c r="AG231" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-norton-1oh.md; TRIAGE CORRECTION</t>
+        </is>
+      </c>
+      <c r="AH231" s="5" t="inlineStr">
+        <is>
+          <t>Lt. George W. Norton, Battery H 1OH ('Huntington's Ohio Battery'); 6x3in Ord Rifle; DISTINCT from the LRT-witness Norton on us-btty-rittenhouse.md</t>
+        </is>
+      </c>
+      <c r="AI231" s="5" t="inlineStr">
+        <is>
+          <t>123 men</t>
+        </is>
+      </c>
+      <c r="AJ231" s="5" t="inlineStr">
+        <is>
+          <t>Cemetery Hill, relieved a 'badly shot up' battery in place, held through the close</t>
+        </is>
+      </c>
+      <c r="AK231" s="5" t="inlineStr">
+        <is>
+          <t>[D] arrival-&gt;relief-in-place</t>
+        </is>
+      </c>
+      <c r="AL231" s="5" t="inlineStr">
+        <is>
+          <t>relief-in-place + sustained defense</t>
+        </is>
+      </c>
+      <c r="AM231" s="5" t="inlineStr">
+        <is>
+          <t>2k(named: Schram,Kirsh)/1mw(named: Edmunds)/4w</t>
+        </is>
+      </c>
       <c r="AN231" s="5" t="n"/>
-      <c r="AO231" s="5" t="n"/>
+      <c r="AO231" s="5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -28405,20 +28873,56 @@
           <t>reg-us-ar-4v-2</t>
         </is>
       </c>
-      <c r="AB235" s="5" t="n"/>
+      <c r="AB235" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC235" s="5" t="n"/>
       <c r="AD235" s="5" t="n"/>
       <c r="AE235" s="5" t="n"/>
       <c r="AF235" s="5" t="n"/>
-      <c r="AG235" s="5" t="n"/>
-      <c r="AH235" s="5" t="n"/>
-      <c r="AI235" s="5" t="n"/>
-      <c r="AJ235" s="5" t="n"/>
-      <c r="AK235" s="5" t="n"/>
-      <c r="AL235" s="5" t="n"/>
-      <c r="AM235" s="5" t="n"/>
+      <c r="AG235" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-rigby.md; TRIAGE CORRECTION</t>
+        </is>
+      </c>
+      <c r="AH235" s="5" t="inlineStr">
+        <is>
+          <t>Capt. James H. Rigby, Battery A 1MD; 6x ord rifle; distinct from CSA '1st Maryland Battery' (Dement) - collision resolved</t>
+        </is>
+      </c>
+      <c r="AI235" s="5" t="inlineStr">
+        <is>
+          <t>4off+102men</t>
+        </is>
+      </c>
+      <c r="AJ235" s="5" t="inlineStr">
+        <is>
+          <t>Powers Hill per Tyler's own order (XII Corps ground)</t>
+        </is>
+      </c>
+      <c r="AK235" s="5" t="inlineStr">
+        <is>
+          <t>not authored beyond assignment</t>
+        </is>
+      </c>
+      <c r="AL235" s="5" t="inlineStr">
+        <is>
+          <t>Culp's Hill infantry + Benner's Hill CSA arty duel; 211 rds fired</t>
+        </is>
+      </c>
+      <c r="AM235" s="5" t="inlineStr">
+        <is>
+          <t>0 (engaged but zero-loss)</t>
+        </is>
+      </c>
       <c r="AN235" s="5" t="n"/>
-      <c r="AO235" s="5" t="n"/>
+      <c r="AO235" s="5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -28973,20 +29477,56 @@
           <t>reg-us-ar-2v-3</t>
         </is>
       </c>
-      <c r="AB239" s="5" t="n"/>
+      <c r="AB239" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC239" s="5" t="n"/>
       <c r="AD239" s="5" t="n"/>
       <c r="AE239" s="5" t="n"/>
       <c r="AF239" s="5" t="n"/>
-      <c r="AG239" s="5" t="n"/>
-      <c r="AH239" s="5" t="n"/>
-      <c r="AI239" s="5" t="n"/>
-      <c r="AJ239" s="5" t="n"/>
-      <c r="AK239" s="5" t="n"/>
-      <c r="AL239" s="5" t="n"/>
-      <c r="AM239" s="5" t="n"/>
+      <c r="AG239" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-sterling.md; TRIAGE CORRECTION</t>
+        </is>
+      </c>
+      <c r="AH239" s="5" t="inlineStr">
+        <is>
+          <t>Capt. John William Sterling, 2CT Light Battery; UNIQUE ordnance - 4x14pdr James Rifle+2x12pdr howitzer, only such battery at Gettysburg</t>
+        </is>
+      </c>
+      <c r="AI239" s="5" t="inlineStr">
+        <is>
+          <t>106 men</t>
+        </is>
+      </c>
+      <c r="AJ239" s="5" t="inlineStr">
+        <is>
+          <t>[D Jul2] reinforced III Corps line, retired into McGilvery's composite line left of II Corps</t>
+        </is>
+      </c>
+      <c r="AK239" s="5" t="inlineStr">
+        <is>
+          <t>[D] reinforce-&gt;retire to McGilvery line</t>
+        </is>
+      </c>
+      <c r="AL239" s="5" t="inlineStr">
+        <is>
+          <t>McGilvery-line reinforcement</t>
+        </is>
+      </c>
+      <c r="AM239" s="5" t="inlineStr">
+        <is>
+          <t>3w/2m = 5</t>
+        </is>
+      </c>
       <c r="AN239" s="5" t="n"/>
-      <c r="AO239" s="5" t="n"/>
+      <c r="AO239" s="5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -29345,20 +29885,56 @@
           <t>reg-us-ar-2v-4</t>
         </is>
       </c>
-      <c r="AB242" s="5" t="n"/>
+      <c r="AB242" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC242" s="5" t="n"/>
       <c r="AD242" s="5" t="n"/>
       <c r="AE242" s="5" t="n"/>
       <c r="AF242" s="5" t="n"/>
-      <c r="AG242" s="5" t="n"/>
-      <c r="AH242" s="5" t="n"/>
-      <c r="AI242" s="5" t="n"/>
-      <c r="AJ242" s="5" t="n"/>
-      <c r="AK242" s="5" t="n"/>
-      <c r="AL242" s="5" t="n"/>
-      <c r="AM242" s="5" t="n"/>
+      <c r="AG242" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-taft.md; THE PASS'S LARGEST TRIAGE/RESEARCH MISMATCH - own commander's report was already the parent brigade dossier's primary source</t>
+        </is>
+      </c>
+      <c r="AH242" s="5" t="inlineStr">
+        <is>
+          <t>Capt. Elijah D. Taft (also 2VBde cmdr), 5th NY Battery; own report No.325</t>
+        </is>
+      </c>
+      <c r="AI242" s="5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AJ242" s="5" t="inlineStr">
+        <is>
+          <t>[C] Taneytown-&gt;10:30am arrival-&gt;4pm cemetery-&gt;5pm position, reporting direct to Howard (XI Corps)</t>
+        </is>
+      </c>
+      <c r="AK242" s="5" t="inlineStr">
+        <is>
+          <t>[B] staged approach; [D] return march Jul5</t>
+        </is>
+      </c>
+      <c r="AL242" s="5" t="inlineStr">
+        <is>
+          <t>counter-battery+infantry fire Jul2; sustained fire Jul3, 20pdr Parrott muzzle burst; itemized rds (80/63/32/382/557)</t>
+        </is>
+      </c>
+      <c r="AM242" s="5" t="inlineStr">
+        <is>
+          <t>4 individually-timed pins (Begg mw died Jul7, Thalheimer mw died midnight Jul3, Dillon slight, Wittenberg severe); brigade tablet total 8 in tension w/ 4 named</t>
+        </is>
+      </c>
       <c r="AN242" s="5" t="n"/>
-      <c r="AO242" s="5" t="n"/>
+      <c r="AO242" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
@@ -29469,20 +30045,56 @@
           <t>reg-us-ar-1r-3</t>
         </is>
       </c>
-      <c r="AB243" s="5" t="n"/>
+      <c r="AB243" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC243" s="5" t="n"/>
       <c r="AD243" s="5" t="n"/>
       <c r="AE243" s="5" t="n"/>
       <c r="AF243" s="5" t="n"/>
-      <c r="AG243" s="5" t="n"/>
-      <c r="AH243" s="5" t="n"/>
-      <c r="AI243" s="5" t="n"/>
-      <c r="AJ243" s="5" t="n"/>
-      <c r="AK243" s="5" t="n"/>
-      <c r="AL243" s="5" t="n"/>
-      <c r="AM243" s="5" t="n"/>
+      <c r="AG243" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-btty-evanthomas.md; TRIAGE CORRECTION, richest of the 3 1st-Regular corrections</t>
+        </is>
+      </c>
+      <c r="AH243" s="5" t="inlineStr">
+        <is>
+          <t>Lt. (bvt Maj) Evan Thomas, Battery C 4US; 6x12pdr; son of Adj-Gen Lorenzo Thomas; k 1873 vs Modoc</t>
+        </is>
+      </c>
+      <c r="AI243" s="5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AJ243" s="5" t="inlineStr">
+        <is>
+          <t>[D Jul2] Leister House crest near Meade's HQ; [D Jul3am] unchanged, engaged CSA arty across Seminary Ridge; slight shift pre-charge; post-bombardment-&gt;Arty Reserve</t>
+        </is>
+      </c>
+      <c r="AK243" s="5" t="inlineStr">
+        <is>
+          <t>[D] 3-leg chain Jul2-3</t>
+        </is>
+      </c>
+      <c r="AL243" s="5" t="inlineStr">
+        <is>
+          <t>'actively engaged' Jul2; Jul3 direct-hit caisson explosion, 3 more blew, drew CSA cheer; 14VT collateral casualties nearby</t>
+        </is>
+      </c>
+      <c r="AM243" s="5" t="inlineStr">
+        <is>
+          <t>1k/1off+16w = 18, +2 named later deaths (Campbell, McNeal)</t>
+        </is>
+      </c>
       <c r="AN243" s="5" t="n"/>
-      <c r="AO243" s="5" t="n"/>
+      <c r="AO243" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -37709,20 +38321,56 @@
           <t>reg-us-v-3-2</t>
         </is>
       </c>
-      <c r="AB302" s="5" t="n"/>
+      <c r="AB302" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC302" s="5" t="n"/>
       <c r="AD302" s="5" t="n"/>
       <c r="AE302" s="5" t="n"/>
       <c r="AF302" s="5" t="n"/>
-      <c r="AG302" s="5" t="n"/>
-      <c r="AH302" s="5" t="n"/>
-      <c r="AI302" s="5" t="n"/>
-      <c r="AJ302" s="5" t="n"/>
-      <c r="AK302" s="5" t="n"/>
-      <c r="AL302" s="5" t="n"/>
-      <c r="AM302" s="5" t="n"/>
+      <c r="AG302" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-v-3-2-fisher.md; independent-discovery claim flagged not adjudicated vs Rice/Chamberlain (403-blocked source)</t>
+        </is>
+      </c>
+      <c r="AH302" s="5" t="inlineStr">
+        <is>
+          <t>Col. Joseph W. Fisher, 5th/9th/10th/11th/12th PA Reserves; own report No.213-class</t>
+        </is>
+      </c>
+      <c r="AI302" s="5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AJ302" s="5" t="inlineStr">
+        <is>
+          <t>[C ~22:00] Big Round Top occupation; stone wall built overnight</t>
+        </is>
+      </c>
+      <c r="AK302" s="5" t="inlineStr">
+        <is>
+          <t>[D] march to the extreme left July 2; [A ~22:00] ascent of Big Round Top w/ 20th Maine</t>
+        </is>
+      </c>
+      <c r="AL302" s="5" t="inlineStr">
+        <is>
+          <t>over 30 prisoners; 1000+ stand of arms claimed, 80 CSA dead buried (own report, unverified vs CSA side)</t>
+        </is>
+      </c>
+      <c r="AM302" s="5" t="inlineStr">
+        <is>
+          <t>55 (1off+5men k/3off+46w) = McCandless 155 + Fisher 55 = Crawford 210 exact</t>
+        </is>
+      </c>
       <c r="AN302" s="5" t="n"/>
-      <c r="AO302" s="5" t="n"/>
+      <c r="AO302" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
@@ -41193,20 +41841,56 @@
           <t>reg-us-xi-2-2</t>
         </is>
       </c>
-      <c r="AB324" s="5" t="n"/>
+      <c r="AB324" s="5" t="inlineStr">
+        <is>
+          <t>authored-ok</t>
+        </is>
+      </c>
       <c r="AC324" s="5" t="n"/>
       <c r="AD324" s="5" t="n"/>
       <c r="AE324" s="5" t="n"/>
       <c r="AF324" s="5" t="n"/>
-      <c r="AG324" s="5" t="n"/>
-      <c r="AH324" s="5" t="n"/>
-      <c r="AI324" s="5" t="n"/>
-      <c r="AJ324" s="5" t="n"/>
-      <c r="AK324" s="5" t="n"/>
-      <c r="AL324" s="5" t="n"/>
-      <c r="AM324" s="5" t="n"/>
+      <c r="AG324" s="5" t="inlineStr">
+        <is>
+          <t>Dossier: reconstruction/dossiers/us-xi-2-2-smith.md; 33MA/Avery-repulse cross-ref flagged not verified</t>
+        </is>
+      </c>
+      <c r="AH324" s="5" t="inlineStr">
+        <is>
+          <t>Col. Orland Smith, 33MA/136NY/55OH/73OH; own report OR27/1 pp.722-725; identity verified NOT W.Smith CSA</t>
+        </is>
+      </c>
+      <c r="AI324" s="5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="AJ324" s="5" t="inlineStr">
+        <is>
+          <t>[C ~14:00 Jul1] Cemetery Hill wall, Emmitsburg/Taneytown Rds; von Steinwehr calls it 'First Bde' internally, Smith's own report says 'Second Bde' matching register</t>
+        </is>
+      </c>
+      <c r="AK324" s="5" t="inlineStr">
+        <is>
+          <t>[C] Jun12-Jul1 full march itinerary; 38mi/24.5hrs Boonsborough-Emmitsburg</t>
+        </is>
+      </c>
+      <c r="AL324" s="5" t="inlineStr">
+        <is>
+          <t>continuous skirmish Jul1-3; no direct assault Jul2 night; Jul3 assault redirected to II Corps</t>
+        </is>
+      </c>
+      <c r="AM324" s="5" t="inlineStr">
+        <is>
+          <t>REPORT-VS-TABLET CONFLICT: tablet 348 (51k/278w/19m) vs report 345 (66k/259w/26m) - every category disagrees, not adjudicated</t>
+        </is>
+      </c>
       <c r="AN324" s="5" t="n"/>
-      <c r="AO324" s="5" t="n"/>
+      <c r="AO324" s="5" t="inlineStr">
+        <is>
+          <t>T4 full-arc</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Wave A2: bundle metadata recompile + master-table regeneration
angle.bundle.json: payload byte-identical, only inputs.battle sha256 +
checksum re-derive (verified by full-file key diff vs main); ED-21
stagingSeed pin HELD (d470c469...e7ac1 verbatim). Master table build
metrics pick up the wave's decays (Poague 32, Taft 3, Hill 2, Torbert
11, Davis's documented 7200 keyframe) and Harrow's re-placed path.
reconstruction 122+1skip, pipeline 59, tool 110 — all green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -9518,29 +9518,29 @@
         <v>384</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>384</v>
+        <v>352</v>
       </c>
       <c r="H88" s="3">
         <f>IF(F88=0,0,1-G88/F88)</f>
         <v/>
       </c>
       <c r="I88" s="2" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="J88" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K88" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L88" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K88" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="L88" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M88" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O88" s="2" t="n">
         <v>0</v>
@@ -9579,7 +9579,7 @@
       </c>
       <c r="X88" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T0</t>
         </is>
       </c>
       <c r="Y88" s="2" t="inlineStr">
@@ -14831,10 +14831,10 @@
         <v>8</v>
       </c>
       <c r="K132" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L132" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M132" s="2" t="n">
         <v>0</v>
@@ -27619,26 +27619,26 @@
         </is>
       </c>
       <c r="F227" s="2" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G227" s="2" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H227" s="3">
         <f>IF(F227=0,0,1-G227/F227)</f>
         <v/>
       </c>
       <c r="I227" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J227" s="2" t="n">
         <v>2</v>
       </c>
       <c r="K227" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L227" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M227" s="2" t="n">
         <v>0</v>
@@ -27683,7 +27683,7 @@
       </c>
       <c r="X227" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T0</t>
         </is>
       </c>
       <c r="Y227" s="2" t="inlineStr">
@@ -28995,7 +28995,7 @@
         </is>
       </c>
       <c r="S236" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T236" s="2" t="n">
         <v>0</v>
@@ -29803,32 +29803,32 @@
         </is>
       </c>
       <c r="F242" s="2" t="n">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G242" s="2" t="n">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H242" s="3">
         <f>IF(F242=0,0,1-G242/F242)</f>
         <v/>
       </c>
       <c r="I242" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J242" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K242" s="2" t="n">
         <v>2</v>
       </c>
       <c r="L242" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M242" s="2" t="n">
         <v>0</v>
       </c>
       <c r="N242" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O242" s="2" t="n">
         <v>0</v>
@@ -39227,7 +39227,7 @@
         <v>5</v>
       </c>
       <c r="O308" s="2" t="n">
-        <v>121.7</v>
+        <v>217</v>
       </c>
       <c r="P308" s="2" t="n">
         <v>0</v>
@@ -42402,23 +42402,23 @@
         <v>1320</v>
       </c>
       <c r="G328" s="2" t="n">
-        <v>1320</v>
+        <v>1309</v>
       </c>
       <c r="H328" s="3">
         <f>IF(F328=0,0,1-G328/F328)</f>
         <v/>
       </c>
       <c r="I328" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J328" s="2" t="n">
         <v>2</v>
       </c>
       <c r="K328" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L328" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M328" s="2" t="n">
         <v>0</v>
@@ -42463,12 +42463,12 @@
       </c>
       <c r="X328" s="2" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T0</t>
         </is>
       </c>
       <c r="Y328" s="2" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="Z328" s="2" t="inlineStr">

</xml_diff>

<commit_message>
ED-75: regenerate master table with placeholder strengths
dossier-overlay.json's EC2 cells for csa-marshall/csa-davis now cite
ED-75; docs/reconstruction/audit/unit-master-table.{csv,xlsx}
regenerated (reconstruction && uv run --with openpyxl python
scripts/build_unit_audit.py) so the two brigades' + eight child
regiments' rows carry the ED-75 placeholder strengths (Marshall
900->268, Davis 1,293->387) instead of the flat 2,000 July-1 figure.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -10435,26 +10435,26 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>500</v>
+        <v>323</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>140</v>
+        <v>97</v>
       </c>
       <c r="H96" s="3">
         <f>IF(F96=0,0,1-G96/F96)</f>
         <v/>
       </c>
       <c r="I96" s="2" t="n">
-        <v>360</v>
+        <v>226</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>9</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M96" s="2" t="n">
         <v>0</v>
@@ -10555,17 +10555,17 @@
         </is>
       </c>
       <c r="F97" s="2" t="n">
-        <v>500</v>
+        <v>225</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>149</v>
+        <v>67</v>
       </c>
       <c r="H97" s="3">
         <f>IF(F97=0,0,1-G97/F97)</f>
         <v/>
       </c>
       <c r="I97" s="2" t="n">
-        <v>351</v>
+        <v>158</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>9</v>
@@ -11755,26 +11755,26 @@
         </is>
       </c>
       <c r="F107" s="2" t="n">
-        <v>500</v>
+        <v>225</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>149</v>
+        <v>67</v>
       </c>
       <c r="H107" s="3">
         <f>IF(F107=0,0,1-G107/F107)</f>
         <v/>
       </c>
       <c r="I107" s="2" t="n">
-        <v>351</v>
+        <v>158</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>9</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L107" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M107" s="2" t="n">
         <v>0</v>
@@ -11995,17 +11995,17 @@
         </is>
       </c>
       <c r="F109" s="2" t="n">
-        <v>500</v>
+        <v>323</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>151</v>
+        <v>97</v>
       </c>
       <c r="H109" s="3">
         <f>IF(F109=0,0,1-G109/F109)</f>
         <v/>
       </c>
       <c r="I109" s="2" t="n">
-        <v>349</v>
+        <v>226</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>8</v>
@@ -12355,17 +12355,17 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>500</v>
+        <v>323</v>
       </c>
       <c r="G112" s="2" t="n">
-        <v>151</v>
+        <v>97</v>
       </c>
       <c r="H112" s="3">
         <f>IF(F112=0,0,1-G112/F112)</f>
         <v/>
       </c>
       <c r="I112" s="2" t="n">
-        <v>349</v>
+        <v>226</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>8</v>
@@ -12475,17 +12475,17 @@
         </is>
       </c>
       <c r="F113" s="2" t="n">
-        <v>500</v>
+        <v>225</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>149</v>
+        <v>67</v>
       </c>
       <c r="H113" s="3">
         <f>IF(F113=0,0,1-G113/F113)</f>
         <v/>
       </c>
       <c r="I113" s="2" t="n">
-        <v>351</v>
+        <v>158</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>9</v>
@@ -12595,17 +12595,17 @@
         </is>
       </c>
       <c r="F114" s="2" t="n">
-        <v>500</v>
+        <v>225</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>149</v>
+        <v>67</v>
       </c>
       <c r="H114" s="3">
         <f>IF(F114=0,0,1-G114/F114)</f>
         <v/>
       </c>
       <c r="I114" s="2" t="n">
-        <v>351</v>
+        <v>158</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>9</v>
@@ -12835,17 +12835,17 @@
         </is>
       </c>
       <c r="F116" s="2" t="n">
-        <v>500</v>
+        <v>323</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>151</v>
+        <v>97</v>
       </c>
       <c r="H116" s="3">
         <f>IF(F116=0,0,1-G116/F116)</f>
         <v/>
       </c>
       <c r="I116" s="2" t="n">
-        <v>349</v>
+        <v>226</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>8</v>
@@ -14815,26 +14815,26 @@
         </is>
       </c>
       <c r="F132" s="2" t="n">
-        <v>2000</v>
+        <v>1293</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>603</v>
+        <v>387</v>
       </c>
       <c r="H132" s="3">
         <f>IF(F132=0,0,1-G132/F132)</f>
         <v/>
       </c>
       <c r="I132" s="2" t="n">
-        <v>1397</v>
+        <v>906</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>9</v>
       </c>
       <c r="K132" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L132" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M132" s="2" t="n">
         <v>0</v>
@@ -14918,7 +14918,7 @@
       </c>
       <c r="AI132" s="5" t="inlineStr">
         <is>
-          <t>2,000 'present first day' (stone-sentinels, scope caveat); 11th Miss DETACHED Jul 1 (division train guard, primary) - fresh regiment atop Jul 1 survivors on Jul 3</t>
+          <t>2,000 'present first day' (stone-sentinels, scope caveat); 11th Miss DETACHED Jul 1 (division train guard, primary) - fresh regiment atop Jul 1 survivors on Jul 3 -- ED-75 (2026-07-13): PROVISIONAL-ADOPTED placeholder (1,293 = ~900 three-regiment survivors + 393 11th Miss's own tablet-corroborated July-3 strength; envelope 1,100-1,550, INFERRED), superseded on arrival by Busey &amp; Martin page-level figures (owner purchase intent stated)</t>
         </is>
       </c>
       <c r="AJ132" s="5" t="inlineStr">
@@ -15471,26 +15471,26 @@
         </is>
       </c>
       <c r="F136" s="2" t="n">
-        <v>2000</v>
+        <v>900</v>
       </c>
       <c r="G136" s="2" t="n">
-        <v>595</v>
+        <v>268</v>
       </c>
       <c r="H136" s="3">
         <f>IF(F136=0,0,1-G136/F136)</f>
         <v/>
       </c>
       <c r="I136" s="2" t="n">
-        <v>1405</v>
+        <v>632</v>
       </c>
       <c r="J136" s="2" t="n">
         <v>10</v>
       </c>
       <c r="K136" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L136" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M136" s="2" t="n">
         <v>0</v>
@@ -15574,7 +15574,7 @@
       </c>
       <c r="AI136" s="5" t="inlineStr">
         <is>
-          <t>2,000 'present on the first day' (stone-sentinels, Jul-1 scope caveat); 26NC regt primary: 800+ -&gt; 216 unhurt (Jul 1) -&gt; ~80 (Jul 4) (young-26nc); Jul 3 basis ~900 [B subtraction, open for primary]</t>
+          <t>2,000 'present on the first day' (stone-sentinels, Jul-1 scope caveat); 26NC regt primary: 800+ -&gt; 216 unhurt (Jul 1) -&gt; ~80 (Jul 4) (young-26nc); Jul 3 basis ~900 [B subtraction] -- ED-75 (2026-07-13): PROVISIONAL-ADOPTED placeholder (900, envelope 750-1,050, INFERRED), superseded on arrival by Busey &amp; Martin page-level figures (owner purchase intent stated)</t>
         </is>
       </c>
       <c r="AJ136" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Angle-v2 data: Kemper/Armistead/Fry bombardment re-timing (P1 deferral)
Two pre-window keyframes each (t=420 signal guns, t=3600 even-split
midpoint), t=7200 citation upgrade with values unchanged, t>=7500
byte-identical (verified: 0 mismatches across 28 units x 661 s of
in-window compiled state). 15 children re-derived by the family share
formula. Authorized pinned-cast sha bump (owner: angle film v2
authorized) with the old pin recorded in the test comment.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reconstruction/audit/unit-master-table.xlsx
+++ b/docs/reconstruction/audit/unit-master-table.xlsx
@@ -10871,19 +10871,19 @@
         <v>146</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M98" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N98" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O98" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P98" s="2" t="n">
         <v>2477.9</v>
@@ -10996,19 +10996,19 @@
         <v>136</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M99" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N99" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O99" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P99" s="2" t="n">
         <v>2362.2</v>
@@ -11121,19 +11121,19 @@
         <v>135</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M100" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N100" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O100" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P100" s="2" t="n">
         <v>2431.2</v>
@@ -11246,19 +11246,19 @@
         <v>238</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L101" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M101" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N101" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O101" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P101" s="2" t="n">
         <v>2690.5</v>
@@ -11621,19 +11621,19 @@
         <v>136</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L104" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M104" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N104" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O104" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P104" s="2" t="n">
         <v>2321.5</v>
@@ -11746,19 +11746,19 @@
         <v>146</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="L105" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M105" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N105" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O105" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P105" s="2" t="n">
         <v>2695.9</v>
@@ -11871,19 +11871,19 @@
         <v>146</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="L106" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M106" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N106" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O106" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P106" s="2" t="n">
         <v>2568.8</v>
@@ -12371,19 +12371,19 @@
         <v>238</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L110" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M110" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N110" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O110" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P110" s="2" t="n">
         <v>2784.1</v>
@@ -12496,19 +12496,19 @@
         <v>146</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="L111" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M111" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N111" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O111" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P111" s="2" t="n">
         <v>2545.4</v>
@@ -12996,19 +12996,19 @@
         <v>238</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L115" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M115" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N115" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O115" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P115" s="2" t="n">
         <v>2643.7</v>
@@ -13371,19 +13371,19 @@
         <v>238</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L118" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M118" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N118" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O118" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P118" s="2" t="n">
         <v>2791.4</v>
@@ -13496,19 +13496,19 @@
         <v>136</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M119" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N119" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O119" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P119" s="2" t="n">
         <v>2447.6</v>
@@ -13621,19 +13621,19 @@
         <v>135</v>
       </c>
       <c r="K120" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L120" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M120" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N120" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O120" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P120" s="2" t="n">
         <v>2350.7</v>
@@ -13746,19 +13746,19 @@
         <v>146</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M121" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N121" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O121" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P121" s="2" t="n">
         <v>2458</v>
@@ -13996,19 +13996,19 @@
         <v>238</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L123" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M123" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N123" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O123" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P123" s="2" t="n">
         <v>2852.1</v>
@@ -14835,19 +14835,19 @@
         <v>1191</v>
       </c>
       <c r="K130" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L130" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M130" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N130" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O130" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="P130" s="2" t="n">
         <v>2593.7</v>
@@ -15330,19 +15330,19 @@
         <v>677</v>
       </c>
       <c r="K133" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="L133" s="2" t="n">
         <v>11</v>
       </c>
       <c r="M133" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N133" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O133" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="P133" s="2" t="n">
         <v>6538.5</v>
@@ -15676,19 +15676,19 @@
         <v>731</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="L135" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M135" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N135" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O135" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P135" s="2" t="n">
         <v>2458</v>

</xml_diff>